<commit_message>
Programme sizing rules editable in the workbook's Rules tab
Warm-up, hard-running caps and floors, run-length limits and the recovery week are now
rows on the Rules tab; the converter carries them into programmes.json and the planner
uses them (same values as before as defaults).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -155,7 +155,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="835" uniqueCount="388">
   <si>
     <t xml:space="preserve">Kinetix programmes</t>
   </si>
@@ -328,7 +328,13 @@
     <t xml:space="preserve">Fewer run days than the programme has sessions? The app drops easy and recovery runs first. More days? It adds easy runs.</t>
   </si>
   <si>
-    <t xml:space="preserve">Rep sessions keep their rep lengths; lower-volume runners get fewer reps so hard running stays a sensible share of their week.</t>
+    <t xml:space="preserve">Rep sessions keep their rep lengths; lower-volume runners get fewer reps so hard running stays a sensible share of their week (Rules: fast, threshold and steady reps max).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rep and tempo sessions get an easy warm-up and cool-down (Rules: warm-up). Other runs share what's left: easy 1, recovery 0.75, shakeout 0.6, progression 1.15, within the Rules' run-length limits.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A race date lines the programme up so its last week is race week (early weeks skipped if it's sooner, base weeks repeated first if it's further away). The race is its full distance and isn't counted in the week's %.</t>
   </si>
   <si>
     <t xml:space="preserve">The worked example columns (grey) show what each week would be for a runner at the volume in Rules → 'Example runner'.</t>
@@ -1037,6 +1043,63 @@
   </si>
   <si>
     <t xml:space="preserve">Only for the grey example columns in Run weeks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warm-up and cool-down, each (fraction of week)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added to rep and tempo sessions. Kept between the min and max below.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warm-up minimum (km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also used when the long run and sessions already fill the week.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warm-up maximum (km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fast reps max (fraction of week): I, R, 5K, hills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard running per session. Lower-volume runners get fewer reps; rep lengths never change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fast reps floor (km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Always allowed at least this much, whatever the week's volume.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threshold reps max (fraction of week): T, 10K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Threshold reps floor (km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady reps max (fraction of week): STEADY, M, HM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Steady reps floor (km)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recovery run max (fraction of long run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spare volume beyond these lengths adds an easy run if there's a free day.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Easy run max (fraction of long run)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shakeout max (fraction of week)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recovery week after the programme (fraction of starting)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Easy running only, then the programme repeats from their recent running.</t>
   </si>
   <si>
     <t xml:space="preserve">Current app defaults are filled in; change any yellow value.</t>
@@ -1767,7 +1830,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -2111,6 +2174,24 @@
       </c>
       <c r="C42" s="10" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1"/>
+      <c r="B43" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C43" s="10" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1"/>
+      <c r="B44" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -2145,189 +2226,189 @@
         <v>8</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>295</v>
+        <v>316</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>27</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>297</v>
+        <v>318</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>298</v>
+        <v>319</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>299</v>
+        <v>320</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>76</v>
-      </c>
       <c r="F3" s="6" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>301</v>
+        <v>322</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2335,24 +2416,24 @@
         <v>35</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2360,367 +2441,367 @@
         <v>45</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I12" s="6" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I13" s="6" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I14" s="6" t="s">
-        <v>302</v>
+        <v>323</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I15" s="6" t="s">
-        <v>303</v>
+        <v>324</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I16" s="6" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I17" s="6" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I18" s="6" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I19" s="6" t="s">
-        <v>306</v>
+        <v>327</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I20" s="6" t="s">
-        <v>307</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I21" s="6" t="s">
-        <v>308</v>
+        <v>329</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I22" s="6" t="s">
-        <v>309</v>
+        <v>330</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I23" s="6" t="s">
-        <v>310</v>
+        <v>331</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I24" s="6" t="s">
-        <v>311</v>
+        <v>332</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I25" s="6" t="s">
-        <v>312</v>
+        <v>333</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I26" s="6" t="s">
-        <v>313</v>
+        <v>334</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I27" s="6" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I28" s="6" t="s">
-        <v>315</v>
+        <v>336</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I29" s="6" t="s">
-        <v>316</v>
+        <v>337</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I30" s="6" t="s">
-        <v>317</v>
+        <v>338</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I31" s="6" t="s">
-        <v>318</v>
+        <v>339</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I32" s="6" t="s">
-        <v>319</v>
+        <v>340</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I33" s="6" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I34" s="6" t="s">
-        <v>320</v>
+        <v>341</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I35" s="6" t="s">
-        <v>321</v>
+        <v>342</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I36" s="6" t="s">
-        <v>322</v>
+        <v>343</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I37" s="6" t="s">
-        <v>323</v>
+        <v>344</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I38" s="6" t="s">
-        <v>324</v>
+        <v>345</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I39" s="6" t="s">
-        <v>325</v>
+        <v>346</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I40" s="6" t="s">
-        <v>326</v>
+        <v>347</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I41" s="6" t="s">
-        <v>327</v>
+        <v>348</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I42" s="6" t="s">
-        <v>328</v>
+        <v>349</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I43" s="6" t="s">
-        <v>329</v>
+        <v>350</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I44" s="6" t="s">
-        <v>330</v>
+        <v>351</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I45" s="6" t="s">
-        <v>331</v>
+        <v>352</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I46" s="6" t="s">
-        <v>332</v>
+        <v>353</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I47" s="6" t="s">
-        <v>333</v>
+        <v>354</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I48" s="6" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I49" s="6" t="s">
-        <v>334</v>
+        <v>355</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I50" s="6" t="s">
-        <v>335</v>
+        <v>356</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I51" s="6" t="s">
-        <v>336</v>
+        <v>357</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I52" s="6" t="s">
-        <v>337</v>
+        <v>358</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I53" s="6" t="s">
-        <v>338</v>
+        <v>359</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I54" s="6" t="s">
-        <v>339</v>
+        <v>360</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I55" s="6" t="s">
-        <v>340</v>
+        <v>361</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I56" s="6" t="s">
-        <v>341</v>
+        <v>362</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I57" s="6" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I58" s="6" t="s">
-        <v>342</v>
+        <v>363</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I59" s="6" t="s">
-        <v>343</v>
+        <v>364</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I60" s="6" t="s">
-        <v>344</v>
+        <v>365</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I61" s="6" t="s">
-        <v>345</v>
+        <v>366</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I62" s="6" t="s">
-        <v>346</v>
+        <v>367</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I63" s="6" t="s">
-        <v>347</v>
+        <v>368</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I64" s="6" t="s">
-        <v>348</v>
+        <v>369</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I65" s="6" t="s">
-        <v>349</v>
+        <v>370</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I66" s="6" t="s">
-        <v>350</v>
+        <v>371</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I67" s="6" t="s">
-        <v>351</v>
+        <v>372</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I68" s="6" t="s">
-        <v>352</v>
+        <v>373</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I69" s="6" t="s">
-        <v>353</v>
+        <v>374</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I70" s="6" t="s">
-        <v>354</v>
+        <v>375</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I71" s="6" t="s">
-        <v>355</v>
+        <v>376</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I72" s="6" t="s">
-        <v>356</v>
+        <v>377</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I73" s="6" t="s">
-        <v>357</v>
+        <v>378</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I74" s="6" t="s">
-        <v>358</v>
+        <v>379</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I75" s="6" t="s">
-        <v>359</v>
+        <v>380</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I76" s="6" t="s">
-        <v>360</v>
+        <v>381</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I77" s="6" t="s">
-        <v>361</v>
+        <v>382</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I78" s="6" t="s">
-        <v>362</v>
+        <v>383</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I79" s="6" t="s">
-        <v>363</v>
+        <v>384</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I80" s="6" t="s">
-        <v>364</v>
+        <v>385</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I81" s="6" t="s">
-        <v>365</v>
+        <v>386</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I82" s="6" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="I83" s="6" t="s">
-        <v>366</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
@@ -2755,63 +2836,63 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="N1" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="O1" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C2" s="12" t="n">
         <v>8</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E2" s="12" t="n">
         <v>3</v>
@@ -2835,10 +2916,10 @@
         <v>1</v>
       </c>
       <c r="L2" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="N2" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A2)</f>
@@ -2851,16 +2932,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C3" s="12" t="n">
         <v>10</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E3" s="12" t="n">
         <v>3</v>
@@ -2884,10 +2965,10 @@
         <v>1</v>
       </c>
       <c r="L3" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M3" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="N3" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A3)</f>
@@ -2900,16 +2981,16 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>12</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E4" s="12" t="n">
         <v>3</v>
@@ -2933,10 +3014,10 @@
         <v>2</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="N4" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A4)</f>
@@ -2949,16 +3030,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>16</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E5" s="12" t="n">
         <v>4</v>
@@ -2982,10 +3063,10 @@
         <v>3</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="N5" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A5)</f>
@@ -2998,16 +3079,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>8</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E6" s="12" t="n">
         <v>1</v>
@@ -3031,10 +3112,10 @@
         <v>1</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="M6" s="12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N6" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A6)</f>
@@ -3047,16 +3128,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>8</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E7" s="12" t="n">
         <v>1</v>
@@ -3080,10 +3161,10 @@
         <v>1</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N7" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A7)</f>
@@ -3096,16 +3177,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>8</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E8" s="12" t="n">
         <v>2</v>
@@ -3129,10 +3210,10 @@
         <v>1</v>
       </c>
       <c r="L8" s="12" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="N8" s="13" t="n">
         <f aca="false">COUNTIF('Run weeks'!$A$2:$A$401,A8)</f>
@@ -3145,7 +3226,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3187,57 +3268,57 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B2" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D2" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G2" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H2" s="13" t="n">
         <f aca="false">IF(A2="","",COUNTIFS('Run sessions'!$A$2:$A$401,A2,'Run sessions'!$B$2:$B$401,B2))</f>
@@ -3254,22 +3335,22 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D3" s="15" t="n">
         <v>1.05</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G3" s="12"/>
       <c r="H3" s="13" t="n">
@@ -3287,22 +3368,22 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D4" s="15" t="n">
         <v>1.1</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G4" s="12"/>
       <c r="H4" s="13" t="n">
@@ -3320,25 +3401,25 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D5" s="15" t="n">
         <v>0.9</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H5" s="13" t="n">
         <f aca="false">IF(A5="","",COUNTIFS('Run sessions'!$A$2:$A$401,A5,'Run sessions'!$B$2:$B$401,B5))</f>
@@ -3355,22 +3436,22 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D6" s="15" t="n">
         <v>1.15</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G6" s="12"/>
       <c r="H6" s="13" t="n">
@@ -3388,22 +3469,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D7" s="15" t="n">
         <v>1.2</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="13" t="n">
@@ -3421,22 +3502,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>7</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D8" s="15" t="n">
         <v>1.25</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G8" s="12"/>
       <c r="H8" s="13" t="n">
@@ -3454,22 +3535,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>8</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D9" s="15" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G9" s="12"/>
       <c r="H9" s="13" t="n">
@@ -3487,25 +3568,25 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>9</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D10" s="15" t="n">
         <v>1.3</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G10" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="H10" s="13" t="n">
         <f aca="false">IF(A10="","",COUNTIFS('Run sessions'!$A$2:$A$401,A10,'Run sessions'!$B$2:$B$401,B10))</f>
@@ -3522,22 +3603,22 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>10</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D11" s="15" t="n">
         <v>1.3</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G11" s="12"/>
       <c r="H11" s="13" t="n">
@@ -3555,25 +3636,25 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>11</v>
       </c>
       <c r="C12" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="D12" s="15" t="n">
         <v>0.85</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G12" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H12" s="13" t="n">
         <f aca="false">IF(A12="","",COUNTIFS('Run sessions'!$A$2:$A$401,A12,'Run sessions'!$B$2:$B$401,B12))</f>
@@ -3590,13 +3671,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D13" s="15" t="n">
         <v>0.55</v>
@@ -3605,10 +3686,10 @@
         <v>45</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="G13" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H13" s="13" t="n">
         <f aca="false">IF(A13="","",COUNTIFS('Run sessions'!$A$2:$A$401,A13,'Run sessions'!$B$2:$B$401,B13))</f>
@@ -11816,30 +11897,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B2" s="12" t="n">
         <v>1</v>
@@ -11848,19 +11929,19 @@
         <v>1</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>1</v>
@@ -11869,19 +11950,19 @@
         <v>2</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F3" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G3" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>1</v>
@@ -11890,19 +11971,19 @@
         <v>3</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>1</v>
@@ -11911,19 +11992,19 @@
         <v>4</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>2</v>
@@ -11935,16 +12016,16 @@
         <v>35</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="G6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>2</v>
@@ -11953,19 +12034,19 @@
         <v>2</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>2</v>
@@ -11974,19 +12055,19 @@
         <v>3</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>2</v>
@@ -11995,19 +12076,19 @@
         <v>4</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>3</v>
@@ -12016,19 +12097,19 @@
         <v>1</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G10" s="12"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B11" s="12" t="n">
         <v>3</v>
@@ -12037,19 +12118,19 @@
         <v>2</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G11" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B12" s="12" t="n">
         <v>3</v>
@@ -12058,19 +12139,19 @@
         <v>3</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G12" s="12"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="12" t="n">
         <v>3</v>
@@ -12079,19 +12160,19 @@
         <v>4</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B14" s="12" t="n">
         <v>4</v>
@@ -12100,19 +12181,19 @@
         <v>1</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="G14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" s="12" t="n">
         <v>4</v>
@@ -12121,19 +12202,19 @@
         <v>2</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F15" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G15" s="12"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B16" s="12" t="n">
         <v>4</v>
@@ -12142,19 +12223,19 @@
         <v>3</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="G16" s="12"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>4</v>
@@ -12163,19 +12244,19 @@
         <v>4</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G17" s="12"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B18" s="12" t="n">
         <v>5</v>
@@ -12187,16 +12268,16 @@
         <v>35</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G18" s="12"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B19" s="12" t="n">
         <v>5</v>
@@ -12205,19 +12286,19 @@
         <v>2</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F19" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B20" s="12" t="n">
         <v>5</v>
@@ -12226,19 +12307,19 @@
         <v>3</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B21" s="12" t="n">
         <v>5</v>
@@ -12247,19 +12328,19 @@
         <v>4</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B22" s="12" t="n">
         <v>6</v>
@@ -12268,19 +12349,19 @@
         <v>1</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F22" s="12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G22" s="12"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B23" s="12" t="n">
         <v>6</v>
@@ -12289,19 +12370,19 @@
         <v>2</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G23" s="12"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B24" s="12" t="n">
         <v>6</v>
@@ -12310,19 +12391,19 @@
         <v>3</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B25" s="12" t="n">
         <v>6</v>
@@ -12331,19 +12412,19 @@
         <v>4</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B26" s="12" t="n">
         <v>7</v>
@@ -12352,19 +12433,19 @@
         <v>1</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B27" s="12" t="n">
         <v>7</v>
@@ -12373,19 +12454,19 @@
         <v>2</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B28" s="12" t="n">
         <v>7</v>
@@ -12394,19 +12475,19 @@
         <v>3</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B29" s="12" t="n">
         <v>7</v>
@@ -12415,19 +12496,19 @@
         <v>4</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F29" s="12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="12" t="n">
         <v>8</v>
@@ -12439,16 +12520,16 @@
         <v>35</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F30" s="12" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B31" s="12" t="n">
         <v>8</v>
@@ -12457,19 +12538,19 @@
         <v>2</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F31" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B32" s="12" t="n">
         <v>8</v>
@@ -12478,19 +12559,19 @@
         <v>3</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G32" s="12"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B33" s="12" t="n">
         <v>8</v>
@@ -12499,19 +12580,19 @@
         <v>4</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F33" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G33" s="12"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B34" s="12" t="n">
         <v>9</v>
@@ -12520,19 +12601,19 @@
         <v>1</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G34" s="12"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B35" s="12" t="n">
         <v>9</v>
@@ -12541,19 +12622,19 @@
         <v>2</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F35" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G35" s="12"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B36" s="12" t="n">
         <v>9</v>
@@ -12562,19 +12643,19 @@
         <v>3</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F36" s="12" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G36" s="12"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B37" s="12" t="n">
         <v>9</v>
@@ -12583,19 +12664,19 @@
         <v>4</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F37" s="12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G37" s="12"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B38" s="12" t="n">
         <v>10</v>
@@ -12604,19 +12685,19 @@
         <v>1</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E38" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F38" s="12" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G38" s="12"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B39" s="12" t="n">
         <v>10</v>
@@ -12625,19 +12706,19 @@
         <v>2</v>
       </c>
       <c r="D39" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="E39" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F39" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G39" s="12"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B40" s="12" t="n">
         <v>10</v>
@@ -12646,19 +12727,19 @@
         <v>3</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E40" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B41" s="12" t="n">
         <v>10</v>
@@ -12667,19 +12748,19 @@
         <v>4</v>
       </c>
       <c r="D41" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E41" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F41" s="12" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G41" s="12"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B42" s="12" t="n">
         <v>11</v>
@@ -12688,19 +12769,19 @@
         <v>1</v>
       </c>
       <c r="D42" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E42" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F42" s="12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G42" s="12"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B43" s="12" t="n">
         <v>11</v>
@@ -12709,19 +12790,19 @@
         <v>2</v>
       </c>
       <c r="D43" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E43" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F43" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G43" s="12"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B44" s="12" t="n">
         <v>11</v>
@@ -12730,19 +12811,19 @@
         <v>3</v>
       </c>
       <c r="D44" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E44" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F44" s="12" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G44" s="12"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B45" s="12" t="n">
         <v>11</v>
@@ -12751,19 +12832,19 @@
         <v>4</v>
       </c>
       <c r="D45" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="E45" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F45" s="12" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B46" s="12" t="n">
         <v>12</v>
@@ -12772,19 +12853,19 @@
         <v>1</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="E46" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F46" s="12" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G46" s="12"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B47" s="12" t="n">
         <v>12</v>
@@ -12793,19 +12874,19 @@
         <v>2</v>
       </c>
       <c r="D47" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E47" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F47" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G47" s="12"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B48" s="12" t="n">
         <v>12</v>
@@ -12814,10 +12895,10 @@
         <v>3</v>
       </c>
       <c r="D48" s="12" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E48" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F48" s="12" t="s">
         <v>42</v>
@@ -12826,7 +12907,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B49" s="12" t="n">
         <v>12</v>
@@ -12838,10 +12919,10 @@
         <v>45</v>
       </c>
       <c r="E49" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F49" s="12" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="G49" s="12"/>
     </row>
@@ -16053,189 +16134,189 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D2" s="16" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F2" s="12"/>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F3" s="12"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F4" s="12"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B5" s="16" t="s">
+        <v>186</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="D5" s="16" t="s">
+        <v>188</v>
+      </c>
+      <c r="E5" s="12" t="s">
         <v>184</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>186</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>182</v>
       </c>
       <c r="F5" s="12"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F7" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F8" s="12"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B9" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="D9" s="16" t="s">
+        <v>205</v>
+      </c>
+      <c r="E9" s="12" t="s">
         <v>201</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>203</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>199</v>
       </c>
       <c r="F9" s="12"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F10" s="12"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -16267,39 +16348,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B2" s="12" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F2" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A2)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16308,19 +16389,19 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D3" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>221</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>219</v>
       </c>
       <c r="F3" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A3)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16329,19 +16410,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B4" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F4" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A4)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16350,19 +16431,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F5" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A5)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16371,19 +16452,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B6" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F6" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A6)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16392,19 +16473,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>6</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F7" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A7)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16413,19 +16494,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B8" s="12" t="n">
         <v>3</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F8" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A8)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16434,19 +16515,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>5</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F9" s="13" t="n">
         <f aca="false">SUMPRODUCT(('Split days'!$A$2:$A$401=A9)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
@@ -16490,51 +16571,51 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C2" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
@@ -16544,19 +16625,19 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C3" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E3" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
@@ -16566,19 +16647,19 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
@@ -16588,19 +16669,19 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
@@ -16610,19 +16691,19 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D6" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="E6" s="12" t="s">
         <v>252</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>250</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
@@ -16632,19 +16713,19 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
@@ -16654,19 +16735,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
@@ -16676,19 +16757,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C9" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
@@ -16698,19 +16779,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C10" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
@@ -16720,19 +16801,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C11" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
@@ -16742,19 +16823,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C12" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
@@ -16764,19 +16845,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="E13" s="12" t="s">
         <v>249</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>247</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="12"/>
@@ -16786,19 +16867,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C14" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
@@ -16808,19 +16889,19 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C15" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="12"/>
@@ -16830,19 +16911,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C16" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
@@ -16852,19 +16933,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C17" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E17" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F17" s="12"/>
       <c r="G17" s="12"/>
@@ -16874,19 +16955,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C18" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="E18" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
@@ -16896,19 +16977,19 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C19" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E19" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F19" s="12"/>
       <c r="G19" s="12"/>
@@ -16918,19 +16999,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C20" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E20" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
@@ -16940,19 +17021,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C21" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D21" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="E21" s="12" t="s">
         <v>252</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>250</v>
       </c>
       <c r="F21" s="12"/>
       <c r="G21" s="12"/>
@@ -16962,19 +17043,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B22" s="12" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C22" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E22" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
@@ -16984,19 +17065,19 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C23" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="E23" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="12"/>
@@ -17006,19 +17087,19 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C24" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
@@ -17028,19 +17109,19 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C25" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F25" s="12"/>
       <c r="G25" s="12"/>
@@ -17050,19 +17131,19 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C26" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D26" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="E26" s="12" t="s">
         <v>252</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>250</v>
       </c>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
@@ -17072,19 +17153,19 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C27" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="12" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F27" s="12"/>
       <c r="G27" s="12"/>
@@ -17094,19 +17175,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C28" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D28" s="12" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F28" s="12"/>
       <c r="G28" s="12"/>
@@ -17116,19 +17197,19 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C29" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D29" s="12" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F29" s="12"/>
       <c r="G29" s="12"/>
@@ -17138,19 +17219,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C30" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D30" s="12" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F30" s="12"/>
       <c r="G30" s="12"/>
@@ -17160,19 +17241,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C31" s="12" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="12" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E31" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F31" s="12" t="n">
         <v>4</v>
@@ -17190,19 +17271,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C32" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F32" s="12"/>
       <c r="G32" s="12"/>
@@ -17212,19 +17293,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C33" s="12" t="n">
         <v>3</v>
       </c>
       <c r="D33" s="12" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F33" s="12"/>
       <c r="G33" s="12"/>
@@ -17234,19 +17315,19 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C34" s="12" t="n">
         <v>4</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E34" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F34" s="12"/>
       <c r="G34" s="12"/>
@@ -17256,19 +17337,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C35" s="12" t="n">
         <v>5</v>
       </c>
       <c r="D35" s="12" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F35" s="12"/>
       <c r="G35" s="12"/>
@@ -17290,7 +17371,7 @@
     </row>
     <row r="37" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="17" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="12"/>
@@ -21713,33 +21794,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C2" s="12" t="n">
         <v>3</v>
@@ -21757,10 +21838,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C3" s="12" t="n">
         <v>2</v>
@@ -21778,10 +21859,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C4" s="12" t="n">
         <v>3</v>
@@ -21799,10 +21880,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C5" s="12" t="n">
         <v>2</v>
@@ -21820,10 +21901,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C6" s="12" t="n">
         <v>3</v>
@@ -21841,10 +21922,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>2</v>
@@ -21862,10 +21943,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>3</v>
@@ -21883,10 +21964,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C9" s="12" t="n">
         <v>2</v>
@@ -21904,10 +21985,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C10" s="12" t="n">
         <v>5</v>
@@ -21925,10 +22006,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C11" s="12" t="n">
         <v>3</v>
@@ -21946,10 +22027,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C12" s="12" t="n">
         <v>4</v>
@@ -21967,10 +22048,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C13" s="12" t="n">
         <v>3</v>
@@ -21988,10 +22069,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C14" s="12" t="n">
         <v>4</v>
@@ -22009,10 +22090,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C15" s="12" t="n">
         <v>3</v>
@@ -22030,12 +22111,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>
@@ -22054,7 +22135,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -22064,24 +22145,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="E1" s="11" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B2" s="18" t="n">
         <v>8</v>
@@ -22093,12 +22174,12 @@
         <v>25</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B3" s="18" t="n">
         <v>8</v>
@@ -22110,12 +22191,12 @@
         <v>25</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B4" s="18" t="n">
         <v>30</v>
@@ -22127,12 +22208,12 @@
         <v>100</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B5" s="18" t="n">
         <v>10</v>
@@ -22144,12 +22225,12 @@
         <v>32</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B6" s="18" t="n">
         <v>3</v>
@@ -22161,12 +22242,12 @@
         <v>4</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B7" s="19" t="n">
         <v>0.1</v>
@@ -22178,12 +22259,12 @@
         <v>0.12</v>
       </c>
       <c r="E7" s="14" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B8" s="19" t="n">
         <v>0.3</v>
@@ -22195,12 +22276,12 @@
         <v>0.32</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B9" s="18" t="n">
         <v>15</v>
@@ -22212,12 +22293,219 @@
         <v>50</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>293</v>
+        <v>295</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="14" t="s">
-        <v>294</v>
+      <c r="A11" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>300</v>
+      </c>
+      <c r="B12" s="18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E12" s="14"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B14" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="B15" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C15" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D15" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E15" s="14"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="B16" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="14"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="B17" s="19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E17" s="14"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>308</v>
+      </c>
+      <c r="B18" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" s="14"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B19" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D19" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>311</v>
+      </c>
+      <c r="B20" s="19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D20" s="19" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>312</v>
+      </c>
+      <c r="B21" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E21" s="14"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="B22" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C22" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D22" s="19" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Marathon programme draft (16 weeks) and race programmes use their own long-run cap
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -2632,7 +2632,7 @@
         <v>85</v>
       </c>
       <c r="N6" s="32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O6" s="32" t="inlineStr">
         <is>
@@ -4617,13 +4617,37 @@
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="21">
-      <c r="A38" s="32" t="n"/>
-      <c r="B38" s="32" t="n"/>
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="35" t="n"/>
-      <c r="E38" s="32" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="32" t="n"/>
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B38" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D38" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F38" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G38" s="32" t="inlineStr">
+        <is>
+          <t>Settle in: one threshold session and an M-pace progression, everything else easy.</t>
+        </is>
+      </c>
       <c r="H38" s="33">
         <f>IF(A38="","",COUNTIFS('Run sessions'!$A$2:$A$401,A38,'Run sessions'!$B$2:$B$401,B38))</f>
         <v/>
@@ -4638,12 +4662,32 @@
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="21">
-      <c r="A39" s="32" t="n"/>
-      <c r="B39" s="32" t="n"/>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="35" t="n"/>
-      <c r="E39" s="32" t="n"/>
-      <c r="F39" s="32" t="n"/>
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D39" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E39" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F39" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G39" s="32" t="n"/>
       <c r="H39" s="33">
         <f>IF(A39="","",COUNTIFS('Run sessions'!$A$2:$A$401,A39,'Run sessions'!$B$2:$B$401,B39))</f>
@@ -4659,12 +4703,32 @@
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="21">
-      <c r="A40" s="32" t="n"/>
-      <c r="B40" s="32" t="n"/>
-      <c r="C40" s="32" t="n"/>
-      <c r="D40" s="35" t="n"/>
-      <c r="E40" s="32" t="n"/>
-      <c r="F40" s="32" t="n"/>
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B40" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D40" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E40" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F40" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G40" s="32" t="n"/>
       <c r="H40" s="33">
         <f>IF(A40="","",COUNTIFS('Run sessions'!$A$2:$A$401,A40,'Run sessions'!$B$2:$B$401,B40))</f>
@@ -4680,13 +4744,37 @@
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="21">
-      <c r="A41" s="32" t="n"/>
-      <c r="B41" s="32" t="n"/>
-      <c r="C41" s="32" t="n"/>
-      <c r="D41" s="35" t="n"/>
-      <c r="E41" s="32" t="n"/>
-      <c r="F41" s="32" t="n"/>
-      <c r="G41" s="32" t="n"/>
+      <c r="A41" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B41" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D41" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E41" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F41" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G41" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week: let the work sink in.</t>
+        </is>
+      </c>
       <c r="H41" s="33">
         <f>IF(A41="","",COUNTIFS('Run sessions'!$A$2:$A$401,A41,'Run sessions'!$B$2:$B$401,B41))</f>
         <v/>
@@ -4701,13 +4789,37 @@
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="21">
-      <c r="A42" s="32" t="n"/>
-      <c r="B42" s="32" t="n"/>
-      <c r="C42" s="32" t="n"/>
-      <c r="D42" s="35" t="n"/>
-      <c r="E42" s="32" t="n"/>
-      <c r="F42" s="32" t="n"/>
-      <c r="G42" s="32" t="n"/>
+      <c r="A42" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B42" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D42" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E42" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F42" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G42" s="32" t="inlineStr">
+        <is>
+          <t>Marathon pace starts to appear in your long run.</t>
+        </is>
+      </c>
       <c r="H42" s="33">
         <f>IF(A42="","",COUNTIFS('Run sessions'!$A$2:$A$401,A42,'Run sessions'!$B$2:$B$401,B42))</f>
         <v/>
@@ -4722,12 +4834,32 @@
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="21">
-      <c r="A43" s="32" t="n"/>
-      <c r="B43" s="32" t="n"/>
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="35" t="n"/>
-      <c r="E43" s="32" t="n"/>
-      <c r="F43" s="32" t="n"/>
+      <c r="A43" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B43" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C43" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D43" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E43" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F43" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G43" s="32" t="n"/>
       <c r="H43" s="33">
         <f>IF(A43="","",COUNTIFS('Run sessions'!$A$2:$A$401,A43,'Run sessions'!$B$2:$B$401,B43))</f>
@@ -4743,12 +4875,32 @@
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="21">
-      <c r="A44" s="32" t="n"/>
-      <c r="B44" s="32" t="n"/>
-      <c r="C44" s="32" t="n"/>
-      <c r="D44" s="35" t="n"/>
-      <c r="E44" s="32" t="n"/>
-      <c r="F44" s="32" t="n"/>
+      <c r="A44" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B44" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C44" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D44" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E44" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F44" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G44" s="32" t="n"/>
       <c r="H44" s="33">
         <f>IF(A44="","",COUNTIFS('Run sessions'!$A$2:$A$401,A44,'Run sessions'!$B$2:$B$401,B44))</f>
@@ -4764,13 +4916,37 @@
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="21">
-      <c r="A45" s="32" t="n"/>
-      <c r="B45" s="32" t="n"/>
-      <c r="C45" s="32" t="n"/>
-      <c r="D45" s="35" t="n"/>
-      <c r="E45" s="32" t="n"/>
-      <c r="F45" s="32" t="n"/>
-      <c r="G45" s="32" t="n"/>
+      <c r="A45" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B45" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C45" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D45" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E45" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F45" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G45" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week before the big block.</t>
+        </is>
+      </c>
       <c r="H45" s="33">
         <f>IF(A45="","",COUNTIFS('Run sessions'!$A$2:$A$401,A45,'Run sessions'!$B$2:$B$401,B45))</f>
         <v/>
@@ -4785,13 +4961,37 @@
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="21">
-      <c r="A46" s="32" t="n"/>
-      <c r="B46" s="32" t="n"/>
-      <c r="C46" s="32" t="n"/>
-      <c r="D46" s="35" t="n"/>
-      <c r="E46" s="32" t="n"/>
-      <c r="F46" s="32" t="n"/>
-      <c r="G46" s="32" t="n"/>
+      <c r="A46" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B46" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C46" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D46" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E46" s="32" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F46" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G46" s="32" t="inlineStr">
+        <is>
+          <t>First really long run: keep it easy.</t>
+        </is>
+      </c>
       <c r="H46" s="33">
         <f>IF(A46="","",COUNTIFS('Run sessions'!$A$2:$A$401,A46,'Run sessions'!$B$2:$B$401,B46))</f>
         <v/>
@@ -4806,12 +5006,32 @@
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="21">
-      <c r="A47" s="32" t="n"/>
-      <c r="B47" s="32" t="n"/>
-      <c r="C47" s="32" t="n"/>
-      <c r="D47" s="35" t="n"/>
-      <c r="E47" s="32" t="n"/>
-      <c r="F47" s="32" t="n"/>
+      <c r="A47" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B47" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C47" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D47" s="35" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E47" s="32" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F47" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G47" s="32" t="n"/>
       <c r="H47" s="33">
         <f>IF(A47="","",COUNTIFS('Run sessions'!$A$2:$A$401,A47,'Run sessions'!$B$2:$B$401,B47))</f>
@@ -4827,13 +5047,37 @@
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="21">
-      <c r="A48" s="32" t="n"/>
-      <c r="B48" s="32" t="n"/>
-      <c r="C48" s="32" t="n"/>
-      <c r="D48" s="35" t="n"/>
-      <c r="E48" s="32" t="n"/>
-      <c r="F48" s="32" t="n"/>
-      <c r="G48" s="32" t="n"/>
+      <c r="A48" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B48" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C48" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D48" s="35" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E48" s="32" t="inlineStr">
+        <is>
+          <t>34%</t>
+        </is>
+      </c>
+      <c r="F48" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G48" s="32" t="inlineStr">
+        <is>
+          <t>Peak block: long runs near their longest.</t>
+        </is>
+      </c>
       <c r="H48" s="33">
         <f>IF(A48="","",COUNTIFS('Run sessions'!$A$2:$A$401,A48,'Run sessions'!$B$2:$B$401,B48))</f>
         <v/>
@@ -4848,13 +5092,37 @@
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="21">
-      <c r="A49" s="32" t="n"/>
-      <c r="B49" s="32" t="n"/>
-      <c r="C49" s="32" t="n"/>
-      <c r="D49" s="35" t="n"/>
-      <c r="E49" s="32" t="n"/>
-      <c r="F49" s="32" t="n"/>
-      <c r="G49" s="32" t="n"/>
+      <c r="A49" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C49" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D49" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F49" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G49" s="32" t="inlineStr">
+        <is>
+          <t>Recover before your longest run.</t>
+        </is>
+      </c>
       <c r="H49" s="33">
         <f>IF(A49="","",COUNTIFS('Run sessions'!$A$2:$A$401,A49,'Run sessions'!$B$2:$B$401,B49))</f>
         <v/>
@@ -4869,13 +5137,37 @@
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="21">
-      <c r="A50" s="32" t="n"/>
-      <c r="B50" s="32" t="n"/>
-      <c r="C50" s="32" t="n"/>
-      <c r="D50" s="35" t="n"/>
-      <c r="E50" s="32" t="n"/>
-      <c r="F50" s="32" t="n"/>
-      <c r="G50" s="32" t="n"/>
+      <c r="A50" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B50" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C50" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D50" s="35" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E50" s="32" t="inlineStr">
+        <is>
+          <t>38%</t>
+        </is>
+      </c>
+      <c r="F50" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G50" s="32" t="inlineStr">
+        <is>
+          <t>Your longest run of the plan.</t>
+        </is>
+      </c>
       <c r="H50" s="33">
         <f>IF(A50="","",COUNTIFS('Run sessions'!$A$2:$A$401,A50,'Run sessions'!$B$2:$B$401,B50))</f>
         <v/>
@@ -4890,13 +5182,37 @@
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="21">
-      <c r="A51" s="32" t="n"/>
-      <c r="B51" s="32" t="n"/>
-      <c r="C51" s="32" t="n"/>
-      <c r="D51" s="35" t="n"/>
-      <c r="E51" s="32" t="n"/>
-      <c r="F51" s="32" t="n"/>
-      <c r="G51" s="32" t="n"/>
+      <c r="A51" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B51" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C51" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D51" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E51" s="32" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="F51" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G51" s="32" t="inlineStr">
+        <is>
+          <t>Last big week: a long run with plenty of marathon pace.</t>
+        </is>
+      </c>
       <c r="H51" s="33">
         <f>IF(A51="","",COUNTIFS('Run sessions'!$A$2:$A$401,A51,'Run sessions'!$B$2:$B$401,B51))</f>
         <v/>
@@ -4911,13 +5227,37 @@
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="21">
-      <c r="A52" s="32" t="n"/>
-      <c r="B52" s="32" t="n"/>
-      <c r="C52" s="32" t="n"/>
-      <c r="D52" s="35" t="n"/>
-      <c r="E52" s="32" t="n"/>
-      <c r="F52" s="32" t="n"/>
-      <c r="G52" s="32" t="n"/>
+      <c r="A52" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B52" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C52" s="32" t="inlineStr">
+        <is>
+          <t>Taper</t>
+        </is>
+      </c>
+      <c r="D52" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E52" s="32" t="inlineStr">
+        <is>
+          <t>30%</t>
+        </is>
+      </c>
+      <c r="F52" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G52" s="32" t="inlineStr">
+        <is>
+          <t>Taper: less running, keep a little pace.</t>
+        </is>
+      </c>
       <c r="H52" s="33">
         <f>IF(A52="","",COUNTIFS('Run sessions'!$A$2:$A$401,A52,'Run sessions'!$B$2:$B$401,B52))</f>
         <v/>
@@ -4932,13 +5272,37 @@
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="21">
-      <c r="A53" s="32" t="n"/>
-      <c r="B53" s="32" t="n"/>
-      <c r="C53" s="32" t="n"/>
-      <c r="D53" s="35" t="n"/>
-      <c r="E53" s="32" t="n"/>
-      <c r="F53" s="32" t="n"/>
-      <c r="G53" s="32" t="n"/>
+      <c r="A53" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B53" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C53" s="32" t="inlineStr">
+        <is>
+          <t>Race week</t>
+        </is>
+      </c>
+      <c r="D53" s="35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E53" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="F53" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G53" s="32" t="inlineStr">
+        <is>
+          <t>Race day!</t>
+        </is>
+      </c>
       <c r="H53" s="33">
         <f>IF(A53="","",COUNTIFS('Run sessions'!$A$2:$A$401,A53,'Run sessions'!$B$2:$B$401,B53))</f>
         <v/>
@@ -16442,714 +16806,2294 @@
       <c r="G141" s="32" t="n"/>
     </row>
     <row r="142" ht="15" customHeight="1" s="21">
-      <c r="A142" s="32" t="n"/>
-      <c r="B142" s="32" t="n"/>
-      <c r="C142" s="32" t="n"/>
-      <c r="D142" s="32" t="n"/>
-      <c r="E142" s="32" t="n"/>
-      <c r="F142" s="32" t="n"/>
+      <c r="A142" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B142" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C142" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E142" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F142" s="32" t="inlineStr">
+        <is>
+          <t>6 x 1 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G142" s="32" t="n"/>
     </row>
     <row r="143" ht="15" customHeight="1" s="21">
-      <c r="A143" s="32" t="n"/>
-      <c r="B143" s="32" t="n"/>
-      <c r="C143" s="32" t="n"/>
-      <c r="D143" s="32" t="n"/>
-      <c r="E143" s="32" t="n"/>
-      <c r="F143" s="32" t="n"/>
+      <c r="A143" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B143" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C143" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D143" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E143" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F143" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G143" s="32" t="n"/>
     </row>
     <row r="144" ht="15" customHeight="1" s="21">
-      <c r="A144" s="32" t="n"/>
-      <c r="B144" s="32" t="n"/>
-      <c r="C144" s="32" t="n"/>
-      <c r="D144" s="32" t="n"/>
-      <c r="E144" s="32" t="n"/>
-      <c r="F144" s="32" t="n"/>
+      <c r="A144" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B144" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C144" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D144" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E144" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F144" s="32" t="inlineStr">
+        <is>
+          <t>5 km E → 4 km STEADY → 2 km M</t>
+        </is>
+      </c>
       <c r="G144" s="32" t="n"/>
     </row>
     <row r="145" ht="15" customHeight="1" s="21">
-      <c r="A145" s="32" t="n"/>
-      <c r="B145" s="32" t="n"/>
-      <c r="C145" s="32" t="n"/>
-      <c r="D145" s="32" t="n"/>
-      <c r="E145" s="32" t="n"/>
-      <c r="F145" s="32" t="n"/>
+      <c r="A145" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B145" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C145" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D145" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E145" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F145" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G145" s="32" t="n"/>
     </row>
     <row r="146" ht="15" customHeight="1" s="21">
-      <c r="A146" s="32" t="n"/>
-      <c r="B146" s="32" t="n"/>
-      <c r="C146" s="32" t="n"/>
-      <c r="D146" s="32" t="n"/>
-      <c r="E146" s="32" t="n"/>
-      <c r="F146" s="32" t="n"/>
+      <c r="A146" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B146" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C146" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D146" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E146" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F146" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G146" s="32" t="n"/>
     </row>
     <row r="147" ht="15" customHeight="1" s="21">
-      <c r="A147" s="32" t="n"/>
-      <c r="B147" s="32" t="n"/>
-      <c r="C147" s="32" t="n"/>
-      <c r="D147" s="32" t="n"/>
-      <c r="E147" s="32" t="n"/>
-      <c r="F147" s="32" t="n"/>
+      <c r="A147" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B147" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C147" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E147" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F147" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1.2 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G147" s="32" t="n"/>
     </row>
     <row r="148" ht="15" customHeight="1" s="21">
-      <c r="A148" s="32" t="n"/>
-      <c r="B148" s="32" t="n"/>
-      <c r="C148" s="32" t="n"/>
-      <c r="D148" s="32" t="n"/>
-      <c r="E148" s="32" t="n"/>
-      <c r="F148" s="32" t="n"/>
+      <c r="A148" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B148" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C148" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D148" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E148" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F148" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G148" s="32" t="n"/>
     </row>
     <row r="149" ht="15" customHeight="1" s="21">
-      <c r="A149" s="32" t="n"/>
-      <c r="B149" s="32" t="n"/>
-      <c r="C149" s="32" t="n"/>
-      <c r="D149" s="32" t="n"/>
-      <c r="E149" s="32" t="n"/>
-      <c r="F149" s="32" t="n"/>
+      <c r="A149" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B149" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C149" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D149" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E149" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F149" s="32" t="inlineStr">
+        <is>
+          <t>2 x 10 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G149" s="32" t="n"/>
     </row>
     <row r="150" ht="15" customHeight="1" s="21">
-      <c r="A150" s="32" t="n"/>
-      <c r="B150" s="32" t="n"/>
-      <c r="C150" s="32" t="n"/>
-      <c r="D150" s="32" t="n"/>
-      <c r="E150" s="32" t="n"/>
-      <c r="F150" s="32" t="n"/>
+      <c r="A150" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B150" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C150" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D150" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E150" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F150" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G150" s="32" t="n"/>
     </row>
     <row r="151" ht="15" customHeight="1" s="21">
-      <c r="A151" s="32" t="n"/>
-      <c r="B151" s="32" t="n"/>
-      <c r="C151" s="32" t="n"/>
-      <c r="D151" s="32" t="n"/>
-      <c r="E151" s="32" t="n"/>
-      <c r="F151" s="32" t="n"/>
+      <c r="A151" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B151" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C151" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D151" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E151" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F151" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G151" s="32" t="n"/>
     </row>
     <row r="152" ht="15" customHeight="1" s="21">
-      <c r="A152" s="32" t="n"/>
-      <c r="B152" s="32" t="n"/>
-      <c r="C152" s="32" t="n"/>
-      <c r="D152" s="32" t="n"/>
-      <c r="E152" s="32" t="n"/>
-      <c r="F152" s="32" t="n"/>
+      <c r="A152" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B152" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C152" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E152" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F152" s="32" t="inlineStr">
+        <is>
+          <t>4 x 1.6 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G152" s="32" t="n"/>
     </row>
     <row r="153" ht="15" customHeight="1" s="21">
-      <c r="A153" s="32" t="n"/>
-      <c r="B153" s="32" t="n"/>
-      <c r="C153" s="32" t="n"/>
-      <c r="D153" s="32" t="n"/>
-      <c r="E153" s="32" t="n"/>
-      <c r="F153" s="32" t="n"/>
+      <c r="A153" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B153" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C153" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D153" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E153" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F153" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G153" s="32" t="n"/>
     </row>
     <row r="154" ht="15" customHeight="1" s="21">
-      <c r="A154" s="32" t="n"/>
-      <c r="B154" s="32" t="n"/>
-      <c r="C154" s="32" t="n"/>
-      <c r="D154" s="32" t="n"/>
-      <c r="E154" s="32" t="n"/>
-      <c r="F154" s="32" t="n"/>
+      <c r="A154" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B154" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C154" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D154" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E154" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F154" s="32" t="inlineStr">
+        <is>
+          <t>3 x 3 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G154" s="32" t="n"/>
     </row>
     <row r="155" ht="15" customHeight="1" s="21">
-      <c r="A155" s="32" t="n"/>
-      <c r="B155" s="32" t="n"/>
-      <c r="C155" s="32" t="n"/>
-      <c r="D155" s="32" t="n"/>
-      <c r="E155" s="32" t="n"/>
-      <c r="F155" s="32" t="n"/>
+      <c r="A155" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B155" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C155" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D155" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E155" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F155" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G155" s="32" t="n"/>
     </row>
     <row r="156" ht="15" customHeight="1" s="21">
-      <c r="A156" s="32" t="n"/>
-      <c r="B156" s="32" t="n"/>
-      <c r="C156" s="32" t="n"/>
-      <c r="D156" s="32" t="n"/>
-      <c r="E156" s="32" t="n"/>
-      <c r="F156" s="32" t="n"/>
+      <c r="A156" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B156" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C156" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D156" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E156" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F156" s="32" t="inlineStr">
+        <is>
+          <t>16 km E, final 3 km @ STEADY</t>
+        </is>
+      </c>
       <c r="G156" s="32" t="n"/>
     </row>
     <row r="157" ht="15" customHeight="1" s="21">
-      <c r="A157" s="32" t="n"/>
-      <c r="B157" s="32" t="n"/>
-      <c r="C157" s="32" t="n"/>
-      <c r="D157" s="32" t="n"/>
-      <c r="E157" s="32" t="n"/>
-      <c r="F157" s="32" t="n"/>
+      <c r="A157" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B157" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C157" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E157" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F157" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G157" s="32" t="n"/>
     </row>
     <row r="158" ht="15" customHeight="1" s="21">
-      <c r="A158" s="32" t="n"/>
-      <c r="B158" s="32" t="n"/>
-      <c r="C158" s="32" t="n"/>
-      <c r="D158" s="32" t="n"/>
-      <c r="E158" s="32" t="n"/>
-      <c r="F158" s="32" t="n"/>
+      <c r="A158" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B158" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C158" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D158" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E158" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F158" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G158" s="32" t="n"/>
     </row>
     <row r="159" ht="15" customHeight="1" s="21">
-      <c r="A159" s="32" t="n"/>
-      <c r="B159" s="32" t="n"/>
-      <c r="C159" s="32" t="n"/>
-      <c r="D159" s="32" t="n"/>
-      <c r="E159" s="32" t="n"/>
-      <c r="F159" s="32" t="n"/>
+      <c r="A159" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B159" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C159" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D159" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E159" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F159" s="32" t="inlineStr">
+        <is>
+          <t>4 km E → 3 km STEADY</t>
+        </is>
+      </c>
       <c r="G159" s="32" t="n"/>
     </row>
     <row r="160" ht="15" customHeight="1" s="21">
-      <c r="A160" s="32" t="n"/>
-      <c r="B160" s="32" t="n"/>
-      <c r="C160" s="32" t="n"/>
-      <c r="D160" s="32" t="n"/>
-      <c r="E160" s="32" t="n"/>
-      <c r="F160" s="32" t="n"/>
+      <c r="A160" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B160" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C160" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D160" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E160" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F160" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G160" s="32" t="n"/>
     </row>
     <row r="161" ht="15" customHeight="1" s="21">
-      <c r="A161" s="32" t="n"/>
-      <c r="B161" s="32" t="n"/>
-      <c r="C161" s="32" t="n"/>
-      <c r="D161" s="32" t="n"/>
-      <c r="E161" s="32" t="n"/>
-      <c r="F161" s="32" t="n"/>
+      <c r="A161" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B161" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C161" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D161" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E161" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F161" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G161" s="32" t="n"/>
     </row>
     <row r="162" ht="15" customHeight="1" s="21">
-      <c r="A162" s="32" t="n"/>
-      <c r="B162" s="32" t="n"/>
-      <c r="C162" s="32" t="n"/>
-      <c r="D162" s="32" t="n"/>
-      <c r="E162" s="32" t="n"/>
-      <c r="F162" s="32" t="n"/>
+      <c r="A162" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B162" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C162" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E162" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F162" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1.6 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G162" s="32" t="n"/>
     </row>
     <row r="163" ht="15" customHeight="1" s="21">
-      <c r="A163" s="32" t="n"/>
-      <c r="B163" s="32" t="n"/>
-      <c r="C163" s="32" t="n"/>
-      <c r="D163" s="32" t="n"/>
-      <c r="E163" s="32" t="n"/>
-      <c r="F163" s="32" t="n"/>
+      <c r="A163" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B163" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C163" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D163" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E163" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F163" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G163" s="32" t="n"/>
     </row>
     <row r="164" ht="15" customHeight="1" s="21">
-      <c r="A164" s="32" t="n"/>
-      <c r="B164" s="32" t="n"/>
-      <c r="C164" s="32" t="n"/>
-      <c r="D164" s="32" t="n"/>
-      <c r="E164" s="32" t="n"/>
-      <c r="F164" s="32" t="n"/>
+      <c r="A164" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B164" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C164" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D164" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E164" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F164" s="32" t="inlineStr">
+        <is>
+          <t>2 x 4 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G164" s="32" t="n"/>
     </row>
     <row r="165" ht="15" customHeight="1" s="21">
-      <c r="A165" s="32" t="n"/>
-      <c r="B165" s="32" t="n"/>
-      <c r="C165" s="32" t="n"/>
-      <c r="D165" s="32" t="n"/>
-      <c r="E165" s="32" t="n"/>
-      <c r="F165" s="32" t="n"/>
+      <c r="A165" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B165" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C165" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D165" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E165" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F165" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G165" s="32" t="n"/>
     </row>
     <row r="166" ht="15" customHeight="1" s="21">
-      <c r="A166" s="32" t="n"/>
-      <c r="B166" s="32" t="n"/>
-      <c r="C166" s="32" t="n"/>
-      <c r="D166" s="32" t="n"/>
-      <c r="E166" s="32" t="n"/>
-      <c r="F166" s="32" t="n"/>
+      <c r="A166" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B166" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C166" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D166" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E166" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F166" s="32" t="inlineStr">
+        <is>
+          <t>20 km E, final 5 km @ M</t>
+        </is>
+      </c>
       <c r="G166" s="32" t="n"/>
     </row>
     <row r="167" ht="15" customHeight="1" s="21">
-      <c r="A167" s="32" t="n"/>
-      <c r="B167" s="32" t="n"/>
-      <c r="C167" s="32" t="n"/>
-      <c r="D167" s="32" t="n"/>
-      <c r="E167" s="32" t="n"/>
-      <c r="F167" s="32" t="n"/>
+      <c r="A167" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B167" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C167" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E167" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F167" s="32" t="inlineStr">
+        <is>
+          <t>3 x 3 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G167" s="32" t="n"/>
     </row>
     <row r="168" ht="15" customHeight="1" s="21">
-      <c r="A168" s="32" t="n"/>
-      <c r="B168" s="32" t="n"/>
-      <c r="C168" s="32" t="n"/>
-      <c r="D168" s="32" t="n"/>
-      <c r="E168" s="32" t="n"/>
-      <c r="F168" s="32" t="n"/>
+      <c r="A168" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B168" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C168" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E168" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F168" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G168" s="32" t="n"/>
     </row>
     <row r="169" ht="15" customHeight="1" s="21">
-      <c r="A169" s="32" t="n"/>
-      <c r="B169" s="32" t="n"/>
-      <c r="C169" s="32" t="n"/>
-      <c r="D169" s="32" t="n"/>
-      <c r="E169" s="32" t="n"/>
-      <c r="F169" s="32" t="n"/>
+      <c r="A169" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B169" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C169" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D169" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E169" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F169" s="32" t="inlineStr">
+        <is>
+          <t>20 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G169" s="32" t="n"/>
     </row>
     <row r="170" ht="15" customHeight="1" s="21">
-      <c r="A170" s="32" t="n"/>
-      <c r="B170" s="32" t="n"/>
-      <c r="C170" s="32" t="n"/>
-      <c r="D170" s="32" t="n"/>
-      <c r="E170" s="32" t="n"/>
-      <c r="F170" s="32" t="n"/>
+      <c r="A170" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B170" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C170" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D170" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E170" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F170" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G170" s="32" t="n"/>
     </row>
     <row r="171" ht="15" customHeight="1" s="21">
-      <c r="A171" s="32" t="n"/>
-      <c r="B171" s="32" t="n"/>
-      <c r="C171" s="32" t="n"/>
-      <c r="D171" s="32" t="n"/>
-      <c r="E171" s="32" t="n"/>
-      <c r="F171" s="32" t="n"/>
+      <c r="A171" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B171" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C171" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D171" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E171" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F171" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G171" s="32" t="n"/>
     </row>
     <row r="172" ht="15" customHeight="1" s="21">
-      <c r="A172" s="32" t="n"/>
-      <c r="B172" s="32" t="n"/>
-      <c r="C172" s="32" t="n"/>
-      <c r="D172" s="32" t="n"/>
-      <c r="E172" s="32" t="n"/>
-      <c r="F172" s="32" t="n"/>
+      <c r="A172" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B172" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C172" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D172" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E172" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F172" s="32" t="inlineStr">
+        <is>
+          <t>6 x 1.6 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G172" s="32" t="n"/>
     </row>
     <row r="173" ht="15" customHeight="1" s="21">
-      <c r="A173" s="32" t="n"/>
-      <c r="B173" s="32" t="n"/>
-      <c r="C173" s="32" t="n"/>
-      <c r="D173" s="32" t="n"/>
-      <c r="E173" s="32" t="n"/>
-      <c r="F173" s="32" t="n"/>
+      <c r="A173" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B173" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C173" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D173" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E173" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F173" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G173" s="32" t="n"/>
     </row>
     <row r="174" ht="15" customHeight="1" s="21">
-      <c r="A174" s="32" t="n"/>
-      <c r="B174" s="32" t="n"/>
-      <c r="C174" s="32" t="n"/>
-      <c r="D174" s="32" t="n"/>
-      <c r="E174" s="32" t="n"/>
-      <c r="F174" s="32" t="n"/>
+      <c r="A174" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B174" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C174" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D174" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E174" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F174" s="32" t="inlineStr">
+        <is>
+          <t>3 x 4 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G174" s="32" t="n"/>
     </row>
     <row r="175" ht="15" customHeight="1" s="21">
-      <c r="A175" s="32" t="n"/>
-      <c r="B175" s="32" t="n"/>
-      <c r="C175" s="32" t="n"/>
-      <c r="D175" s="32" t="n"/>
-      <c r="E175" s="32" t="n"/>
-      <c r="F175" s="32" t="n"/>
+      <c r="A175" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B175" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C175" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D175" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E175" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F175" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G175" s="32" t="n"/>
     </row>
     <row r="176" ht="15" customHeight="1" s="21">
-      <c r="A176" s="32" t="n"/>
-      <c r="B176" s="32" t="n"/>
-      <c r="C176" s="32" t="n"/>
-      <c r="D176" s="32" t="n"/>
-      <c r="E176" s="32" t="n"/>
-      <c r="F176" s="32" t="n"/>
+      <c r="A176" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B176" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C176" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D176" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E176" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F176" s="32" t="inlineStr">
+        <is>
+          <t>22 km E, final 8 km @ M</t>
+        </is>
+      </c>
       <c r="G176" s="32" t="n"/>
     </row>
     <row r="177" ht="15" customHeight="1" s="21">
-      <c r="A177" s="32" t="n"/>
-      <c r="B177" s="32" t="n"/>
-      <c r="C177" s="32" t="n"/>
-      <c r="D177" s="32" t="n"/>
-      <c r="E177" s="32" t="n"/>
-      <c r="F177" s="32" t="n"/>
+      <c r="A177" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B177" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C177" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D177" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E177" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F177" s="32" t="inlineStr">
+        <is>
+          <t>4 x 1.6 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G177" s="32" t="n"/>
     </row>
     <row r="178" ht="15" customHeight="1" s="21">
-      <c r="A178" s="32" t="n"/>
-      <c r="B178" s="32" t="n"/>
-      <c r="C178" s="32" t="n"/>
-      <c r="D178" s="32" t="n"/>
-      <c r="E178" s="32" t="n"/>
-      <c r="F178" s="32" t="n"/>
+      <c r="A178" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B178" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C178" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D178" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E178" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F178" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G178" s="32" t="n"/>
     </row>
     <row r="179" ht="15" customHeight="1" s="21">
-      <c r="A179" s="32" t="n"/>
-      <c r="B179" s="32" t="n"/>
-      <c r="C179" s="32" t="n"/>
-      <c r="D179" s="32" t="n"/>
-      <c r="E179" s="32" t="n"/>
-      <c r="F179" s="32" t="n"/>
+      <c r="A179" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B179" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C179" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D179" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E179" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F179" s="32" t="inlineStr">
+        <is>
+          <t>4 km E → 4 km STEADY → 2 km M</t>
+        </is>
+      </c>
       <c r="G179" s="32" t="n"/>
     </row>
     <row r="180" ht="15" customHeight="1" s="21">
-      <c r="A180" s="32" t="n"/>
-      <c r="B180" s="32" t="n"/>
-      <c r="C180" s="32" t="n"/>
-      <c r="D180" s="32" t="n"/>
-      <c r="E180" s="32" t="n"/>
-      <c r="F180" s="32" t="n"/>
+      <c r="A180" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B180" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C180" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D180" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E180" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F180" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G180" s="32" t="n"/>
     </row>
     <row r="181" ht="15" customHeight="1" s="21">
-      <c r="A181" s="32" t="n"/>
-      <c r="B181" s="32" t="n"/>
-      <c r="C181" s="32" t="n"/>
-      <c r="D181" s="32" t="n"/>
-      <c r="E181" s="32" t="n"/>
-      <c r="F181" s="32" t="n"/>
+      <c r="A181" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B181" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C181" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D181" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E181" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F181" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G181" s="32" t="n"/>
     </row>
     <row r="182" ht="15" customHeight="1" s="21">
-      <c r="A182" s="32" t="n"/>
-      <c r="B182" s="32" t="n"/>
-      <c r="C182" s="32" t="n"/>
-      <c r="D182" s="32" t="n"/>
-      <c r="E182" s="32" t="n"/>
-      <c r="F182" s="32" t="n"/>
+      <c r="A182" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B182" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C182" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D182" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E182" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F182" s="32" t="inlineStr">
+        <is>
+          <t>4 x 3 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G182" s="32" t="n"/>
     </row>
     <row r="183" ht="15" customHeight="1" s="21">
-      <c r="A183" s="32" t="n"/>
-      <c r="B183" s="32" t="n"/>
-      <c r="C183" s="32" t="n"/>
-      <c r="D183" s="32" t="n"/>
-      <c r="E183" s="32" t="n"/>
-      <c r="F183" s="32" t="n"/>
+      <c r="A183" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B183" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C183" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D183" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E183" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F183" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G183" s="32" t="n"/>
     </row>
     <row r="184" ht="15" customHeight="1" s="21">
-      <c r="A184" s="32" t="n"/>
-      <c r="B184" s="32" t="n"/>
-      <c r="C184" s="32" t="n"/>
-      <c r="D184" s="32" t="n"/>
-      <c r="E184" s="32" t="n"/>
-      <c r="F184" s="32" t="n"/>
+      <c r="A184" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B184" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C184" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D184" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E184" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F184" s="32" t="inlineStr">
+        <is>
+          <t>50 min continuous @ M</t>
+        </is>
+      </c>
       <c r="G184" s="32" t="n"/>
     </row>
     <row r="185" ht="15" customHeight="1" s="21">
-      <c r="A185" s="32" t="n"/>
-      <c r="B185" s="32" t="n"/>
-      <c r="C185" s="32" t="n"/>
-      <c r="D185" s="32" t="n"/>
-      <c r="E185" s="32" t="n"/>
-      <c r="F185" s="32" t="n"/>
+      <c r="A185" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B185" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C185" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D185" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E185" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F185" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G185" s="32" t="n"/>
     </row>
     <row r="186" ht="15" customHeight="1" s="21">
-      <c r="A186" s="32" t="n"/>
-      <c r="B186" s="32" t="n"/>
-      <c r="C186" s="32" t="n"/>
-      <c r="D186" s="32" t="n"/>
-      <c r="E186" s="32" t="n"/>
-      <c r="F186" s="32" t="n"/>
+      <c r="A186" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B186" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C186" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D186" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E186" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F186" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G186" s="32" t="n"/>
     </row>
     <row r="187" ht="15" customHeight="1" s="21">
-      <c r="A187" s="32" t="n"/>
-      <c r="B187" s="32" t="n"/>
-      <c r="C187" s="32" t="n"/>
-      <c r="D187" s="32" t="n"/>
-      <c r="E187" s="32" t="n"/>
-      <c r="F187" s="32" t="n"/>
+      <c r="A187" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B187" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C187" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D187" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E187" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F187" s="32" t="inlineStr">
+        <is>
+          <t>5 x 2 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G187" s="32" t="n"/>
     </row>
     <row r="188" ht="15" customHeight="1" s="21">
-      <c r="A188" s="32" t="n"/>
-      <c r="B188" s="32" t="n"/>
-      <c r="C188" s="32" t="n"/>
-      <c r="D188" s="32" t="n"/>
-      <c r="E188" s="32" t="n"/>
-      <c r="F188" s="32" t="n"/>
+      <c r="A188" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B188" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C188" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D188" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E188" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F188" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G188" s="32" t="n"/>
     </row>
     <row r="189" ht="15" customHeight="1" s="21">
-      <c r="A189" s="32" t="n"/>
-      <c r="B189" s="32" t="n"/>
-      <c r="C189" s="32" t="n"/>
-      <c r="D189" s="32" t="n"/>
-      <c r="E189" s="32" t="n"/>
-      <c r="F189" s="32" t="n"/>
+      <c r="A189" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B189" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C189" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D189" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E189" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F189" s="32" t="inlineStr">
+        <is>
+          <t>25 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G189" s="32" t="n"/>
     </row>
     <row r="190" ht="15" customHeight="1" s="21">
-      <c r="A190" s="32" t="n"/>
-      <c r="B190" s="32" t="n"/>
-      <c r="C190" s="32" t="n"/>
-      <c r="D190" s="32" t="n"/>
-      <c r="E190" s="32" t="n"/>
-      <c r="F190" s="32" t="n"/>
+      <c r="A190" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B190" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C190" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D190" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E190" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F190" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G190" s="32" t="n"/>
     </row>
     <row r="191" ht="15" customHeight="1" s="21">
-      <c r="A191" s="32" t="n"/>
-      <c r="B191" s="32" t="n"/>
-      <c r="C191" s="32" t="n"/>
-      <c r="D191" s="32" t="n"/>
-      <c r="E191" s="32" t="n"/>
-      <c r="F191" s="32" t="n"/>
+      <c r="A191" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B191" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C191" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D191" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E191" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F191" s="32" t="inlineStr">
+        <is>
+          <t>26 km E, final 12 km @ M</t>
+        </is>
+      </c>
       <c r="G191" s="32" t="n"/>
     </row>
     <row r="192" ht="15" customHeight="1" s="21">
-      <c r="A192" s="32" t="n"/>
-      <c r="B192" s="32" t="n"/>
-      <c r="C192" s="32" t="n"/>
-      <c r="D192" s="32" t="n"/>
-      <c r="E192" s="32" t="n"/>
-      <c r="F192" s="32" t="n"/>
+      <c r="A192" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B192" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C192" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D192" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E192" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F192" s="32" t="inlineStr">
+        <is>
+          <t>6 x 1.6 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G192" s="32" t="n"/>
     </row>
     <row r="193" ht="15" customHeight="1" s="21">
-      <c r="A193" s="32" t="n"/>
-      <c r="B193" s="32" t="n"/>
-      <c r="C193" s="32" t="n"/>
-      <c r="D193" s="32" t="n"/>
-      <c r="E193" s="32" t="n"/>
-      <c r="F193" s="32" t="n"/>
+      <c r="A193" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B193" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C193" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D193" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E193" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F193" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G193" s="32" t="n"/>
     </row>
     <row r="194" ht="15" customHeight="1" s="21">
-      <c r="A194" s="32" t="n"/>
-      <c r="B194" s="32" t="n"/>
-      <c r="C194" s="32" t="n"/>
-      <c r="D194" s="32" t="n"/>
-      <c r="E194" s="32" t="n"/>
-      <c r="F194" s="32" t="n"/>
+      <c r="A194" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B194" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C194" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D194" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E194" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F194" s="32" t="inlineStr">
+        <is>
+          <t>3 x 5 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G194" s="32" t="n"/>
     </row>
     <row r="195" ht="15" customHeight="1" s="21">
-      <c r="A195" s="32" t="n"/>
-      <c r="B195" s="32" t="n"/>
-      <c r="C195" s="32" t="n"/>
-      <c r="D195" s="32" t="n"/>
-      <c r="E195" s="32" t="n"/>
-      <c r="F195" s="32" t="n"/>
+      <c r="A195" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B195" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C195" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D195" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E195" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F195" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G195" s="32" t="n"/>
     </row>
     <row r="196" ht="15" customHeight="1" s="21">
-      <c r="A196" s="32" t="n"/>
-      <c r="B196" s="32" t="n"/>
-      <c r="C196" s="32" t="n"/>
-      <c r="D196" s="32" t="n"/>
-      <c r="E196" s="32" t="n"/>
-      <c r="F196" s="32" t="n"/>
+      <c r="A196" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B196" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C196" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D196" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E196" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F196" s="32" t="inlineStr">
+        <is>
+          <t>30 km E, final 5 km @ STEADY</t>
+        </is>
+      </c>
       <c r="G196" s="32" t="n"/>
     </row>
     <row r="197" ht="15" customHeight="1" s="21">
-      <c r="A197" s="32" t="n"/>
-      <c r="B197" s="32" t="n"/>
-      <c r="C197" s="32" t="n"/>
-      <c r="D197" s="32" t="n"/>
-      <c r="E197" s="32" t="n"/>
-      <c r="F197" s="32" t="n"/>
+      <c r="A197" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B197" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C197" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E197" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F197" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1 km @ T, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G197" s="32" t="n"/>
     </row>
     <row r="198" ht="15" customHeight="1" s="21">
-      <c r="A198" s="32" t="n"/>
-      <c r="B198" s="32" t="n"/>
-      <c r="C198" s="32" t="n"/>
-      <c r="D198" s="32" t="n"/>
-      <c r="E198" s="32" t="n"/>
-      <c r="F198" s="32" t="n"/>
+      <c r="A198" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B198" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C198" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D198" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E198" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F198" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G198" s="32" t="n"/>
     </row>
     <row r="199" ht="15" customHeight="1" s="21">
-      <c r="A199" s="32" t="n"/>
-      <c r="B199" s="32" t="n"/>
-      <c r="C199" s="32" t="n"/>
-      <c r="D199" s="32" t="n"/>
-      <c r="E199" s="32" t="n"/>
-      <c r="F199" s="32" t="n"/>
+      <c r="A199" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B199" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C199" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D199" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E199" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F199" s="32" t="inlineStr">
+        <is>
+          <t>5 km E → 5 km M</t>
+        </is>
+      </c>
       <c r="G199" s="32" t="n"/>
     </row>
     <row r="200" ht="15" customHeight="1" s="21">
-      <c r="A200" s="32" t="n"/>
-      <c r="B200" s="32" t="n"/>
-      <c r="C200" s="32" t="n"/>
-      <c r="D200" s="32" t="n"/>
-      <c r="E200" s="32" t="n"/>
-      <c r="F200" s="32" t="n"/>
+      <c r="A200" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B200" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C200" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D200" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E200" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F200" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G200" s="32" t="n"/>
     </row>
     <row r="201" ht="15" customHeight="1" s="21">
-      <c r="A201" s="32" t="n"/>
-      <c r="B201" s="32" t="n"/>
-      <c r="C201" s="32" t="n"/>
-      <c r="D201" s="32" t="n"/>
-      <c r="E201" s="32" t="n"/>
-      <c r="F201" s="32" t="n"/>
+      <c r="A201" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B201" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C201" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D201" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E201" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F201" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G201" s="32" t="n"/>
     </row>
     <row r="202" ht="15" customHeight="1" s="21">
-      <c r="A202" s="32" t="n"/>
-      <c r="B202" s="32" t="n"/>
-      <c r="C202" s="32" t="n"/>
-      <c r="D202" s="32" t="n"/>
-      <c r="E202" s="32" t="n"/>
-      <c r="F202" s="32" t="n"/>
+      <c r="A202" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B202" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C202" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D202" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E202" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F202" s="32" t="inlineStr">
+        <is>
+          <t>4 x 3 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G202" s="32" t="n"/>
     </row>
     <row r="203" ht="15" customHeight="1" s="21">
-      <c r="A203" s="32" t="n"/>
-      <c r="B203" s="32" t="n"/>
-      <c r="C203" s="32" t="n"/>
-      <c r="D203" s="32" t="n"/>
-      <c r="E203" s="32" t="n"/>
-      <c r="F203" s="32" t="n"/>
+      <c r="A203" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B203" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C203" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D203" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E203" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F203" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G203" s="32" t="n"/>
     </row>
     <row r="204" ht="15" customHeight="1" s="21">
-      <c r="A204" s="32" t="n"/>
-      <c r="B204" s="32" t="n"/>
-      <c r="C204" s="32" t="n"/>
-      <c r="D204" s="32" t="n"/>
-      <c r="E204" s="32" t="n"/>
-      <c r="F204" s="32" t="n"/>
+      <c r="A204" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B204" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C204" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D204" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E204" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F204" s="32" t="inlineStr">
+        <is>
+          <t>60 min continuous @ M</t>
+        </is>
+      </c>
       <c r="G204" s="32" t="n"/>
     </row>
     <row r="205" ht="15" customHeight="1" s="21">
-      <c r="A205" s="32" t="n"/>
-      <c r="B205" s="32" t="n"/>
-      <c r="C205" s="32" t="n"/>
-      <c r="D205" s="32" t="n"/>
-      <c r="E205" s="32" t="n"/>
-      <c r="F205" s="32" t="n"/>
+      <c r="A205" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B205" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C205" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D205" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E205" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F205" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G205" s="32" t="n"/>
     </row>
     <row r="206" ht="15" customHeight="1" s="21">
-      <c r="A206" s="32" t="n"/>
-      <c r="B206" s="32" t="n"/>
-      <c r="C206" s="32" t="n"/>
-      <c r="D206" s="32" t="n"/>
-      <c r="E206" s="32" t="n"/>
-      <c r="F206" s="32" t="n"/>
+      <c r="A206" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B206" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="C206" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D206" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E206" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F206" s="32" t="inlineStr">
+        <is>
+          <t>Longest run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G206" s="32" t="n"/>
     </row>
     <row r="207" ht="15" customHeight="1" s="21">
-      <c r="A207" s="32" t="n"/>
-      <c r="B207" s="32" t="n"/>
-      <c r="C207" s="32" t="n"/>
-      <c r="D207" s="32" t="n"/>
-      <c r="E207" s="32" t="n"/>
-      <c r="F207" s="32" t="n"/>
+      <c r="A207" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B207" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C207" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E207" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F207" s="32" t="inlineStr">
+        <is>
+          <t>5 x 2 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G207" s="32" t="n"/>
     </row>
     <row r="208" ht="15" customHeight="1" s="21">
-      <c r="A208" s="32" t="n"/>
-      <c r="B208" s="32" t="n"/>
-      <c r="C208" s="32" t="n"/>
-      <c r="D208" s="32" t="n"/>
-      <c r="E208" s="32" t="n"/>
-      <c r="F208" s="32" t="n"/>
+      <c r="A208" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B208" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C208" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D208" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E208" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F208" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G208" s="32" t="n"/>
     </row>
     <row r="209" ht="15" customHeight="1" s="21">
-      <c r="A209" s="32" t="n"/>
-      <c r="B209" s="32" t="n"/>
-      <c r="C209" s="32" t="n"/>
-      <c r="D209" s="32" t="n"/>
-      <c r="E209" s="32" t="n"/>
-      <c r="F209" s="32" t="n"/>
+      <c r="A209" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B209" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C209" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D209" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E209" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F209" s="32" t="inlineStr">
+        <is>
+          <t>2 x 6 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G209" s="32" t="n"/>
     </row>
     <row r="210" ht="15" customHeight="1" s="21">
-      <c r="A210" s="32" t="n"/>
-      <c r="B210" s="32" t="n"/>
-      <c r="C210" s="32" t="n"/>
-      <c r="D210" s="32" t="n"/>
-      <c r="E210" s="32" t="n"/>
-      <c r="F210" s="32" t="n"/>
+      <c r="A210" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B210" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C210" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D210" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E210" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F210" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G210" s="32" t="n"/>
     </row>
     <row r="211" ht="15" customHeight="1" s="21">
-      <c r="A211" s="32" t="n"/>
-      <c r="B211" s="32" t="n"/>
-      <c r="C211" s="32" t="n"/>
-      <c r="D211" s="32" t="n"/>
-      <c r="E211" s="32" t="n"/>
-      <c r="F211" s="32" t="n"/>
+      <c r="A211" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B211" s="32" t="n">
+        <v>14</v>
+      </c>
+      <c r="C211" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D211" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E211" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F211" s="32" t="inlineStr">
+        <is>
+          <t>24 km E, final 12 km @ M</t>
+        </is>
+      </c>
       <c r="G211" s="32" t="n"/>
     </row>
     <row r="212" ht="15" customHeight="1" s="21">
-      <c r="A212" s="32" t="n"/>
-      <c r="B212" s="32" t="n"/>
-      <c r="C212" s="32" t="n"/>
-      <c r="D212" s="32" t="n"/>
-      <c r="E212" s="32" t="n"/>
-      <c r="F212" s="32" t="n"/>
+      <c r="A212" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B212" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C212" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D212" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E212" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F212" s="32" t="inlineStr">
+        <is>
+          <t>4 x 1.6 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G212" s="32" t="n"/>
     </row>
     <row r="213" ht="15" customHeight="1" s="21">
-      <c r="A213" s="32" t="n"/>
-      <c r="B213" s="32" t="n"/>
-      <c r="C213" s="32" t="n"/>
-      <c r="D213" s="32" t="n"/>
-      <c r="E213" s="32" t="n"/>
-      <c r="F213" s="32" t="n"/>
+      <c r="A213" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B213" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C213" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D213" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E213" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F213" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G213" s="32" t="n"/>
     </row>
     <row r="214" ht="15" customHeight="1" s="21">
-      <c r="A214" s="32" t="n"/>
-      <c r="B214" s="32" t="n"/>
-      <c r="C214" s="32" t="n"/>
-      <c r="D214" s="32" t="n"/>
-      <c r="E214" s="32" t="n"/>
-      <c r="F214" s="32" t="n"/>
+      <c r="A214" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B214" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C214" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D214" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E214" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F214" s="32" t="inlineStr">
+        <is>
+          <t>2 x 4 km @ M, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G214" s="32" t="n"/>
     </row>
     <row r="215" ht="15" customHeight="1" s="21">
-      <c r="A215" s="32" t="n"/>
-      <c r="B215" s="32" t="n"/>
-      <c r="C215" s="32" t="n"/>
-      <c r="D215" s="32" t="n"/>
-      <c r="E215" s="32" t="n"/>
-      <c r="F215" s="32" t="n"/>
+      <c r="A215" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B215" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C215" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D215" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E215" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F215" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G215" s="32" t="n"/>
     </row>
     <row r="216" ht="15" customHeight="1" s="21">
-      <c r="A216" s="32" t="n"/>
-      <c r="B216" s="32" t="n"/>
-      <c r="C216" s="32" t="n"/>
-      <c r="D216" s="32" t="n"/>
-      <c r="E216" s="32" t="n"/>
-      <c r="F216" s="32" t="n"/>
+      <c r="A216" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B216" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="C216" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D216" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E216" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F216" s="32" t="inlineStr">
+        <is>
+          <t>18 km E, final 4 km @ M</t>
+        </is>
+      </c>
       <c r="G216" s="32" t="n"/>
     </row>
     <row r="217" ht="15" customHeight="1" s="21">
-      <c r="A217" s="32" t="n"/>
-      <c r="B217" s="32" t="n"/>
-      <c r="C217" s="32" t="n"/>
-      <c r="D217" s="32" t="n"/>
-      <c r="E217" s="32" t="n"/>
-      <c r="F217" s="32" t="n"/>
+      <c r="A217" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B217" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C217" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D217" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E217" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F217" s="32" t="inlineStr">
+        <is>
+          <t>6 x (1 min @ HM effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G217" s="32" t="n"/>
     </row>
     <row r="218" ht="15" customHeight="1" s="21">
-      <c r="A218" s="32" t="n"/>
-      <c r="B218" s="32" t="n"/>
-      <c r="C218" s="32" t="n"/>
-      <c r="D218" s="32" t="n"/>
-      <c r="E218" s="32" t="n"/>
-      <c r="F218" s="32" t="n"/>
+      <c r="A218" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B218" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C218" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D218" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E218" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F218" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G218" s="32" t="n"/>
     </row>
     <row r="219" ht="15" customHeight="1" s="21">
-      <c r="A219" s="32" t="n"/>
-      <c r="B219" s="32" t="n"/>
-      <c r="C219" s="32" t="n"/>
-      <c r="D219" s="32" t="n"/>
-      <c r="E219" s="32" t="n"/>
-      <c r="F219" s="32" t="n"/>
+      <c r="A219" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B219" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C219" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D219" s="32" t="inlineStr">
+        <is>
+          <t>Shakeout</t>
+        </is>
+      </c>
+      <c r="E219" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F219" s="32" t="inlineStr">
+        <is>
+          <t>4 km E + 4 x 20 s strides</t>
+        </is>
+      </c>
       <c r="G219" s="32" t="n"/>
     </row>
     <row r="220" ht="15" customHeight="1" s="21">
-      <c r="A220" s="32" t="n"/>
-      <c r="B220" s="32" t="n"/>
-      <c r="C220" s="32" t="n"/>
-      <c r="D220" s="32" t="n"/>
-      <c r="E220" s="32" t="n"/>
-      <c r="F220" s="32" t="n"/>
+      <c r="A220" s="32" t="inlineStr">
+        <is>
+          <t>Marathon</t>
+        </is>
+      </c>
+      <c r="B220" s="32" t="n">
+        <v>16</v>
+      </c>
+      <c r="C220" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D220" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="E220" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F220" s="32" t="inlineStr">
+        <is>
+          <t>MARATHON – race at goal M pace</t>
+        </is>
+      </c>
       <c r="G220" s="32" t="n"/>
     </row>
     <row r="221" ht="15" customHeight="1" s="21">
@@ -30080,7 +32024,7 @@
       </c>
       <c r="E5" s="34" t="inlineStr">
         <is>
-          <t>No run is longer than this (the programme's long-run cap can be lower).</t>
+          <t>No run is longer than this, except in race programmes (5K to marathon, Hyrox), which use their own long-run cap on the Programmes tab.</t>
         </is>
       </c>
     </row>
@@ -30455,6 +32399,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="21">
       <c r="A26" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Gym: ask whether any workout counts towards this week's plan; Faster 5K programme draft
- Starting a gym workout offers this week's unfinished gym sessions (today first), not just
  today's; one from another day is ticked off and moved to today
- Faster 5K: 12 weeks, 4 runs a week (goal-paced intervals or fartlek, easy, tempo, easy long run)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="C3" s="32" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D3" s="32" t="inlineStr">
         <is>
@@ -5317,13 +5317,37 @@
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="21">
-      <c r="A54" s="32" t="n"/>
-      <c r="B54" s="32" t="n"/>
-      <c r="C54" s="32" t="n"/>
-      <c r="D54" s="35" t="n"/>
-      <c r="E54" s="32" t="n"/>
-      <c r="F54" s="32" t="n"/>
-      <c r="G54" s="32" t="n"/>
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B54" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D54" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E54" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F54" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G54" s="32" t="inlineStr">
+        <is>
+          <t>Settle in: one quality session, the rest easy.</t>
+        </is>
+      </c>
       <c r="H54" s="33">
         <f>IF(A54="","",COUNTIFS('Run sessions'!$A$2:$A$401,A54,'Run sessions'!$B$2:$B$401,B54))</f>
         <v/>
@@ -5338,12 +5362,32 @@
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="21">
-      <c r="A55" s="32" t="n"/>
-      <c r="B55" s="32" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="35" t="n"/>
-      <c r="E55" s="32" t="n"/>
-      <c r="F55" s="32" t="n"/>
+      <c r="A55" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B55" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D55" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E55" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F55" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G55" s="32" t="n"/>
       <c r="H55" s="33">
         <f>IF(A55="","",COUNTIFS('Run sessions'!$A$2:$A$401,A55,'Run sessions'!$B$2:$B$401,B55))</f>
@@ -5359,12 +5403,32 @@
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="21">
-      <c r="A56" s="32" t="n"/>
-      <c r="B56" s="32" t="n"/>
-      <c r="C56" s="32" t="n"/>
-      <c r="D56" s="35" t="n"/>
-      <c r="E56" s="32" t="n"/>
-      <c r="F56" s="32" t="n"/>
+      <c r="A56" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B56" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D56" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E56" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F56" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G56" s="32" t="n"/>
       <c r="H56" s="33">
         <f>IF(A56="","",COUNTIFS('Run sessions'!$A$2:$A$401,A56,'Run sessions'!$B$2:$B$401,B56))</f>
@@ -5380,13 +5444,37 @@
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="21">
-      <c r="A57" s="32" t="n"/>
-      <c r="B57" s="32" t="n"/>
-      <c r="C57" s="32" t="n"/>
-      <c r="D57" s="35" t="n"/>
-      <c r="E57" s="32" t="n"/>
-      <c r="F57" s="32" t="n"/>
-      <c r="G57" s="32" t="n"/>
+      <c r="A57" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B57" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D57" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E57" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F57" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G57" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week: let the work sink in.</t>
+        </is>
+      </c>
       <c r="H57" s="33">
         <f>IF(A57="","",COUNTIFS('Run sessions'!$A$2:$A$401,A57,'Run sessions'!$B$2:$B$401,B57))</f>
         <v/>
@@ -5401,12 +5489,32 @@
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="21">
-      <c r="A58" s="32" t="n"/>
-      <c r="B58" s="32" t="n"/>
-      <c r="C58" s="32" t="n"/>
-      <c r="D58" s="35" t="n"/>
-      <c r="E58" s="32" t="n"/>
-      <c r="F58" s="32" t="n"/>
+      <c r="A58" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B58" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D58" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E58" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F58" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G58" s="32" t="n"/>
       <c r="H58" s="33">
         <f>IF(A58="","",COUNTIFS('Run sessions'!$A$2:$A$401,A58,'Run sessions'!$B$2:$B$401,B58))</f>
@@ -5422,12 +5530,32 @@
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="21">
-      <c r="A59" s="32" t="n"/>
-      <c r="B59" s="32" t="n"/>
-      <c r="C59" s="32" t="n"/>
-      <c r="D59" s="35" t="n"/>
-      <c r="E59" s="32" t="n"/>
-      <c r="F59" s="32" t="n"/>
+      <c r="A59" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B59" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D59" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E59" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F59" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G59" s="32" t="n"/>
       <c r="H59" s="33">
         <f>IF(A59="","",COUNTIFS('Run sessions'!$A$2:$A$401,A59,'Run sessions'!$B$2:$B$401,B59))</f>
@@ -5443,12 +5571,32 @@
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="21">
-      <c r="A60" s="32" t="n"/>
-      <c r="B60" s="32" t="n"/>
-      <c r="C60" s="32" t="n"/>
-      <c r="D60" s="35" t="n"/>
-      <c r="E60" s="32" t="n"/>
-      <c r="F60" s="32" t="n"/>
+      <c r="A60" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B60" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C60" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D60" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E60" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F60" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G60" s="32" t="n"/>
       <c r="H60" s="33">
         <f>IF(A60="","",COUNTIFS('Run sessions'!$A$2:$A$401,A60,'Run sessions'!$B$2:$B$401,B60))</f>
@@ -5464,13 +5612,37 @@
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="21">
-      <c r="A61" s="32" t="n"/>
-      <c r="B61" s="32" t="n"/>
-      <c r="C61" s="32" t="n"/>
-      <c r="D61" s="35" t="n"/>
-      <c r="E61" s="32" t="n"/>
-      <c r="F61" s="32" t="n"/>
-      <c r="G61" s="32" t="n"/>
+      <c r="A61" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B61" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C61" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D61" s="35" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E61" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F61" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G61" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week before the peak.</t>
+        </is>
+      </c>
       <c r="H61" s="33">
         <f>IF(A61="","",COUNTIFS('Run sessions'!$A$2:$A$401,A61,'Run sessions'!$B$2:$B$401,B61))</f>
         <v/>
@@ -5485,13 +5657,37 @@
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="21">
-      <c r="A62" s="32" t="n"/>
-      <c r="B62" s="32" t="n"/>
-      <c r="C62" s="32" t="n"/>
-      <c r="D62" s="35" t="n"/>
-      <c r="E62" s="32" t="n"/>
-      <c r="F62" s="32" t="n"/>
-      <c r="G62" s="32" t="n"/>
+      <c r="A62" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B62" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C62" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D62" s="35" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E62" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F62" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G62" s="32" t="inlineStr">
+        <is>
+          <t>Biggest week.</t>
+        </is>
+      </c>
       <c r="H62" s="33">
         <f>IF(A62="","",COUNTIFS('Run sessions'!$A$2:$A$401,A62,'Run sessions'!$B$2:$B$401,B62))</f>
         <v/>
@@ -5506,12 +5702,32 @@
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="21">
-      <c r="A63" s="32" t="n"/>
-      <c r="B63" s="32" t="n"/>
-      <c r="C63" s="32" t="n"/>
-      <c r="D63" s="35" t="n"/>
-      <c r="E63" s="32" t="n"/>
-      <c r="F63" s="32" t="n"/>
+      <c r="A63" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B63" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C63" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D63" s="35" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="E63" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F63" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G63" s="32" t="n"/>
       <c r="H63" s="33">
         <f>IF(A63="","",COUNTIFS('Run sessions'!$A$2:$A$401,A63,'Run sessions'!$B$2:$B$401,B63))</f>
@@ -5527,13 +5743,37 @@
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="21">
-      <c r="A64" s="32" t="n"/>
-      <c r="B64" s="32" t="n"/>
-      <c r="C64" s="32" t="n"/>
-      <c r="D64" s="35" t="n"/>
-      <c r="E64" s="32" t="n"/>
-      <c r="F64" s="32" t="n"/>
-      <c r="G64" s="32" t="n"/>
+      <c r="A64" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B64" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C64" s="32" t="inlineStr">
+        <is>
+          <t>Taper</t>
+        </is>
+      </c>
+      <c r="D64" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E64" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F64" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G64" s="32" t="inlineStr">
+        <is>
+          <t>Freshen up.</t>
+        </is>
+      </c>
       <c r="H64" s="33">
         <f>IF(A64="","",COUNTIFS('Run sessions'!$A$2:$A$401,A64,'Run sessions'!$B$2:$B$401,B64))</f>
         <v/>
@@ -5548,13 +5788,37 @@
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="21">
-      <c r="A65" s="32" t="n"/>
-      <c r="B65" s="32" t="n"/>
-      <c r="C65" s="32" t="n"/>
-      <c r="D65" s="35" t="n"/>
-      <c r="E65" s="32" t="n"/>
-      <c r="F65" s="32" t="n"/>
-      <c r="G65" s="32" t="n"/>
+      <c r="A65" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B65" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C65" s="32" t="inlineStr">
+        <is>
+          <t>Race week</t>
+        </is>
+      </c>
+      <c r="D65" s="35" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E65" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="F65" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G65" s="32" t="inlineStr">
+        <is>
+          <t>Race day!</t>
+        </is>
+      </c>
       <c r="H65" s="33">
         <f>IF(A65="","",COUNTIFS('Run sessions'!$A$2:$A$401,A65,'Run sessions'!$B$2:$B$401,B65))</f>
         <v/>
@@ -19097,435 +19361,1395 @@
       <c r="G220" s="32" t="n"/>
     </row>
     <row r="221" ht="15" customHeight="1" s="21">
-      <c r="A221" s="32" t="n"/>
-      <c r="B221" s="32" t="n"/>
-      <c r="C221" s="32" t="n"/>
-      <c r="D221" s="32" t="n"/>
-      <c r="E221" s="32" t="n"/>
-      <c r="F221" s="32" t="n"/>
+      <c r="A221" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B221" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C221" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D221" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E221" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F221" s="32" t="inlineStr">
+        <is>
+          <t>8 x (1 min @ I effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G221" s="32" t="n"/>
     </row>
     <row r="222" ht="15" customHeight="1" s="21">
-      <c r="A222" s="32" t="n"/>
-      <c r="B222" s="32" t="n"/>
-      <c r="C222" s="32" t="n"/>
-      <c r="D222" s="32" t="n"/>
-      <c r="E222" s="32" t="n"/>
-      <c r="F222" s="32" t="n"/>
+      <c r="A222" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B222" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C222" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D222" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E222" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F222" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G222" s="32" t="n"/>
     </row>
     <row r="223" ht="15" customHeight="1" s="21">
-      <c r="A223" s="32" t="n"/>
-      <c r="B223" s="32" t="n"/>
-      <c r="C223" s="32" t="n"/>
-      <c r="D223" s="32" t="n"/>
-      <c r="E223" s="32" t="n"/>
-      <c r="F223" s="32" t="n"/>
+      <c r="A223" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B223" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C223" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D223" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E223" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F223" s="32" t="inlineStr">
+        <is>
+          <t>3 km E → 2 km STEADY → 1 km T</t>
+        </is>
+      </c>
       <c r="G223" s="32" t="n"/>
     </row>
     <row r="224" ht="15" customHeight="1" s="21">
-      <c r="A224" s="32" t="n"/>
-      <c r="B224" s="32" t="n"/>
-      <c r="C224" s="32" t="n"/>
-      <c r="D224" s="32" t="n"/>
-      <c r="E224" s="32" t="n"/>
-      <c r="F224" s="32" t="n"/>
+      <c r="A224" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B224" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C224" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D224" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E224" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F224" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G224" s="32" t="n"/>
     </row>
     <row r="225" ht="15" customHeight="1" s="21">
-      <c r="A225" s="32" t="n"/>
-      <c r="B225" s="32" t="n"/>
-      <c r="C225" s="32" t="n"/>
-      <c r="D225" s="32" t="n"/>
-      <c r="E225" s="32" t="n"/>
-      <c r="F225" s="32" t="n"/>
+      <c r="A225" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B225" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C225" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D225" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E225" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F225" s="32" t="inlineStr">
+        <is>
+          <t>10 x 400 m @ I, 75 s jog between</t>
+        </is>
+      </c>
       <c r="G225" s="32" t="n"/>
     </row>
     <row r="226" ht="15" customHeight="1" s="21">
-      <c r="A226" s="32" t="n"/>
-      <c r="B226" s="32" t="n"/>
-      <c r="C226" s="32" t="n"/>
-      <c r="D226" s="32" t="n"/>
-      <c r="E226" s="32" t="n"/>
-      <c r="F226" s="32" t="n"/>
+      <c r="A226" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B226" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C226" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D226" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E226" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F226" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G226" s="32" t="n"/>
     </row>
     <row r="227" ht="15" customHeight="1" s="21">
-      <c r="A227" s="32" t="n"/>
-      <c r="B227" s="32" t="n"/>
-      <c r="C227" s="32" t="n"/>
-      <c r="D227" s="32" t="n"/>
-      <c r="E227" s="32" t="n"/>
-      <c r="F227" s="32" t="n"/>
+      <c r="A227" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B227" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C227" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D227" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E227" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F227" s="32" t="inlineStr">
+        <is>
+          <t>2 x 8 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G227" s="32" t="n"/>
     </row>
     <row r="228" ht="15" customHeight="1" s="21">
-      <c r="A228" s="32" t="n"/>
-      <c r="B228" s="32" t="n"/>
-      <c r="C228" s="32" t="n"/>
-      <c r="D228" s="32" t="n"/>
-      <c r="E228" s="32" t="n"/>
-      <c r="F228" s="32" t="n"/>
+      <c r="A228" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B228" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C228" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D228" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E228" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F228" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G228" s="32" t="n"/>
     </row>
     <row r="229" ht="15" customHeight="1" s="21">
-      <c r="A229" s="32" t="n"/>
-      <c r="B229" s="32" t="n"/>
-      <c r="C229" s="32" t="n"/>
-      <c r="D229" s="32" t="n"/>
-      <c r="E229" s="32" t="n"/>
-      <c r="F229" s="32" t="n"/>
+      <c r="A229" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B229" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C229" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D229" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E229" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F229" s="32" t="inlineStr">
+        <is>
+          <t>6 x 600 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G229" s="32" t="n"/>
     </row>
     <row r="230" ht="15" customHeight="1" s="21">
-      <c r="A230" s="32" t="n"/>
-      <c r="B230" s="32" t="n"/>
-      <c r="C230" s="32" t="n"/>
-      <c r="D230" s="32" t="n"/>
-      <c r="E230" s="32" t="n"/>
-      <c r="F230" s="32" t="n"/>
+      <c r="A230" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B230" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C230" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D230" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E230" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F230" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G230" s="32" t="n"/>
     </row>
     <row r="231" ht="15" customHeight="1" s="21">
-      <c r="A231" s="32" t="n"/>
-      <c r="B231" s="32" t="n"/>
-      <c r="C231" s="32" t="n"/>
-      <c r="D231" s="32" t="n"/>
-      <c r="E231" s="32" t="n"/>
-      <c r="F231" s="32" t="n"/>
+      <c r="A231" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B231" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C231" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D231" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E231" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F231" s="32" t="inlineStr">
+        <is>
+          <t>3 km E → 2 km STEADY → 2 km T</t>
+        </is>
+      </c>
       <c r="G231" s="32" t="n"/>
     </row>
     <row r="232" ht="15" customHeight="1" s="21">
-      <c r="A232" s="32" t="n"/>
-      <c r="B232" s="32" t="n"/>
-      <c r="C232" s="32" t="n"/>
-      <c r="D232" s="32" t="n"/>
-      <c r="E232" s="32" t="n"/>
-      <c r="F232" s="32" t="n"/>
+      <c r="A232" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B232" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C232" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D232" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E232" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F232" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G232" s="32" t="n"/>
     </row>
     <row r="233" ht="15" customHeight="1" s="21">
-      <c r="A233" s="32" t="n"/>
-      <c r="B233" s="32" t="n"/>
-      <c r="C233" s="32" t="n"/>
-      <c r="D233" s="32" t="n"/>
-      <c r="E233" s="32" t="n"/>
-      <c r="F233" s="32" t="n"/>
+      <c r="A233" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B233" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C233" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D233" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E233" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F233" s="32" t="inlineStr">
+        <is>
+          <t>6 x (2 min @ 5K effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G233" s="32" t="n"/>
     </row>
     <row r="234" ht="15" customHeight="1" s="21">
-      <c r="A234" s="32" t="n"/>
-      <c r="B234" s="32" t="n"/>
-      <c r="C234" s="32" t="n"/>
-      <c r="D234" s="32" t="n"/>
-      <c r="E234" s="32" t="n"/>
-      <c r="F234" s="32" t="n"/>
+      <c r="A234" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B234" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C234" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D234" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E234" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F234" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G234" s="32" t="n"/>
     </row>
     <row r="235" ht="15" customHeight="1" s="21">
-      <c r="A235" s="32" t="n"/>
-      <c r="B235" s="32" t="n"/>
-      <c r="C235" s="32" t="n"/>
-      <c r="D235" s="32" t="n"/>
-      <c r="E235" s="32" t="n"/>
-      <c r="F235" s="32" t="n"/>
+      <c r="A235" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B235" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C235" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D235" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E235" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F235" s="32" t="inlineStr">
+        <is>
+          <t>15 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G235" s="32" t="n"/>
     </row>
     <row r="236" ht="15" customHeight="1" s="21">
-      <c r="A236" s="32" t="n"/>
-      <c r="B236" s="32" t="n"/>
-      <c r="C236" s="32" t="n"/>
-      <c r="D236" s="32" t="n"/>
-      <c r="E236" s="32" t="n"/>
-      <c r="F236" s="32" t="n"/>
+      <c r="A236" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B236" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C236" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D236" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E236" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F236" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G236" s="32" t="n"/>
     </row>
     <row r="237" ht="15" customHeight="1" s="21">
-      <c r="A237" s="32" t="n"/>
-      <c r="B237" s="32" t="n"/>
-      <c r="C237" s="32" t="n"/>
-      <c r="D237" s="32" t="n"/>
-      <c r="E237" s="32" t="n"/>
-      <c r="F237" s="32" t="n"/>
+      <c r="A237" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B237" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C237" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D237" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E237" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F237" s="32" t="inlineStr">
+        <is>
+          <t>5 x 800 m @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G237" s="32" t="n"/>
     </row>
     <row r="238" ht="15" customHeight="1" s="21">
-      <c r="A238" s="32" t="n"/>
-      <c r="B238" s="32" t="n"/>
-      <c r="C238" s="32" t="n"/>
-      <c r="D238" s="32" t="n"/>
-      <c r="E238" s="32" t="n"/>
-      <c r="F238" s="32" t="n"/>
+      <c r="A238" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B238" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C238" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D238" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E238" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F238" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G238" s="32" t="n"/>
     </row>
     <row r="239" ht="15" customHeight="1" s="21">
-      <c r="A239" s="32" t="n"/>
-      <c r="B239" s="32" t="n"/>
-      <c r="C239" s="32" t="n"/>
-      <c r="D239" s="32" t="n"/>
-      <c r="E239" s="32" t="n"/>
-      <c r="F239" s="32" t="n"/>
+      <c r="A239" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B239" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C239" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D239" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E239" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F239" s="32" t="inlineStr">
+        <is>
+          <t>3 x 8 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G239" s="32" t="n"/>
     </row>
     <row r="240" ht="15" customHeight="1" s="21">
-      <c r="A240" s="32" t="n"/>
-      <c r="B240" s="32" t="n"/>
-      <c r="C240" s="32" t="n"/>
-      <c r="D240" s="32" t="n"/>
-      <c r="E240" s="32" t="n"/>
-      <c r="F240" s="32" t="n"/>
+      <c r="A240" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B240" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C240" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D240" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E240" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F240" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G240" s="32" t="n"/>
     </row>
     <row r="241" ht="15" customHeight="1" s="21">
-      <c r="A241" s="32" t="n"/>
-      <c r="B241" s="32" t="n"/>
-      <c r="C241" s="32" t="n"/>
-      <c r="D241" s="32" t="n"/>
-      <c r="E241" s="32" t="n"/>
-      <c r="F241" s="32" t="n"/>
+      <c r="A241" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B241" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C241" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D241" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E241" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F241" s="32" t="inlineStr">
+        <is>
+          <t>12 x 400 m @ I, 60 s jog between</t>
+        </is>
+      </c>
       <c r="G241" s="32" t="n"/>
     </row>
     <row r="242" ht="15" customHeight="1" s="21">
-      <c r="A242" s="32" t="n"/>
-      <c r="B242" s="32" t="n"/>
-      <c r="C242" s="32" t="n"/>
-      <c r="D242" s="32" t="n"/>
-      <c r="E242" s="32" t="n"/>
-      <c r="F242" s="32" t="n"/>
+      <c r="A242" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B242" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C242" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D242" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E242" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F242" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G242" s="32" t="n"/>
     </row>
     <row r="243" ht="15" customHeight="1" s="21">
-      <c r="A243" s="32" t="n"/>
-      <c r="B243" s="32" t="n"/>
-      <c r="C243" s="32" t="n"/>
-      <c r="D243" s="32" t="n"/>
-      <c r="E243" s="32" t="n"/>
-      <c r="F243" s="32" t="n"/>
+      <c r="A243" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B243" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C243" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D243" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E243" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F243" s="32" t="inlineStr">
+        <is>
+          <t>3 km E → 3 km STEADY → 2 km T</t>
+        </is>
+      </c>
       <c r="G243" s="32" t="n"/>
     </row>
     <row r="244" ht="15" customHeight="1" s="21">
-      <c r="A244" s="32" t="n"/>
-      <c r="B244" s="32" t="n"/>
-      <c r="C244" s="32" t="n"/>
-      <c r="D244" s="32" t="n"/>
-      <c r="E244" s="32" t="n"/>
-      <c r="F244" s="32" t="n"/>
+      <c r="A244" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B244" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C244" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D244" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E244" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F244" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G244" s="32" t="n"/>
     </row>
     <row r="245" ht="15" customHeight="1" s="21">
-      <c r="A245" s="32" t="n"/>
-      <c r="B245" s="32" t="n"/>
-      <c r="C245" s="32" t="n"/>
-      <c r="D245" s="32" t="n"/>
-      <c r="E245" s="32" t="n"/>
-      <c r="F245" s="32" t="n"/>
+      <c r="A245" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B245" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C245" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D245" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E245" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F245" s="32" t="inlineStr">
+        <is>
+          <t>5 x (3 min @ 5K / 1 min @ I / 2 min E)</t>
+        </is>
+      </c>
       <c r="G245" s="32" t="n"/>
     </row>
     <row r="246" ht="15" customHeight="1" s="21">
-      <c r="A246" s="32" t="n"/>
-      <c r="B246" s="32" t="n"/>
-      <c r="C246" s="32" t="n"/>
-      <c r="D246" s="32" t="n"/>
-      <c r="E246" s="32" t="n"/>
-      <c r="F246" s="32" t="n"/>
+      <c r="A246" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B246" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C246" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D246" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E246" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F246" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G246" s="32" t="n"/>
     </row>
     <row r="247" ht="15" customHeight="1" s="21">
-      <c r="A247" s="32" t="n"/>
-      <c r="B247" s="32" t="n"/>
-      <c r="C247" s="32" t="n"/>
-      <c r="D247" s="32" t="n"/>
-      <c r="E247" s="32" t="n"/>
-      <c r="F247" s="32" t="n"/>
+      <c r="A247" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B247" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C247" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D247" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E247" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F247" s="32" t="inlineStr">
+        <is>
+          <t>2 x 12 min @ T, 3 min jog between</t>
+        </is>
+      </c>
       <c r="G247" s="32" t="n"/>
     </row>
     <row r="248" ht="15" customHeight="1" s="21">
-      <c r="A248" s="32" t="n"/>
-      <c r="B248" s="32" t="n"/>
-      <c r="C248" s="32" t="n"/>
-      <c r="D248" s="32" t="n"/>
-      <c r="E248" s="32" t="n"/>
-      <c r="F248" s="32" t="n"/>
+      <c r="A248" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B248" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C248" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D248" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E248" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F248" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G248" s="32" t="n"/>
     </row>
     <row r="249" ht="15" customHeight="1" s="21">
-      <c r="A249" s="32" t="n"/>
-      <c r="B249" s="32" t="n"/>
-      <c r="C249" s="32" t="n"/>
-      <c r="D249" s="32" t="n"/>
-      <c r="E249" s="32" t="n"/>
-      <c r="F249" s="32" t="n"/>
+      <c r="A249" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B249" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C249" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D249" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E249" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F249" s="32" t="inlineStr">
+        <is>
+          <t>8 x (1 min @ I effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G249" s="32" t="n"/>
     </row>
     <row r="250" ht="15" customHeight="1" s="21">
-      <c r="A250" s="32" t="n"/>
-      <c r="B250" s="32" t="n"/>
-      <c r="C250" s="32" t="n"/>
-      <c r="D250" s="32" t="n"/>
-      <c r="E250" s="32" t="n"/>
-      <c r="F250" s="32" t="n"/>
+      <c r="A250" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B250" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C250" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D250" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E250" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F250" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G250" s="32" t="n"/>
     </row>
     <row r="251" ht="15" customHeight="1" s="21">
-      <c r="A251" s="32" t="n"/>
-      <c r="B251" s="32" t="n"/>
-      <c r="C251" s="32" t="n"/>
-      <c r="D251" s="32" t="n"/>
-      <c r="E251" s="32" t="n"/>
-      <c r="F251" s="32" t="n"/>
+      <c r="A251" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B251" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C251" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D251" s="32" t="inlineStr">
+        <is>
+          <t>Progression</t>
+        </is>
+      </c>
+      <c r="E251" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F251" s="32" t="inlineStr">
+        <is>
+          <t>3 km E → 2 km STEADY → 2 km T</t>
+        </is>
+      </c>
       <c r="G251" s="32" t="n"/>
     </row>
     <row r="252" ht="15" customHeight="1" s="21">
-      <c r="A252" s="32" t="n"/>
-      <c r="B252" s="32" t="n"/>
-      <c r="C252" s="32" t="n"/>
-      <c r="D252" s="32" t="n"/>
-      <c r="E252" s="32" t="n"/>
-      <c r="F252" s="32" t="n"/>
+      <c r="A252" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B252" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C252" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D252" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E252" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F252" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G252" s="32" t="n"/>
     </row>
     <row r="253" ht="15" customHeight="1" s="21">
-      <c r="A253" s="32" t="n"/>
-      <c r="B253" s="32" t="n"/>
-      <c r="C253" s="32" t="n"/>
-      <c r="D253" s="32" t="n"/>
-      <c r="E253" s="32" t="n"/>
-      <c r="F253" s="32" t="n"/>
+      <c r="A253" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B253" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C253" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D253" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E253" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F253" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1 km @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G253" s="32" t="n"/>
     </row>
     <row r="254" ht="15" customHeight="1" s="21">
-      <c r="A254" s="32" t="n"/>
-      <c r="B254" s="32" t="n"/>
-      <c r="C254" s="32" t="n"/>
-      <c r="D254" s="32" t="n"/>
-      <c r="E254" s="32" t="n"/>
-      <c r="F254" s="32" t="n"/>
+      <c r="A254" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B254" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C254" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D254" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E254" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F254" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G254" s="32" t="n"/>
     </row>
     <row r="255" ht="15" customHeight="1" s="21">
-      <c r="A255" s="32" t="n"/>
-      <c r="B255" s="32" t="n"/>
-      <c r="C255" s="32" t="n"/>
-      <c r="D255" s="32" t="n"/>
-      <c r="E255" s="32" t="n"/>
-      <c r="F255" s="32" t="n"/>
+      <c r="A255" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B255" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C255" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D255" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E255" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F255" s="32" t="inlineStr">
+        <is>
+          <t>25 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G255" s="32" t="n"/>
     </row>
     <row r="256" ht="15" customHeight="1" s="21">
-      <c r="A256" s="32" t="n"/>
-      <c r="B256" s="32" t="n"/>
-      <c r="C256" s="32" t="n"/>
-      <c r="D256" s="32" t="n"/>
-      <c r="E256" s="32" t="n"/>
-      <c r="F256" s="32" t="n"/>
+      <c r="A256" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B256" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="C256" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D256" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E256" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F256" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G256" s="32" t="n"/>
     </row>
     <row r="257" ht="15" customHeight="1" s="21">
-      <c r="A257" s="32" t="n"/>
-      <c r="B257" s="32" t="n"/>
-      <c r="C257" s="32" t="n"/>
-      <c r="D257" s="32" t="n"/>
-      <c r="E257" s="32" t="n"/>
-      <c r="F257" s="32" t="n"/>
+      <c r="A257" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B257" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C257" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D257" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E257" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F257" s="32" t="inlineStr">
+        <is>
+          <t>8 x 600 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G257" s="32" t="n"/>
     </row>
     <row r="258" ht="15" customHeight="1" s="21">
-      <c r="A258" s="32" t="n"/>
-      <c r="B258" s="32" t="n"/>
-      <c r="C258" s="32" t="n"/>
-      <c r="D258" s="32" t="n"/>
-      <c r="E258" s="32" t="n"/>
-      <c r="F258" s="32" t="n"/>
+      <c r="A258" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B258" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C258" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D258" s="32" t="inlineStr">
+        <is>
+          <t>Recovery</t>
+        </is>
+      </c>
+      <c r="E258" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F258" s="32" t="inlineStr">
+        <is>
+          <t>Very relaxed recovery run</t>
+        </is>
+      </c>
       <c r="G258" s="32" t="n"/>
     </row>
     <row r="259" ht="15" customHeight="1" s="21">
-      <c r="A259" s="32" t="n"/>
-      <c r="B259" s="32" t="n"/>
-      <c r="C259" s="32" t="n"/>
-      <c r="D259" s="32" t="n"/>
-      <c r="E259" s="32" t="n"/>
-      <c r="F259" s="32" t="n"/>
+      <c r="A259" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B259" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C259" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D259" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E259" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F259" s="32" t="inlineStr">
+        <is>
+          <t>3 x 2 km @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G259" s="32" t="n"/>
     </row>
     <row r="260" ht="15" customHeight="1" s="21">
-      <c r="A260" s="32" t="n"/>
-      <c r="B260" s="32" t="n"/>
-      <c r="C260" s="32" t="n"/>
-      <c r="D260" s="32" t="n"/>
-      <c r="E260" s="32" t="n"/>
-      <c r="F260" s="32" t="n"/>
+      <c r="A260" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B260" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C260" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D260" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E260" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F260" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G260" s="32" t="n"/>
     </row>
     <row r="261" ht="15" customHeight="1" s="21">
-      <c r="A261" s="32" t="n"/>
-      <c r="B261" s="32" t="n"/>
-      <c r="C261" s="32" t="n"/>
-      <c r="D261" s="32" t="n"/>
-      <c r="E261" s="32" t="n"/>
-      <c r="F261" s="32" t="n"/>
+      <c r="A261" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B261" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C261" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E261" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F261" s="32" t="inlineStr">
+        <is>
+          <t>6 x 400 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G261" s="32" t="n"/>
     </row>
     <row r="262" ht="15" customHeight="1" s="21">
-      <c r="A262" s="32" t="n"/>
-      <c r="B262" s="32" t="n"/>
-      <c r="C262" s="32" t="n"/>
-      <c r="D262" s="32" t="n"/>
-      <c r="E262" s="32" t="n"/>
-      <c r="F262" s="32" t="n"/>
+      <c r="A262" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B262" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C262" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D262" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E262" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F262" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G262" s="32" t="n"/>
     </row>
     <row r="263" ht="15" customHeight="1" s="21">
-      <c r="A263" s="32" t="n"/>
-      <c r="B263" s="32" t="n"/>
-      <c r="C263" s="32" t="n"/>
-      <c r="D263" s="32" t="n"/>
-      <c r="E263" s="32" t="n"/>
-      <c r="F263" s="32" t="n"/>
+      <c r="A263" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B263" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C263" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D263" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E263" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F263" s="32" t="inlineStr">
+        <is>
+          <t>6 x (90 s @ 5K / 90 s E)</t>
+        </is>
+      </c>
       <c r="G263" s="32" t="n"/>
     </row>
     <row r="264" ht="15" customHeight="1" s="21">
-      <c r="A264" s="32" t="n"/>
-      <c r="B264" s="32" t="n"/>
-      <c r="C264" s="32" t="n"/>
-      <c r="D264" s="32" t="n"/>
-      <c r="E264" s="32" t="n"/>
-      <c r="F264" s="32" t="n"/>
+      <c r="A264" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B264" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="C264" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D264" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E264" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F264" s="32" t="inlineStr">
+        <is>
+          <t>Reduced long run, E</t>
+        </is>
+      </c>
       <c r="G264" s="32" t="n"/>
     </row>
     <row r="265" ht="15" customHeight="1" s="21">
-      <c r="A265" s="32" t="n"/>
-      <c r="B265" s="32" t="n"/>
-      <c r="C265" s="32" t="n"/>
-      <c r="D265" s="32" t="n"/>
-      <c r="E265" s="32" t="n"/>
-      <c r="F265" s="32" t="n"/>
+      <c r="A265" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B265" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C265" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D265" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E265" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F265" s="32" t="inlineStr">
+        <is>
+          <t>4 x 400 m @ 5K, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G265" s="32" t="n"/>
     </row>
     <row r="266" ht="15" customHeight="1" s="21">
-      <c r="A266" s="32" t="n"/>
-      <c r="B266" s="32" t="n"/>
-      <c r="C266" s="32" t="n"/>
-      <c r="D266" s="32" t="n"/>
-      <c r="E266" s="32" t="n"/>
-      <c r="F266" s="32" t="n"/>
+      <c r="A266" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B266" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C266" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D266" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E266" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F266" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G266" s="32" t="n"/>
     </row>
     <row r="267" ht="15" customHeight="1" s="21">
-      <c r="A267" s="32" t="n"/>
-      <c r="B267" s="32" t="n"/>
-      <c r="C267" s="32" t="n"/>
-      <c r="D267" s="32" t="n"/>
-      <c r="E267" s="32" t="n"/>
-      <c r="F267" s="32" t="n"/>
+      <c r="A267" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B267" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C267" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D267" s="32" t="inlineStr">
+        <is>
+          <t>Shakeout</t>
+        </is>
+      </c>
+      <c r="E267" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F267" s="32" t="inlineStr">
+        <is>
+          <t>3 km E + 4 x 20 s strides</t>
+        </is>
+      </c>
       <c r="G267" s="32" t="n"/>
     </row>
     <row r="268" ht="15" customHeight="1" s="21">
-      <c r="A268" s="32" t="n"/>
-      <c r="B268" s="32" t="n"/>
-      <c r="C268" s="32" t="n"/>
-      <c r="D268" s="32" t="n"/>
-      <c r="E268" s="32" t="n"/>
-      <c r="F268" s="32" t="n"/>
+      <c r="A268" s="32" t="inlineStr">
+        <is>
+          <t>Faster 5K</t>
+        </is>
+      </c>
+      <c r="B268" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="C268" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D268" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="E268" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F268" s="32" t="inlineStr">
+        <is>
+          <t>5K RACE – race at goal 5K pace</t>
+        </is>
+      </c>
       <c r="G268" s="32" t="n"/>
     </row>
     <row r="269" ht="15" customHeight="1" s="21">
@@ -32399,7 +33623,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26" ht="15" customHeight="1" s="21">
       <c r="A26" s="34" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
First 5K programme: run/walk weeks building to 25 minutes non-stop, then a 5K by feel
- Planner: run/walk sessions (walk breaks) keep their prescription, brisk walk either side,
  no pace on walks; First 5K race is run by feel unless a goal time is set
- Converter labels walk steps inside mixed reps

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -2316,7 +2316,7 @@
         <v>3</v>
       </c>
       <c r="F2" s="32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2" s="32" t="n">
         <v>1</v>
@@ -5833,13 +5833,37 @@
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="21">
-      <c r="A66" s="32" t="n"/>
-      <c r="B66" s="32" t="n"/>
-      <c r="C66" s="32" t="n"/>
-      <c r="D66" s="35" t="n"/>
-      <c r="E66" s="32" t="n"/>
-      <c r="F66" s="32" t="n"/>
-      <c r="G66" s="32" t="n"/>
+      <c r="A66" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B66" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D66" s="35" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E66" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F66" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G66" s="32" t="inlineStr">
+        <is>
+          <t>Run/walk: short runs with walking breaks. Easy enough to chat throughout.</t>
+        </is>
+      </c>
       <c r="H66" s="33">
         <f>IF(A66="","",COUNTIFS('Run sessions'!$A$2:$A$401,A66,'Run sessions'!$B$2:$B$401,B66))</f>
         <v/>
@@ -5854,12 +5878,32 @@
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="21">
-      <c r="A67" s="32" t="n"/>
-      <c r="B67" s="32" t="n"/>
-      <c r="C67" s="32" t="n"/>
-      <c r="D67" s="35" t="n"/>
-      <c r="E67" s="32" t="n"/>
-      <c r="F67" s="32" t="n"/>
+      <c r="A67" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B67" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C67" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D67" s="35" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="E67" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F67" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G67" s="32" t="n"/>
       <c r="H67" s="33">
         <f>IF(A67="","",COUNTIFS('Run sessions'!$A$2:$A$401,A67,'Run sessions'!$B$2:$B$401,B67))</f>
@@ -5875,12 +5919,32 @@
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="21">
-      <c r="A68" s="32" t="n"/>
-      <c r="B68" s="32" t="n"/>
-      <c r="C68" s="32" t="n"/>
-      <c r="D68" s="35" t="n"/>
-      <c r="E68" s="32" t="n"/>
-      <c r="F68" s="32" t="n"/>
+      <c r="A68" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B68" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C68" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D68" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E68" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F68" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G68" s="32" t="n"/>
       <c r="H68" s="33">
         <f>IF(A68="","",COUNTIFS('Run sessions'!$A$2:$A$401,A68,'Run sessions'!$B$2:$B$401,B68))</f>
@@ -5896,13 +5960,37 @@
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="21">
-      <c r="A69" s="32" t="n"/>
-      <c r="B69" s="32" t="n"/>
-      <c r="C69" s="32" t="n"/>
-      <c r="D69" s="35" t="n"/>
-      <c r="E69" s="32" t="n"/>
-      <c r="F69" s="32" t="n"/>
-      <c r="G69" s="32" t="n"/>
+      <c r="A69" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B69" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C69" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D69" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E69" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F69" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G69" s="32" t="inlineStr">
+        <is>
+          <t>Longer runs, fewer walks.</t>
+        </is>
+      </c>
       <c r="H69" s="33">
         <f>IF(A69="","",COUNTIFS('Run sessions'!$A$2:$A$401,A69,'Run sessions'!$B$2:$B$401,B69))</f>
         <v/>
@@ -5917,13 +6005,37 @@
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="21">
-      <c r="A70" s="32" t="n"/>
-      <c r="B70" s="32" t="n"/>
-      <c r="C70" s="32" t="n"/>
-      <c r="D70" s="35" t="n"/>
-      <c r="E70" s="32" t="n"/>
-      <c r="F70" s="32" t="n"/>
-      <c r="G70" s="32" t="n"/>
+      <c r="A70" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B70" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C70" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D70" s="35" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E70" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F70" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G70" s="32" t="inlineStr">
+        <is>
+          <t>A few short pick-ups to wake the legs up.</t>
+        </is>
+      </c>
       <c r="H70" s="33">
         <f>IF(A70="","",COUNTIFS('Run sessions'!$A$2:$A$401,A70,'Run sessions'!$B$2:$B$401,B70))</f>
         <v/>
@@ -5938,13 +6050,37 @@
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="21">
-      <c r="A71" s="32" t="n"/>
-      <c r="B71" s="32" t="n"/>
-      <c r="C71" s="32" t="n"/>
-      <c r="D71" s="35" t="n"/>
-      <c r="E71" s="32" t="n"/>
-      <c r="F71" s="32" t="n"/>
-      <c r="G71" s="32" t="n"/>
+      <c r="A71" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B71" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C71" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D71" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F71" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>Your first 20 minutes without stopping.</t>
+        </is>
+      </c>
       <c r="H71" s="33">
         <f>IF(A71="","",COUNTIFS('Run sessions'!$A$2:$A$401,A71,'Run sessions'!$B$2:$B$401,B71))</f>
         <v/>
@@ -5959,13 +6095,37 @@
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="21">
-      <c r="A72" s="32" t="n"/>
-      <c r="B72" s="32" t="n"/>
-      <c r="C72" s="32" t="n"/>
-      <c r="D72" s="35" t="n"/>
-      <c r="E72" s="32" t="n"/>
-      <c r="F72" s="32" t="n"/>
-      <c r="G72" s="32" t="n"/>
+      <c r="A72" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B72" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C72" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D72" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E72" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F72" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>25 minutes non-stop: you're nearly there.</t>
+        </is>
+      </c>
       <c r="H72" s="33">
         <f>IF(A72="","",COUNTIFS('Run sessions'!$A$2:$A$401,A72,'Run sessions'!$B$2:$B$401,B72))</f>
         <v/>
@@ -5980,13 +6140,37 @@
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="21">
-      <c r="A73" s="32" t="n"/>
-      <c r="B73" s="32" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="35" t="n"/>
-      <c r="E73" s="32" t="n"/>
-      <c r="F73" s="32" t="n"/>
-      <c r="G73" s="32" t="n"/>
+      <c r="A73" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B73" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C73" s="32" t="inlineStr">
+        <is>
+          <t>Race week</t>
+        </is>
+      </c>
+      <c r="D73" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E73" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="F73" s="32" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>Race day! Run it comfortably and finish strong.</t>
+        </is>
+      </c>
       <c r="H73" s="33">
         <f>IF(A73="","",COUNTIFS('Run sessions'!$A$2:$A$401,A73,'Run sessions'!$B$2:$B$401,B73))</f>
         <v/>
@@ -20753,219 +20937,699 @@
       <c r="G268" s="32" t="n"/>
     </row>
     <row r="269" ht="15" customHeight="1" s="21">
-      <c r="A269" s="32" t="n"/>
-      <c r="B269" s="32" t="n"/>
-      <c r="C269" s="32" t="n"/>
-      <c r="D269" s="32" t="n"/>
-      <c r="E269" s="32" t="n"/>
-      <c r="F269" s="32" t="n"/>
+      <c r="A269" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B269" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C269" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D269" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E269" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F269" s="32" t="inlineStr">
+        <is>
+          <t>8 x 1 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G269" s="32" t="n"/>
     </row>
     <row r="270" ht="15" customHeight="1" s="21">
-      <c r="A270" s="32" t="n"/>
-      <c r="B270" s="32" t="n"/>
-      <c r="C270" s="32" t="n"/>
-      <c r="D270" s="32" t="n"/>
-      <c r="E270" s="32" t="n"/>
-      <c r="F270" s="32" t="n"/>
+      <c r="A270" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B270" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C270" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D270" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E270" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F270" s="32" t="inlineStr">
+        <is>
+          <t>8 x 1 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G270" s="32" t="n"/>
     </row>
     <row r="271" ht="15" customHeight="1" s="21">
-      <c r="A271" s="32" t="n"/>
-      <c r="B271" s="32" t="n"/>
-      <c r="C271" s="32" t="n"/>
-      <c r="D271" s="32" t="n"/>
-      <c r="E271" s="32" t="n"/>
-      <c r="F271" s="32" t="n"/>
+      <c r="A271" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B271" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C271" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D271" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E271" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F271" s="32" t="inlineStr">
+        <is>
+          <t>8 x 1 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G271" s="32" t="n"/>
     </row>
     <row r="272" ht="15" customHeight="1" s="21">
-      <c r="A272" s="32" t="n"/>
-      <c r="B272" s="32" t="n"/>
-      <c r="C272" s="32" t="n"/>
-      <c r="D272" s="32" t="n"/>
-      <c r="E272" s="32" t="n"/>
-      <c r="F272" s="32" t="n"/>
+      <c r="A272" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B272" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C272" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D272" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E272" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F272" s="32" t="inlineStr">
+        <is>
+          <t>6 x 2 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G272" s="32" t="n"/>
     </row>
     <row r="273" ht="15" customHeight="1" s="21">
-      <c r="A273" s="32" t="n"/>
-      <c r="B273" s="32" t="n"/>
-      <c r="C273" s="32" t="n"/>
-      <c r="D273" s="32" t="n"/>
-      <c r="E273" s="32" t="n"/>
-      <c r="F273" s="32" t="n"/>
+      <c r="A273" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B273" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C273" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D273" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E273" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F273" s="32" t="inlineStr">
+        <is>
+          <t>6 x 2 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G273" s="32" t="n"/>
     </row>
     <row r="274" ht="15" customHeight="1" s="21">
-      <c r="A274" s="32" t="n"/>
-      <c r="B274" s="32" t="n"/>
-      <c r="C274" s="32" t="n"/>
-      <c r="D274" s="32" t="n"/>
-      <c r="E274" s="32" t="n"/>
-      <c r="F274" s="32" t="n"/>
+      <c r="A274" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B274" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C274" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D274" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E274" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F274" s="32" t="inlineStr">
+        <is>
+          <t>5 x 3 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G274" s="32" t="n"/>
     </row>
     <row r="275" ht="15" customHeight="1" s="21">
-      <c r="A275" s="32" t="n"/>
-      <c r="B275" s="32" t="n"/>
-      <c r="C275" s="32" t="n"/>
-      <c r="D275" s="32" t="n"/>
-      <c r="E275" s="32" t="n"/>
-      <c r="F275" s="32" t="n"/>
+      <c r="A275" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B275" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C275" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D275" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E275" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F275" s="32" t="inlineStr">
+        <is>
+          <t>5 x 3 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G275" s="32" t="n"/>
     </row>
     <row r="276" ht="15" customHeight="1" s="21">
-      <c r="A276" s="32" t="n"/>
-      <c r="B276" s="32" t="n"/>
-      <c r="C276" s="32" t="n"/>
-      <c r="D276" s="32" t="n"/>
-      <c r="E276" s="32" t="n"/>
-      <c r="F276" s="32" t="n"/>
+      <c r="A276" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B276" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C276" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D276" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E276" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F276" s="32" t="inlineStr">
+        <is>
+          <t>4 x 4 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G276" s="32" t="n"/>
     </row>
     <row r="277" ht="15" customHeight="1" s="21">
-      <c r="A277" s="32" t="n"/>
-      <c r="B277" s="32" t="n"/>
-      <c r="C277" s="32" t="n"/>
-      <c r="D277" s="32" t="n"/>
-      <c r="E277" s="32" t="n"/>
-      <c r="F277" s="32" t="n"/>
+      <c r="A277" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B277" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C277" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D277" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E277" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F277" s="32" t="inlineStr">
+        <is>
+          <t>4 x 5 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G277" s="32" t="n"/>
     </row>
     <row r="278" ht="15" customHeight="1" s="21">
-      <c r="A278" s="32" t="n"/>
-      <c r="B278" s="32" t="n"/>
-      <c r="C278" s="32" t="n"/>
-      <c r="D278" s="32" t="n"/>
-      <c r="E278" s="32" t="n"/>
-      <c r="F278" s="32" t="n"/>
+      <c r="A278" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B278" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C278" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D278" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E278" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F278" s="32" t="inlineStr">
+        <is>
+          <t>3 x 6 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G278" s="32" t="n"/>
     </row>
     <row r="279" ht="15" customHeight="1" s="21">
-      <c r="A279" s="32" t="n"/>
-      <c r="B279" s="32" t="n"/>
-      <c r="C279" s="32" t="n"/>
-      <c r="D279" s="32" t="n"/>
-      <c r="E279" s="32" t="n"/>
-      <c r="F279" s="32" t="n"/>
+      <c r="A279" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B279" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C279" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D279" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E279" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F279" s="32" t="inlineStr">
+        <is>
+          <t>3 x 7 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G279" s="32" t="n"/>
     </row>
     <row r="280" ht="15" customHeight="1" s="21">
-      <c r="A280" s="32" t="n"/>
-      <c r="B280" s="32" t="n"/>
-      <c r="C280" s="32" t="n"/>
-      <c r="D280" s="32" t="n"/>
-      <c r="E280" s="32" t="n"/>
-      <c r="F280" s="32" t="n"/>
+      <c r="A280" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B280" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C280" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D280" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E280" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F280" s="32" t="inlineStr">
+        <is>
+          <t>2 x 10 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G280" s="32" t="n"/>
     </row>
     <row r="281" ht="15" customHeight="1" s="21">
-      <c r="A281" s="32" t="n"/>
-      <c r="B281" s="32" t="n"/>
-      <c r="C281" s="32" t="n"/>
-      <c r="D281" s="32" t="n"/>
-      <c r="E281" s="32" t="n"/>
-      <c r="F281" s="32" t="n"/>
+      <c r="A281" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B281" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C281" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D281" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E281" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F281" s="32" t="inlineStr">
+        <is>
+          <t>2 x 10 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G281" s="32" t="n"/>
     </row>
     <row r="282" ht="15" customHeight="1" s="21">
-      <c r="A282" s="32" t="n"/>
-      <c r="B282" s="32" t="n"/>
-      <c r="C282" s="32" t="n"/>
-      <c r="D282" s="32" t="n"/>
-      <c r="E282" s="32" t="n"/>
-      <c r="F282" s="32" t="n"/>
+      <c r="A282" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B282" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C282" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D282" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E282" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F282" s="32" t="inlineStr">
+        <is>
+          <t>5 x (3 min @ E effort / 30 s @ 5K effort / 90 s walk)</t>
+        </is>
+      </c>
       <c r="G282" s="32" t="n"/>
     </row>
     <row r="283" ht="15" customHeight="1" s="21">
-      <c r="A283" s="32" t="n"/>
-      <c r="B283" s="32" t="n"/>
-      <c r="C283" s="32" t="n"/>
-      <c r="D283" s="32" t="n"/>
-      <c r="E283" s="32" t="n"/>
-      <c r="F283" s="32" t="n"/>
+      <c r="A283" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B283" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C283" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D283" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E283" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F283" s="32" t="inlineStr">
+        <is>
+          <t>2 x 12 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G283" s="32" t="n"/>
     </row>
     <row r="284" ht="15" customHeight="1" s="21">
-      <c r="A284" s="32" t="n"/>
-      <c r="B284" s="32" t="n"/>
-      <c r="C284" s="32" t="n"/>
-      <c r="D284" s="32" t="n"/>
-      <c r="E284" s="32" t="n"/>
-      <c r="F284" s="32" t="n"/>
+      <c r="A284" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B284" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C284" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D284" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E284" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F284" s="32" t="inlineStr">
+        <is>
+          <t>2 x 12 min @ E effort, 90 s walk between</t>
+        </is>
+      </c>
       <c r="G284" s="32" t="n"/>
     </row>
     <row r="285" ht="15" customHeight="1" s="21">
-      <c r="A285" s="32" t="n"/>
-      <c r="B285" s="32" t="n"/>
-      <c r="C285" s="32" t="n"/>
-      <c r="D285" s="32" t="n"/>
-      <c r="E285" s="32" t="n"/>
-      <c r="F285" s="32" t="n"/>
+      <c r="A285" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B285" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C285" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D285" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E285" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F285" s="32" t="inlineStr">
+        <is>
+          <t>6 x (3 min @ E effort / 30 s @ 5K effort / 90 s walk)</t>
+        </is>
+      </c>
       <c r="G285" s="32" t="n"/>
     </row>
     <row r="286" ht="15" customHeight="1" s="21">
-      <c r="A286" s="32" t="n"/>
-      <c r="B286" s="32" t="n"/>
-      <c r="C286" s="32" t="n"/>
-      <c r="D286" s="32" t="n"/>
-      <c r="E286" s="32" t="n"/>
-      <c r="F286" s="32" t="n"/>
+      <c r="A286" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B286" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C286" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D286" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E286" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F286" s="32" t="inlineStr">
+        <is>
+          <t>1 x 20 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G286" s="32" t="n"/>
     </row>
     <row r="287" ht="15" customHeight="1" s="21">
-      <c r="A287" s="32" t="n"/>
-      <c r="B287" s="32" t="n"/>
-      <c r="C287" s="32" t="n"/>
-      <c r="D287" s="32" t="n"/>
-      <c r="E287" s="32" t="n"/>
-      <c r="F287" s="32" t="n"/>
+      <c r="A287" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B287" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C287" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D287" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E287" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F287" s="32" t="inlineStr">
+        <is>
+          <t>1 x 20 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G287" s="32" t="n"/>
     </row>
     <row r="288" ht="15" customHeight="1" s="21">
-      <c r="A288" s="32" t="n"/>
-      <c r="B288" s="32" t="n"/>
-      <c r="C288" s="32" t="n"/>
-      <c r="D288" s="32" t="n"/>
-      <c r="E288" s="32" t="n"/>
-      <c r="F288" s="32" t="n"/>
+      <c r="A288" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B288" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C288" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D288" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E288" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F288" s="32" t="inlineStr">
+        <is>
+          <t>6 x (4 min @ E effort / 30 s @ 5K effort / 60 s walk)</t>
+        </is>
+      </c>
       <c r="G288" s="32" t="n"/>
     </row>
     <row r="289" ht="15" customHeight="1" s="21">
-      <c r="A289" s="32" t="n"/>
-      <c r="B289" s="32" t="n"/>
-      <c r="C289" s="32" t="n"/>
-      <c r="D289" s="32" t="n"/>
-      <c r="E289" s="32" t="n"/>
-      <c r="F289" s="32" t="n"/>
+      <c r="A289" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B289" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C289" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D289" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E289" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F289" s="32" t="inlineStr">
+        <is>
+          <t>1 x 25 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G289" s="32" t="n"/>
     </row>
     <row r="290" ht="15" customHeight="1" s="21">
-      <c r="A290" s="32" t="n"/>
-      <c r="B290" s="32" t="n"/>
-      <c r="C290" s="32" t="n"/>
-      <c r="D290" s="32" t="n"/>
-      <c r="E290" s="32" t="n"/>
-      <c r="F290" s="32" t="n"/>
+      <c r="A290" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B290" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C290" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D290" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E290" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F290" s="32" t="inlineStr">
+        <is>
+          <t>1 x 15 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G290" s="32" t="n"/>
     </row>
     <row r="291" ht="15" customHeight="1" s="21">
-      <c r="A291" s="32" t="n"/>
-      <c r="B291" s="32" t="n"/>
-      <c r="C291" s="32" t="n"/>
-      <c r="D291" s="32" t="n"/>
-      <c r="E291" s="32" t="n"/>
-      <c r="F291" s="32" t="n"/>
+      <c r="A291" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B291" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C291" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D291" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E291" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F291" s="32" t="inlineStr">
+        <is>
+          <t>1 x 10 min @ E effort, 2 min walk between</t>
+        </is>
+      </c>
       <c r="G291" s="32" t="n"/>
     </row>
     <row r="292" ht="15" customHeight="1" s="21">
-      <c r="A292" s="32" t="n"/>
-      <c r="B292" s="32" t="n"/>
-      <c r="C292" s="32" t="n"/>
-      <c r="D292" s="32" t="n"/>
-      <c r="E292" s="32" t="n"/>
-      <c r="F292" s="32" t="n"/>
+      <c r="A292" s="32" t="inlineStr">
+        <is>
+          <t>First 5K</t>
+        </is>
+      </c>
+      <c r="B292" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C292" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D292" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="E292" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F292" s="32" t="inlineStr">
+        <is>
+          <t>5K – run it comfortably and finish strong</t>
+        </is>
+      </c>
       <c r="G292" s="32" t="n"/>
     </row>
     <row r="293" ht="15" customHeight="1" s="21">

</xml_diff>

<commit_message>
Balanced hybrid programme with a 5K time trial, and update paces from a race or time trial
- Balanced hybrid: 8 weeks, deloads in weeks 4 and 8, 3 runs (intervals or tempo, easy, long)
- Time trials in goals without a race are a 5K
- Run summary: after a planned race or time trial, 'Use this result' sets the runner's race
  time and rebuilds the rest of the plan with the new paces

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -2834,7 +2834,7 @@
         <v>2</v>
       </c>
       <c r="F9" s="32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G9" s="32" t="n">
         <v>2</v>
@@ -2858,7 +2858,7 @@
         <v>40</v>
       </c>
       <c r="N9" s="32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" s="32" t="inlineStr">
         <is>
@@ -6185,13 +6185,37 @@
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="21">
-      <c r="A74" s="32" t="n"/>
-      <c r="B74" s="32" t="n"/>
-      <c r="C74" s="32" t="n"/>
-      <c r="D74" s="35" t="n"/>
-      <c r="E74" s="32" t="n"/>
-      <c r="F74" s="32" t="n"/>
-      <c r="G74" s="32" t="n"/>
+      <c r="A74" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B74" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D74" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F74" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G74" s="32" t="inlineStr">
+        <is>
+          <t>Settle in: one quality run, the rest easy, and full-body lifting.</t>
+        </is>
+      </c>
       <c r="H74" s="33">
         <f>IF(A74="","",COUNTIFS('Run sessions'!$A$2:$A$401,A74,'Run sessions'!$B$2:$B$401,B74))</f>
         <v/>
@@ -6206,12 +6230,32 @@
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="21">
-      <c r="A75" s="32" t="n"/>
-      <c r="B75" s="32" t="n"/>
-      <c r="C75" s="32" t="n"/>
-      <c r="D75" s="35" t="n"/>
-      <c r="E75" s="32" t="n"/>
-      <c r="F75" s="32" t="n"/>
+      <c r="A75" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B75" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C75" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D75" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E75" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F75" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G75" s="32" t="n"/>
       <c r="H75" s="33">
         <f>IF(A75="","",COUNTIFS('Run sessions'!$A$2:$A$401,A75,'Run sessions'!$B$2:$B$401,B75))</f>
@@ -6227,12 +6271,32 @@
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="21">
-      <c r="A76" s="32" t="n"/>
-      <c r="B76" s="32" t="n"/>
-      <c r="C76" s="32" t="n"/>
-      <c r="D76" s="35" t="n"/>
-      <c r="E76" s="32" t="n"/>
-      <c r="F76" s="32" t="n"/>
+      <c r="A76" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B76" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C76" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D76" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E76" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F76" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G76" s="32" t="n"/>
       <c r="H76" s="33">
         <f>IF(A76="","",COUNTIFS('Run sessions'!$A$2:$A$401,A76,'Run sessions'!$B$2:$B$401,B76))</f>
@@ -6248,13 +6312,37 @@
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="21">
-      <c r="A77" s="32" t="n"/>
-      <c r="B77" s="32" t="n"/>
-      <c r="C77" s="32" t="n"/>
-      <c r="D77" s="35" t="n"/>
-      <c r="E77" s="32" t="n"/>
-      <c r="F77" s="32" t="n"/>
-      <c r="G77" s="32" t="n"/>
+      <c r="A77" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B77" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C77" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D77" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E77" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F77" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G77" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week for running and lifting.</t>
+        </is>
+      </c>
       <c r="H77" s="33">
         <f>IF(A77="","",COUNTIFS('Run sessions'!$A$2:$A$401,A77,'Run sessions'!$B$2:$B$401,B77))</f>
         <v/>
@@ -6269,12 +6357,32 @@
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="21">
-      <c r="A78" s="32" t="n"/>
-      <c r="B78" s="32" t="n"/>
-      <c r="C78" s="32" t="n"/>
-      <c r="D78" s="35" t="n"/>
-      <c r="E78" s="32" t="n"/>
-      <c r="F78" s="32" t="n"/>
+      <c r="A78" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B78" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D78" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E78" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F78" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G78" s="32" t="n"/>
       <c r="H78" s="33">
         <f>IF(A78="","",COUNTIFS('Run sessions'!$A$2:$A$401,A78,'Run sessions'!$B$2:$B$401,B78))</f>
@@ -6290,12 +6398,32 @@
       </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="21">
-      <c r="A79" s="32" t="n"/>
-      <c r="B79" s="32" t="n"/>
-      <c r="C79" s="32" t="n"/>
-      <c r="D79" s="35" t="n"/>
-      <c r="E79" s="32" t="n"/>
-      <c r="F79" s="32" t="n"/>
+      <c r="A79" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B79" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D79" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E79" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F79" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G79" s="32" t="n"/>
       <c r="H79" s="33">
         <f>IF(A79="","",COUNTIFS('Run sessions'!$A$2:$A$401,A79,'Run sessions'!$B$2:$B$401,B79))</f>
@@ -6311,13 +6439,37 @@
       </c>
     </row>
     <row r="80" ht="15" customHeight="1" s="21">
-      <c r="A80" s="32" t="n"/>
-      <c r="B80" s="32" t="n"/>
-      <c r="C80" s="32" t="n"/>
-      <c r="D80" s="35" t="n"/>
-      <c r="E80" s="32" t="n"/>
-      <c r="F80" s="32" t="n"/>
-      <c r="G80" s="32" t="n"/>
+      <c r="A80" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B80" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C80" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D80" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E80" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F80" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G80" s="32" t="inlineStr">
+        <is>
+          <t>Biggest week of the block.</t>
+        </is>
+      </c>
       <c r="H80" s="33">
         <f>IF(A80="","",COUNTIFS('Run sessions'!$A$2:$A$401,A80,'Run sessions'!$B$2:$B$401,B80))</f>
         <v/>
@@ -6332,13 +6484,37 @@
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="21">
-      <c r="A81" s="32" t="n"/>
-      <c r="B81" s="32" t="n"/>
-      <c r="C81" s="32" t="n"/>
-      <c r="D81" s="35" t="n"/>
-      <c r="E81" s="32" t="n"/>
-      <c r="F81" s="32" t="n"/>
-      <c r="G81" s="32" t="n"/>
+      <c r="A81" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B81" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D81" s="35" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E81" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F81" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G81" s="32" t="inlineStr">
+        <is>
+          <t>Lighter week with a 5K time trial: your result can update your paces for the next block.</t>
+        </is>
+      </c>
       <c r="H81" s="33">
         <f>IF(A81="","",COUNTIFS('Run sessions'!$A$2:$A$401,A81,'Run sessions'!$B$2:$B$401,B81))</f>
         <v/>
@@ -21633,219 +21809,699 @@
       <c r="G292" s="32" t="n"/>
     </row>
     <row r="293" ht="15" customHeight="1" s="21">
-      <c r="A293" s="32" t="n"/>
-      <c r="B293" s="32" t="n"/>
-      <c r="C293" s="32" t="n"/>
-      <c r="D293" s="32" t="n"/>
-      <c r="E293" s="32" t="n"/>
-      <c r="F293" s="32" t="n"/>
+      <c r="A293" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B293" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C293" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D293" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E293" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F293" s="32" t="inlineStr">
+        <is>
+          <t>6 x 800 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G293" s="32" t="n"/>
     </row>
     <row r="294" ht="15" customHeight="1" s="21">
-      <c r="A294" s="32" t="n"/>
-      <c r="B294" s="32" t="n"/>
-      <c r="C294" s="32" t="n"/>
-      <c r="D294" s="32" t="n"/>
-      <c r="E294" s="32" t="n"/>
-      <c r="F294" s="32" t="n"/>
+      <c r="A294" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B294" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C294" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D294" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E294" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F294" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G294" s="32" t="n"/>
     </row>
     <row r="295" ht="15" customHeight="1" s="21">
-      <c r="A295" s="32" t="n"/>
-      <c r="B295" s="32" t="n"/>
-      <c r="C295" s="32" t="n"/>
-      <c r="D295" s="32" t="n"/>
-      <c r="E295" s="32" t="n"/>
-      <c r="F295" s="32" t="n"/>
+      <c r="A295" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B295" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C295" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D295" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E295" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F295" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G295" s="32" t="n"/>
     </row>
     <row r="296" ht="15" customHeight="1" s="21">
-      <c r="A296" s="32" t="n"/>
-      <c r="B296" s="32" t="n"/>
-      <c r="C296" s="32" t="n"/>
-      <c r="D296" s="32" t="n"/>
-      <c r="E296" s="32" t="n"/>
-      <c r="F296" s="32" t="n"/>
+      <c r="A296" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B296" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C296" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D296" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E296" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F296" s="32" t="inlineStr">
+        <is>
+          <t>2 x 10 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G296" s="32" t="n"/>
     </row>
     <row r="297" ht="15" customHeight="1" s="21">
-      <c r="A297" s="32" t="n"/>
-      <c r="B297" s="32" t="n"/>
-      <c r="C297" s="32" t="n"/>
-      <c r="D297" s="32" t="n"/>
-      <c r="E297" s="32" t="n"/>
-      <c r="F297" s="32" t="n"/>
+      <c r="A297" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B297" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C297" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D297" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E297" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F297" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G297" s="32" t="n"/>
     </row>
     <row r="298" ht="15" customHeight="1" s="21">
-      <c r="A298" s="32" t="n"/>
-      <c r="B298" s="32" t="n"/>
-      <c r="C298" s="32" t="n"/>
-      <c r="D298" s="32" t="n"/>
-      <c r="E298" s="32" t="n"/>
-      <c r="F298" s="32" t="n"/>
+      <c r="A298" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B298" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C298" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D298" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E298" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F298" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G298" s="32" t="n"/>
     </row>
     <row r="299" ht="15" customHeight="1" s="21">
-      <c r="A299" s="32" t="n"/>
-      <c r="B299" s="32" t="n"/>
-      <c r="C299" s="32" t="n"/>
-      <c r="D299" s="32" t="n"/>
-      <c r="E299" s="32" t="n"/>
-      <c r="F299" s="32" t="n"/>
+      <c r="A299" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B299" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C299" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D299" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E299" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F299" s="32" t="inlineStr">
+        <is>
+          <t>5 x 1 km @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G299" s="32" t="n"/>
     </row>
     <row r="300" ht="15" customHeight="1" s="21">
-      <c r="A300" s="32" t="n"/>
-      <c r="B300" s="32" t="n"/>
-      <c r="C300" s="32" t="n"/>
-      <c r="D300" s="32" t="n"/>
-      <c r="E300" s="32" t="n"/>
-      <c r="F300" s="32" t="n"/>
+      <c r="A300" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B300" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C300" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D300" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E300" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F300" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G300" s="32" t="n"/>
     </row>
     <row r="301" ht="15" customHeight="1" s="21">
-      <c r="A301" s="32" t="n"/>
-      <c r="B301" s="32" t="n"/>
-      <c r="C301" s="32" t="n"/>
-      <c r="D301" s="32" t="n"/>
-      <c r="E301" s="32" t="n"/>
-      <c r="F301" s="32" t="n"/>
+      <c r="A301" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B301" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C301" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D301" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E301" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F301" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G301" s="32" t="n"/>
     </row>
     <row r="302" ht="15" customHeight="1" s="21">
-      <c r="A302" s="32" t="n"/>
-      <c r="B302" s="32" t="n"/>
-      <c r="C302" s="32" t="n"/>
-      <c r="D302" s="32" t="n"/>
-      <c r="E302" s="32" t="n"/>
-      <c r="F302" s="32" t="n"/>
+      <c r="A302" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B302" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C302" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D302" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E302" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F302" s="32" t="inlineStr">
+        <is>
+          <t>15 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G302" s="32" t="n"/>
     </row>
     <row r="303" ht="15" customHeight="1" s="21">
-      <c r="A303" s="32" t="n"/>
-      <c r="B303" s="32" t="n"/>
-      <c r="C303" s="32" t="n"/>
-      <c r="D303" s="32" t="n"/>
-      <c r="E303" s="32" t="n"/>
-      <c r="F303" s="32" t="n"/>
+      <c r="A303" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B303" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C303" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D303" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E303" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F303" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G303" s="32" t="n"/>
     </row>
     <row r="304" ht="15" customHeight="1" s="21">
-      <c r="A304" s="32" t="n"/>
-      <c r="B304" s="32" t="n"/>
-      <c r="C304" s="32" t="n"/>
-      <c r="D304" s="32" t="n"/>
-      <c r="E304" s="32" t="n"/>
-      <c r="F304" s="32" t="n"/>
+      <c r="A304" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B304" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C304" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D304" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E304" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F304" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G304" s="32" t="n"/>
     </row>
     <row r="305" ht="15" customHeight="1" s="21">
-      <c r="A305" s="32" t="n"/>
-      <c r="B305" s="32" t="n"/>
-      <c r="C305" s="32" t="n"/>
-      <c r="D305" s="32" t="n"/>
-      <c r="E305" s="32" t="n"/>
-      <c r="F305" s="32" t="n"/>
+      <c r="A305" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B305" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C305" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D305" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E305" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F305" s="32" t="inlineStr">
+        <is>
+          <t>8 x 600 m @ I, 75 s jog between</t>
+        </is>
+      </c>
       <c r="G305" s="32" t="n"/>
     </row>
     <row r="306" ht="15" customHeight="1" s="21">
-      <c r="A306" s="32" t="n"/>
-      <c r="B306" s="32" t="n"/>
-      <c r="C306" s="32" t="n"/>
-      <c r="D306" s="32" t="n"/>
-      <c r="E306" s="32" t="n"/>
-      <c r="F306" s="32" t="n"/>
+      <c r="A306" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B306" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C306" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D306" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E306" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F306" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G306" s="32" t="n"/>
     </row>
     <row r="307" ht="15" customHeight="1" s="21">
-      <c r="A307" s="32" t="n"/>
-      <c r="B307" s="32" t="n"/>
-      <c r="C307" s="32" t="n"/>
-      <c r="D307" s="32" t="n"/>
-      <c r="E307" s="32" t="n"/>
-      <c r="F307" s="32" t="n"/>
+      <c r="A307" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B307" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C307" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D307" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E307" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F307" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G307" s="32" t="n"/>
     </row>
     <row r="308" ht="15" customHeight="1" s="21">
-      <c r="A308" s="32" t="n"/>
-      <c r="B308" s="32" t="n"/>
-      <c r="C308" s="32" t="n"/>
-      <c r="D308" s="32" t="n"/>
-      <c r="E308" s="32" t="n"/>
-      <c r="F308" s="32" t="n"/>
+      <c r="A308" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B308" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C308" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D308" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E308" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F308" s="32" t="inlineStr">
+        <is>
+          <t>3 x 8 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G308" s="32" t="n"/>
     </row>
     <row r="309" ht="15" customHeight="1" s="21">
-      <c r="A309" s="32" t="n"/>
-      <c r="B309" s="32" t="n"/>
-      <c r="C309" s="32" t="n"/>
-      <c r="D309" s="32" t="n"/>
-      <c r="E309" s="32" t="n"/>
-      <c r="F309" s="32" t="n"/>
+      <c r="A309" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B309" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C309" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D309" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E309" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F309" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G309" s="32" t="n"/>
     </row>
     <row r="310" ht="15" customHeight="1" s="21">
-      <c r="A310" s="32" t="n"/>
-      <c r="B310" s="32" t="n"/>
-      <c r="C310" s="32" t="n"/>
-      <c r="D310" s="32" t="n"/>
-      <c r="E310" s="32" t="n"/>
-      <c r="F310" s="32" t="n"/>
+      <c r="A310" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B310" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C310" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D310" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E310" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F310" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G310" s="32" t="n"/>
     </row>
     <row r="311" ht="15" customHeight="1" s="21">
-      <c r="A311" s="32" t="n"/>
-      <c r="B311" s="32" t="n"/>
-      <c r="C311" s="32" t="n"/>
-      <c r="D311" s="32" t="n"/>
-      <c r="E311" s="32" t="n"/>
-      <c r="F311" s="32" t="n"/>
+      <c r="A311" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B311" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C311" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D311" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E311" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F311" s="32" t="inlineStr">
+        <is>
+          <t>6 x 1 km @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G311" s="32" t="n"/>
     </row>
     <row r="312" ht="15" customHeight="1" s="21">
-      <c r="A312" s="32" t="n"/>
-      <c r="B312" s="32" t="n"/>
-      <c r="C312" s="32" t="n"/>
-      <c r="D312" s="32" t="n"/>
-      <c r="E312" s="32" t="n"/>
-      <c r="F312" s="32" t="n"/>
+      <c r="A312" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B312" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C312" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D312" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E312" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F312" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G312" s="32" t="n"/>
     </row>
     <row r="313" ht="15" customHeight="1" s="21">
-      <c r="A313" s="32" t="n"/>
-      <c r="B313" s="32" t="n"/>
-      <c r="C313" s="32" t="n"/>
-      <c r="D313" s="32" t="n"/>
-      <c r="E313" s="32" t="n"/>
-      <c r="F313" s="32" t="n"/>
+      <c r="A313" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B313" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C313" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D313" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E313" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F313" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G313" s="32" t="n"/>
     </row>
     <row r="314" ht="15" customHeight="1" s="21">
-      <c r="A314" s="32" t="n"/>
-      <c r="B314" s="32" t="n"/>
-      <c r="C314" s="32" t="n"/>
-      <c r="D314" s="32" t="n"/>
-      <c r="E314" s="32" t="n"/>
-      <c r="F314" s="32" t="n"/>
+      <c r="A314" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B314" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C314" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D314" s="32" t="inlineStr">
+        <is>
+          <t>Race</t>
+        </is>
+      </c>
+      <c r="E314" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F314" s="32" t="inlineStr">
+        <is>
+          <t>5K time trial – hard but even, to update your paces</t>
+        </is>
+      </c>
       <c r="G314" s="32" t="n"/>
     </row>
     <row r="315" ht="15" customHeight="1" s="21">
-      <c r="A315" s="32" t="n"/>
-      <c r="B315" s="32" t="n"/>
-      <c r="C315" s="32" t="n"/>
-      <c r="D315" s="32" t="n"/>
-      <c r="E315" s="32" t="n"/>
-      <c r="F315" s="32" t="n"/>
+      <c r="A315" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B315" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C315" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D315" s="32" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="E315" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F315" s="32" t="inlineStr">
+        <is>
+          <t>E continuous run</t>
+        </is>
+      </c>
       <c r="G315" s="32" t="n"/>
     </row>
     <row r="316" ht="15" customHeight="1" s="21">
-      <c r="A316" s="32" t="n"/>
-      <c r="B316" s="32" t="n"/>
-      <c r="C316" s="32" t="n"/>
-      <c r="D316" s="32" t="n"/>
-      <c r="E316" s="32" t="n"/>
-      <c r="F316" s="32" t="n"/>
+      <c r="A316" s="32" t="inlineStr">
+        <is>
+          <t>Balanced hybrid</t>
+        </is>
+      </c>
+      <c r="B316" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C316" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D316" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E316" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F316" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G316" s="32" t="n"/>
     </row>
     <row r="317" ht="15" customHeight="1" s="21">

</xml_diff>

<commit_message>
Build strength and Build muscle programmes (8 weeks, two runs, deload in week 8)
Lifting goals place gym days first and keep leg sessions over a hard run.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -2682,7 +2682,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G7" s="32" t="n">
         <v>2</v>
@@ -2706,7 +2706,7 @@
         <v>25</v>
       </c>
       <c r="N7" s="32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="32" t="inlineStr">
         <is>
@@ -2756,7 +2756,7 @@
         <v>1</v>
       </c>
       <c r="F8" s="32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G8" s="32" t="n">
         <v>3</v>
@@ -2780,7 +2780,7 @@
         <v>25</v>
       </c>
       <c r="N8" s="32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O8" s="32" t="inlineStr">
         <is>
@@ -6529,13 +6529,37 @@
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="21">
-      <c r="A82" s="32" t="n"/>
-      <c r="B82" s="32" t="n"/>
-      <c r="C82" s="32" t="n"/>
-      <c r="D82" s="35" t="n"/>
-      <c r="E82" s="32" t="n"/>
-      <c r="F82" s="32" t="n"/>
-      <c r="G82" s="32" t="n"/>
+      <c r="A82" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B82" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D82" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F82" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G82" s="32" t="inlineStr">
+        <is>
+          <t>Settle in: heavy lifting with two runs to keep your engine.</t>
+        </is>
+      </c>
       <c r="H82" s="33">
         <f>IF(A82="","",COUNTIFS('Run sessions'!$A$2:$A$401,A82,'Run sessions'!$B$2:$B$401,B82))</f>
         <v/>
@@ -6550,12 +6574,32 @@
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="21">
-      <c r="A83" s="32" t="n"/>
-      <c r="B83" s="32" t="n"/>
-      <c r="C83" s="32" t="n"/>
-      <c r="D83" s="35" t="n"/>
-      <c r="E83" s="32" t="n"/>
-      <c r="F83" s="32" t="n"/>
+      <c r="A83" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B83" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D83" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E83" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F83" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G83" s="32" t="n"/>
       <c r="H83" s="33">
         <f>IF(A83="","",COUNTIFS('Run sessions'!$A$2:$A$401,A83,'Run sessions'!$B$2:$B$401,B83))</f>
@@ -6571,12 +6615,32 @@
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="21">
-      <c r="A84" s="32" t="n"/>
-      <c r="B84" s="32" t="n"/>
-      <c r="C84" s="32" t="n"/>
-      <c r="D84" s="35" t="n"/>
-      <c r="E84" s="32" t="n"/>
-      <c r="F84" s="32" t="n"/>
+      <c r="A84" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B84" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C84" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D84" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E84" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F84" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G84" s="32" t="n"/>
       <c r="H84" s="33">
         <f>IF(A84="","",COUNTIFS('Run sessions'!$A$2:$A$401,A84,'Run sessions'!$B$2:$B$401,B84))</f>
@@ -6592,12 +6656,32 @@
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="21">
-      <c r="A85" s="32" t="n"/>
-      <c r="B85" s="32" t="n"/>
-      <c r="C85" s="32" t="n"/>
-      <c r="D85" s="35" t="n"/>
-      <c r="E85" s="32" t="n"/>
-      <c r="F85" s="32" t="n"/>
+      <c r="A85" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B85" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C85" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D85" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E85" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F85" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G85" s="32" t="n"/>
       <c r="H85" s="33">
         <f>IF(A85="","",COUNTIFS('Run sessions'!$A$2:$A$401,A85,'Run sessions'!$B$2:$B$401,B85))</f>
@@ -6613,12 +6697,32 @@
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="21">
-      <c r="A86" s="32" t="n"/>
-      <c r="B86" s="32" t="n"/>
-      <c r="C86" s="32" t="n"/>
-      <c r="D86" s="35" t="n"/>
-      <c r="E86" s="32" t="n"/>
-      <c r="F86" s="32" t="n"/>
+      <c r="A86" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B86" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C86" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D86" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E86" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F86" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G86" s="32" t="n"/>
       <c r="H86" s="33">
         <f>IF(A86="","",COUNTIFS('Run sessions'!$A$2:$A$401,A86,'Run sessions'!$B$2:$B$401,B86))</f>
@@ -6634,12 +6738,32 @@
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="21">
-      <c r="A87" s="32" t="n"/>
-      <c r="B87" s="32" t="n"/>
-      <c r="C87" s="32" t="n"/>
-      <c r="D87" s="35" t="n"/>
-      <c r="E87" s="32" t="n"/>
-      <c r="F87" s="32" t="n"/>
+      <c r="A87" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B87" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C87" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D87" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E87" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F87" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G87" s="32" t="n"/>
       <c r="H87" s="33">
         <f>IF(A87="","",COUNTIFS('Run sessions'!$A$2:$A$401,A87,'Run sessions'!$B$2:$B$401,B87))</f>
@@ -6655,13 +6779,37 @@
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="21">
-      <c r="A88" s="32" t="n"/>
-      <c r="B88" s="32" t="n"/>
-      <c r="C88" s="32" t="n"/>
-      <c r="D88" s="35" t="n"/>
-      <c r="E88" s="32" t="n"/>
-      <c r="F88" s="32" t="n"/>
-      <c r="G88" s="32" t="n"/>
+      <c r="A88" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B88" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C88" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D88" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E88" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F88" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="G88" s="32" t="inlineStr">
+        <is>
+          <t>Hardest week of the block.</t>
+        </is>
+      </c>
       <c r="H88" s="33">
         <f>IF(A88="","",COUNTIFS('Run sessions'!$A$2:$A$401,A88,'Run sessions'!$B$2:$B$401,B88))</f>
         <v/>
@@ -6676,13 +6824,37 @@
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="21">
-      <c r="A89" s="32" t="n"/>
-      <c r="B89" s="32" t="n"/>
-      <c r="C89" s="32" t="n"/>
-      <c r="D89" s="35" t="n"/>
-      <c r="E89" s="32" t="n"/>
-      <c r="F89" s="32" t="n"/>
-      <c r="G89" s="32" t="n"/>
+      <c r="A89" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B89" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C89" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D89" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E89" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F89" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G89" s="32" t="inlineStr">
+        <is>
+          <t>Deload: lighter lifting and easy running before the next block.</t>
+        </is>
+      </c>
       <c r="H89" s="33">
         <f>IF(A89="","",COUNTIFS('Run sessions'!$A$2:$A$401,A89,'Run sessions'!$B$2:$B$401,B89))</f>
         <v/>
@@ -6697,13 +6869,37 @@
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="21">
-      <c r="A90" s="32" t="n"/>
-      <c r="B90" s="32" t="n"/>
-      <c r="C90" s="32" t="n"/>
-      <c r="D90" s="35" t="n"/>
-      <c r="E90" s="32" t="n"/>
-      <c r="F90" s="32" t="n"/>
-      <c r="G90" s="32" t="n"/>
+      <c r="A90" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B90" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D90" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F90" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G90" s="32" t="inlineStr">
+        <is>
+          <t>Settle in: muscle-building lifting with two runs to keep your engine.</t>
+        </is>
+      </c>
       <c r="H90" s="33">
         <f>IF(A90="","",COUNTIFS('Run sessions'!$A$2:$A$401,A90,'Run sessions'!$B$2:$B$401,B90))</f>
         <v/>
@@ -6718,12 +6914,32 @@
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="21">
-      <c r="A91" s="32" t="n"/>
-      <c r="B91" s="32" t="n"/>
-      <c r="C91" s="32" t="n"/>
-      <c r="D91" s="35" t="n"/>
-      <c r="E91" s="32" t="n"/>
-      <c r="F91" s="32" t="n"/>
+      <c r="A91" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B91" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" s="32" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D91" s="35" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E91" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F91" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G91" s="32" t="n"/>
       <c r="H91" s="33">
         <f>IF(A91="","",COUNTIFS('Run sessions'!$A$2:$A$401,A91,'Run sessions'!$B$2:$B$401,B91))</f>
@@ -6739,12 +6955,32 @@
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="21">
-      <c r="A92" s="32" t="n"/>
-      <c r="B92" s="32" t="n"/>
-      <c r="C92" s="32" t="n"/>
-      <c r="D92" s="35" t="n"/>
-      <c r="E92" s="32" t="n"/>
-      <c r="F92" s="32" t="n"/>
+      <c r="A92" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B92" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C92" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D92" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E92" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F92" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G92" s="32" t="n"/>
       <c r="H92" s="33">
         <f>IF(A92="","",COUNTIFS('Run sessions'!$A$2:$A$401,A92,'Run sessions'!$B$2:$B$401,B92))</f>
@@ -6760,12 +6996,32 @@
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="21">
-      <c r="A93" s="32" t="n"/>
-      <c r="B93" s="32" t="n"/>
-      <c r="C93" s="32" t="n"/>
-      <c r="D93" s="35" t="n"/>
-      <c r="E93" s="32" t="n"/>
-      <c r="F93" s="32" t="n"/>
+      <c r="A93" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B93" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C93" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D93" s="35" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E93" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F93" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G93" s="32" t="n"/>
       <c r="H93" s="33">
         <f>IF(A93="","",COUNTIFS('Run sessions'!$A$2:$A$401,A93,'Run sessions'!$B$2:$B$401,B93))</f>
@@ -6781,12 +7037,32 @@
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="21">
-      <c r="A94" s="32" t="n"/>
-      <c r="B94" s="32" t="n"/>
-      <c r="C94" s="32" t="n"/>
-      <c r="D94" s="35" t="n"/>
-      <c r="E94" s="32" t="n"/>
-      <c r="F94" s="32" t="n"/>
+      <c r="A94" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B94" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C94" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D94" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E94" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F94" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
       <c r="G94" s="32" t="n"/>
       <c r="H94" s="33">
         <f>IF(A94="","",COUNTIFS('Run sessions'!$A$2:$A$401,A94,'Run sessions'!$B$2:$B$401,B94))</f>
@@ -6802,12 +7078,32 @@
       </c>
     </row>
     <row r="95" ht="15" customHeight="1" s="21">
-      <c r="A95" s="32" t="n"/>
-      <c r="B95" s="32" t="n"/>
-      <c r="C95" s="32" t="n"/>
-      <c r="D95" s="35" t="n"/>
-      <c r="E95" s="32" t="n"/>
-      <c r="F95" s="32" t="n"/>
+      <c r="A95" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B95" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C95" s="32" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D95" s="35" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="E95" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F95" s="32" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
       <c r="G95" s="32" t="n"/>
       <c r="H95" s="33">
         <f>IF(A95="","",COUNTIFS('Run sessions'!$A$2:$A$401,A95,'Run sessions'!$B$2:$B$401,B95))</f>
@@ -6823,13 +7119,37 @@
       </c>
     </row>
     <row r="96" ht="15" customHeight="1" s="21">
-      <c r="A96" s="32" t="n"/>
-      <c r="B96" s="32" t="n"/>
-      <c r="C96" s="32" t="n"/>
-      <c r="D96" s="35" t="n"/>
-      <c r="E96" s="32" t="n"/>
-      <c r="F96" s="32" t="n"/>
-      <c r="G96" s="32" t="n"/>
+      <c r="A96" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B96" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C96" s="32" t="inlineStr">
+        <is>
+          <t>Peak</t>
+        </is>
+      </c>
+      <c r="D96" s="35" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E96" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F96" s="32" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="G96" s="32" t="inlineStr">
+        <is>
+          <t>Hardest week of the block.</t>
+        </is>
+      </c>
       <c r="H96" s="33">
         <f>IF(A96="","",COUNTIFS('Run sessions'!$A$2:$A$401,A96,'Run sessions'!$B$2:$B$401,B96))</f>
         <v/>
@@ -6844,13 +7164,37 @@
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="21">
-      <c r="A97" s="32" t="n"/>
-      <c r="B97" s="32" t="n"/>
-      <c r="C97" s="32" t="n"/>
-      <c r="D97" s="35" t="n"/>
-      <c r="E97" s="32" t="n"/>
-      <c r="F97" s="32" t="n"/>
-      <c r="G97" s="32" t="n"/>
+      <c r="A97" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B97" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C97" s="32" t="inlineStr">
+        <is>
+          <t>Deload</t>
+        </is>
+      </c>
+      <c r="D97" s="35" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E97" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F97" s="32" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="G97" s="32" t="inlineStr">
+        <is>
+          <t>Deload: lighter lifting and easy running before the next block.</t>
+        </is>
+      </c>
       <c r="H97" s="33">
         <f>IF(A97="","",COUNTIFS('Run sessions'!$A$2:$A$401,A97,'Run sessions'!$B$2:$B$401,B97))</f>
         <v/>
@@ -22505,291 +22849,931 @@
       <c r="G316" s="32" t="n"/>
     </row>
     <row r="317" ht="15" customHeight="1" s="21">
-      <c r="A317" s="32" t="n"/>
-      <c r="B317" s="32" t="n"/>
-      <c r="C317" s="32" t="n"/>
-      <c r="D317" s="32" t="n"/>
-      <c r="E317" s="32" t="n"/>
-      <c r="F317" s="32" t="n"/>
+      <c r="A317" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B317" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C317" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D317" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E317" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F317" s="32" t="inlineStr">
+        <is>
+          <t>2 x 8 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G317" s="32" t="n"/>
     </row>
     <row r="318" ht="15" customHeight="1" s="21">
-      <c r="A318" s="32" t="n"/>
-      <c r="B318" s="32" t="n"/>
-      <c r="C318" s="32" t="n"/>
-      <c r="D318" s="32" t="n"/>
-      <c r="E318" s="32" t="n"/>
-      <c r="F318" s="32" t="n"/>
+      <c r="A318" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B318" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C318" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D318" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E318" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F318" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G318" s="32" t="n"/>
     </row>
     <row r="319" ht="15" customHeight="1" s="21">
-      <c r="A319" s="32" t="n"/>
-      <c r="B319" s="32" t="n"/>
-      <c r="C319" s="32" t="n"/>
-      <c r="D319" s="32" t="n"/>
-      <c r="E319" s="32" t="n"/>
-      <c r="F319" s="32" t="n"/>
+      <c r="A319" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B319" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C319" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D319" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E319" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F319" s="32" t="inlineStr">
+        <is>
+          <t>6 x 600 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G319" s="32" t="n"/>
     </row>
     <row r="320" ht="15" customHeight="1" s="21">
-      <c r="A320" s="32" t="n"/>
-      <c r="B320" s="32" t="n"/>
-      <c r="C320" s="32" t="n"/>
-      <c r="D320" s="32" t="n"/>
-      <c r="E320" s="32" t="n"/>
-      <c r="F320" s="32" t="n"/>
+      <c r="A320" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B320" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C320" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D320" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E320" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F320" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G320" s="32" t="n"/>
     </row>
     <row r="321" ht="15" customHeight="1" s="21">
-      <c r="A321" s="32" t="n"/>
-      <c r="B321" s="32" t="n"/>
-      <c r="C321" s="32" t="n"/>
-      <c r="D321" s="32" t="n"/>
-      <c r="E321" s="32" t="n"/>
-      <c r="F321" s="32" t="n"/>
+      <c r="A321" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B321" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C321" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D321" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E321" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F321" s="32" t="inlineStr">
+        <is>
+          <t>15 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G321" s="32" t="n"/>
     </row>
     <row r="322" ht="15" customHeight="1" s="21">
-      <c r="A322" s="32" t="n"/>
-      <c r="B322" s="32" t="n"/>
-      <c r="C322" s="32" t="n"/>
-      <c r="D322" s="32" t="n"/>
-      <c r="E322" s="32" t="n"/>
-      <c r="F322" s="32" t="n"/>
+      <c r="A322" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B322" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C322" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D322" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E322" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F322" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G322" s="32" t="n"/>
     </row>
     <row r="323" ht="15" customHeight="1" s="21">
-      <c r="A323" s="32" t="n"/>
-      <c r="B323" s="32" t="n"/>
-      <c r="C323" s="32" t="n"/>
-      <c r="D323" s="32" t="n"/>
-      <c r="E323" s="32" t="n"/>
-      <c r="F323" s="32" t="n"/>
+      <c r="A323" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B323" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C323" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D323" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E323" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F323" s="32" t="inlineStr">
+        <is>
+          <t>5 x 800 m @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G323" s="32" t="n"/>
     </row>
     <row r="324" ht="15" customHeight="1" s="21">
-      <c r="A324" s="32" t="n"/>
-      <c r="B324" s="32" t="n"/>
-      <c r="C324" s="32" t="n"/>
-      <c r="D324" s="32" t="n"/>
-      <c r="E324" s="32" t="n"/>
-      <c r="F324" s="32" t="n"/>
+      <c r="A324" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B324" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C324" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D324" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E324" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F324" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G324" s="32" t="n"/>
     </row>
     <row r="325" ht="15" customHeight="1" s="21">
-      <c r="A325" s="32" t="n"/>
-      <c r="B325" s="32" t="n"/>
-      <c r="C325" s="32" t="n"/>
-      <c r="D325" s="32" t="n"/>
-      <c r="E325" s="32" t="n"/>
-      <c r="F325" s="32" t="n"/>
+      <c r="A325" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B325" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C325" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D325" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E325" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F325" s="32" t="inlineStr">
+        <is>
+          <t>3 x 6 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G325" s="32" t="n"/>
     </row>
     <row r="326" ht="15" customHeight="1" s="21">
-      <c r="A326" s="32" t="n"/>
-      <c r="B326" s="32" t="n"/>
-      <c r="C326" s="32" t="n"/>
-      <c r="D326" s="32" t="n"/>
-      <c r="E326" s="32" t="n"/>
-      <c r="F326" s="32" t="n"/>
+      <c r="A326" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B326" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C326" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D326" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E326" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F326" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G326" s="32" t="n"/>
     </row>
     <row r="327" ht="15" customHeight="1" s="21">
-      <c r="A327" s="32" t="n"/>
-      <c r="B327" s="32" t="n"/>
-      <c r="C327" s="32" t="n"/>
-      <c r="D327" s="32" t="n"/>
-      <c r="E327" s="32" t="n"/>
-      <c r="F327" s="32" t="n"/>
+      <c r="A327" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B327" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C327" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D327" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E327" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F327" s="32" t="inlineStr">
+        <is>
+          <t>6 x 800 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G327" s="32" t="n"/>
     </row>
     <row r="328" ht="15" customHeight="1" s="21">
-      <c r="A328" s="32" t="n"/>
-      <c r="B328" s="32" t="n"/>
-      <c r="C328" s="32" t="n"/>
-      <c r="D328" s="32" t="n"/>
-      <c r="E328" s="32" t="n"/>
-      <c r="F328" s="32" t="n"/>
+      <c r="A328" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B328" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C328" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D328" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E328" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F328" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G328" s="32" t="n"/>
     </row>
     <row r="329" ht="15" customHeight="1" s="21">
-      <c r="A329" s="32" t="n"/>
-      <c r="B329" s="32" t="n"/>
-      <c r="C329" s="32" t="n"/>
-      <c r="D329" s="32" t="n"/>
-      <c r="E329" s="32" t="n"/>
-      <c r="F329" s="32" t="n"/>
+      <c r="A329" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B329" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C329" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D329" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E329" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F329" s="32" t="inlineStr">
+        <is>
+          <t>20 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G329" s="32" t="n"/>
     </row>
     <row r="330" ht="15" customHeight="1" s="21">
-      <c r="A330" s="32" t="n"/>
-      <c r="B330" s="32" t="n"/>
-      <c r="C330" s="32" t="n"/>
-      <c r="D330" s="32" t="n"/>
-      <c r="E330" s="32" t="n"/>
-      <c r="F330" s="32" t="n"/>
+      <c r="A330" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B330" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C330" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D330" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E330" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F330" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G330" s="32" t="n"/>
     </row>
     <row r="331" ht="15" customHeight="1" s="21">
-      <c r="A331" s="32" t="n"/>
-      <c r="B331" s="32" t="n"/>
-      <c r="C331" s="32" t="n"/>
-      <c r="D331" s="32" t="n"/>
-      <c r="E331" s="32" t="n"/>
-      <c r="F331" s="32" t="n"/>
+      <c r="A331" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B331" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C331" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D331" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E331" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F331" s="32" t="inlineStr">
+        <is>
+          <t>6 x (1 min @ T effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G331" s="32" t="n"/>
     </row>
     <row r="332" ht="15" customHeight="1" s="21">
-      <c r="A332" s="32" t="n"/>
-      <c r="B332" s="32" t="n"/>
-      <c r="C332" s="32" t="n"/>
-      <c r="D332" s="32" t="n"/>
-      <c r="E332" s="32" t="n"/>
-      <c r="F332" s="32" t="n"/>
+      <c r="A332" s="32" t="inlineStr">
+        <is>
+          <t>Build strength</t>
+        </is>
+      </c>
+      <c r="B332" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C332" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D332" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E332" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F332" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G332" s="32" t="n"/>
     </row>
     <row r="333" ht="15" customHeight="1" s="21">
-      <c r="A333" s="32" t="n"/>
-      <c r="B333" s="32" t="n"/>
-      <c r="C333" s="32" t="n"/>
-      <c r="D333" s="32" t="n"/>
-      <c r="E333" s="32" t="n"/>
-      <c r="F333" s="32" t="n"/>
+      <c r="A333" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B333" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C333" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D333" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E333" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F333" s="32" t="inlineStr">
+        <is>
+          <t>2 x 8 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G333" s="32" t="n"/>
     </row>
     <row r="334" ht="15" customHeight="1" s="21">
-      <c r="A334" s="32" t="n"/>
-      <c r="B334" s="32" t="n"/>
-      <c r="C334" s="32" t="n"/>
-      <c r="D334" s="32" t="n"/>
-      <c r="E334" s="32" t="n"/>
-      <c r="F334" s="32" t="n"/>
+      <c r="A334" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B334" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C334" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D334" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E334" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F334" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G334" s="32" t="n"/>
     </row>
     <row r="335" ht="15" customHeight="1" s="21">
-      <c r="A335" s="32" t="n"/>
-      <c r="B335" s="32" t="n"/>
-      <c r="C335" s="32" t="n"/>
-      <c r="D335" s="32" t="n"/>
-      <c r="E335" s="32" t="n"/>
-      <c r="F335" s="32" t="n"/>
+      <c r="A335" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B335" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C335" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D335" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E335" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F335" s="32" t="inlineStr">
+        <is>
+          <t>6 x 600 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G335" s="32" t="n"/>
     </row>
     <row r="336" ht="15" customHeight="1" s="21">
-      <c r="A336" s="32" t="n"/>
-      <c r="B336" s="32" t="n"/>
-      <c r="C336" s="32" t="n"/>
-      <c r="D336" s="32" t="n"/>
-      <c r="E336" s="32" t="n"/>
-      <c r="F336" s="32" t="n"/>
+      <c r="A336" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B336" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C336" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D336" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E336" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F336" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G336" s="32" t="n"/>
     </row>
     <row r="337" ht="15" customHeight="1" s="21">
-      <c r="A337" s="32" t="n"/>
-      <c r="B337" s="32" t="n"/>
-      <c r="C337" s="32" t="n"/>
-      <c r="D337" s="32" t="n"/>
-      <c r="E337" s="32" t="n"/>
-      <c r="F337" s="32" t="n"/>
+      <c r="A337" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B337" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C337" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D337" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E337" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F337" s="32" t="inlineStr">
+        <is>
+          <t>15 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G337" s="32" t="n"/>
     </row>
     <row r="338" ht="15" customHeight="1" s="21">
-      <c r="A338" s="32" t="n"/>
-      <c r="B338" s="32" t="n"/>
-      <c r="C338" s="32" t="n"/>
-      <c r="D338" s="32" t="n"/>
-      <c r="E338" s="32" t="n"/>
-      <c r="F338" s="32" t="n"/>
+      <c r="A338" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B338" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C338" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D338" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E338" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F338" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G338" s="32" t="n"/>
     </row>
     <row r="339" ht="15" customHeight="1" s="21">
-      <c r="A339" s="32" t="n"/>
-      <c r="B339" s="32" t="n"/>
-      <c r="C339" s="32" t="n"/>
-      <c r="D339" s="32" t="n"/>
-      <c r="E339" s="32" t="n"/>
-      <c r="F339" s="32" t="n"/>
+      <c r="A339" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B339" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C339" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D339" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E339" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F339" s="32" t="inlineStr">
+        <is>
+          <t>5 x 800 m @ I, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G339" s="32" t="n"/>
     </row>
     <row r="340" ht="15" customHeight="1" s="21">
-      <c r="A340" s="32" t="n"/>
-      <c r="B340" s="32" t="n"/>
-      <c r="C340" s="32" t="n"/>
-      <c r="D340" s="32" t="n"/>
-      <c r="E340" s="32" t="n"/>
-      <c r="F340" s="32" t="n"/>
+      <c r="A340" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B340" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="C340" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D340" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E340" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F340" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G340" s="32" t="n"/>
     </row>
     <row r="341" ht="15" customHeight="1" s="21">
-      <c r="A341" s="32" t="n"/>
-      <c r="B341" s="32" t="n"/>
-      <c r="C341" s="32" t="n"/>
-      <c r="D341" s="32" t="n"/>
-      <c r="E341" s="32" t="n"/>
-      <c r="F341" s="32" t="n"/>
+      <c r="A341" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B341" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C341" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D341" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E341" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F341" s="32" t="inlineStr">
+        <is>
+          <t>3 x 6 min @ T, 2 min jog between</t>
+        </is>
+      </c>
       <c r="G341" s="32" t="n"/>
     </row>
     <row r="342" ht="15" customHeight="1" s="21">
-      <c r="A342" s="32" t="n"/>
-      <c r="B342" s="32" t="n"/>
-      <c r="C342" s="32" t="n"/>
-      <c r="D342" s="32" t="n"/>
-      <c r="E342" s="32" t="n"/>
-      <c r="F342" s="32" t="n"/>
+      <c r="A342" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B342" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C342" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D342" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E342" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F342" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G342" s="32" t="n"/>
     </row>
     <row r="343" ht="15" customHeight="1" s="21">
-      <c r="A343" s="32" t="n"/>
-      <c r="B343" s="32" t="n"/>
-      <c r="C343" s="32" t="n"/>
-      <c r="D343" s="32" t="n"/>
-      <c r="E343" s="32" t="n"/>
-      <c r="F343" s="32" t="n"/>
+      <c r="A343" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B343" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C343" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D343" s="32" t="inlineStr">
+        <is>
+          <t>Intervals</t>
+        </is>
+      </c>
+      <c r="E343" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F343" s="32" t="inlineStr">
+        <is>
+          <t>6 x 800 m @ I, 90 s jog between</t>
+        </is>
+      </c>
       <c r="G343" s="32" t="n"/>
     </row>
     <row r="344" ht="15" customHeight="1" s="21">
-      <c r="A344" s="32" t="n"/>
-      <c r="B344" s="32" t="n"/>
-      <c r="C344" s="32" t="n"/>
-      <c r="D344" s="32" t="n"/>
-      <c r="E344" s="32" t="n"/>
-      <c r="F344" s="32" t="n"/>
+      <c r="A344" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B344" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="C344" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D344" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E344" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F344" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G344" s="32" t="n"/>
     </row>
     <row r="345" ht="15" customHeight="1" s="21">
-      <c r="A345" s="32" t="n"/>
-      <c r="B345" s="32" t="n"/>
-      <c r="C345" s="32" t="n"/>
-      <c r="D345" s="32" t="n"/>
-      <c r="E345" s="32" t="n"/>
-      <c r="F345" s="32" t="n"/>
+      <c r="A345" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B345" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C345" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D345" s="32" t="inlineStr">
+        <is>
+          <t>Tempo</t>
+        </is>
+      </c>
+      <c r="E345" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F345" s="32" t="inlineStr">
+        <is>
+          <t>20 min continuous @ T</t>
+        </is>
+      </c>
       <c r="G345" s="32" t="n"/>
     </row>
     <row r="346" ht="15" customHeight="1" s="21">
-      <c r="A346" s="32" t="n"/>
-      <c r="B346" s="32" t="n"/>
-      <c r="C346" s="32" t="n"/>
-      <c r="D346" s="32" t="n"/>
-      <c r="E346" s="32" t="n"/>
-      <c r="F346" s="32" t="n"/>
+      <c r="A346" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B346" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="C346" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D346" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E346" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F346" s="32" t="inlineStr">
+        <is>
+          <t>Long run, conversational throughout</t>
+        </is>
+      </c>
       <c r="G346" s="32" t="n"/>
     </row>
     <row r="347" ht="15" customHeight="1" s="21">
-      <c r="A347" s="32" t="n"/>
-      <c r="B347" s="32" t="n"/>
-      <c r="C347" s="32" t="n"/>
-      <c r="D347" s="32" t="n"/>
-      <c r="E347" s="32" t="n"/>
-      <c r="F347" s="32" t="n"/>
+      <c r="A347" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B347" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C347" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D347" s="32" t="inlineStr">
+        <is>
+          <t>Fartlek</t>
+        </is>
+      </c>
+      <c r="E347" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F347" s="32" t="inlineStr">
+        <is>
+          <t>6 x (1 min @ T effort / 1 min E)</t>
+        </is>
+      </c>
       <c r="G347" s="32" t="n"/>
     </row>
     <row r="348" ht="15" customHeight="1" s="21">
-      <c r="A348" s="32" t="n"/>
-      <c r="B348" s="32" t="n"/>
-      <c r="C348" s="32" t="n"/>
-      <c r="D348" s="32" t="n"/>
-      <c r="E348" s="32" t="n"/>
-      <c r="F348" s="32" t="n"/>
+      <c r="A348" s="32" t="inlineStr">
+        <is>
+          <t>Build muscle</t>
+        </is>
+      </c>
+      <c r="B348" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="C348" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D348" s="32" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="E348" s="32" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
+      <c r="F348" s="32" t="inlineStr">
+        <is>
+          <t>Shorter long run, E</t>
+        </is>
+      </c>
       <c r="G348" s="32" t="n"/>
     </row>
     <row r="349" ht="15" customHeight="1" s="21">

</xml_diff>

<commit_message>
Planner: gym week first with no same-muscle sessions back to back, long run on a chosen day; runner strength ×1 and ×2 gym splits
- Long run goes on the day they pick (else the weekend), then the gym week is laid out as a
  whole: Push/Upper/Shoulders & arms (and Pull/Upper) never on consecutive days if it can be
  helped, split order kept where it fits, room left for the hard runs; other runs fit around.
- AthleteProfile.longRunDay (stored and synced).
- Runner strength ×1 / ×2 in the programmes workbook: single-leg strength, hamstrings, calves,
  hip power and core; suggested for 5K to marathon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T6u6ov9HaybuWy59SNZhPU
</commit_message>
<xml_diff>
--- a/programmes/Kinetix Programmes.xlsx
+++ b/programmes/Kinetix Programmes.xlsx
@@ -1595,6 +1595,11 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="21">
+      <c r="E14" s="27" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
       <c r="I14" s="27" t="inlineStr">
         <is>
           <t>Any Hyrox station</t>
@@ -1602,6 +1607,11 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="21">
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
       <c r="I15" s="27" t="inlineStr">
         <is>
           <t>Arnold Press</t>
@@ -2361,7 +2371,11 @@
         <f>COUNTIF('Run sessions'!$A$2:$A$401,A2)</f>
         <v/>
       </c>
-      <c r="T2" s="32" t="n"/>
+      <c r="T2" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2, Runner strength ×1</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="21">
       <c r="A3" s="30" t="inlineStr">
@@ -2435,7 +2449,11 @@
         <f>COUNTIF('Run sessions'!$A$2:$A$401,A3)</f>
         <v/>
       </c>
-      <c r="T3" s="32" t="n"/>
+      <c r="T3" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2, Runner strength ×1</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="21">
       <c r="A4" s="30" t="inlineStr">
@@ -2509,7 +2527,11 @@
         <f>COUNTIF('Run sessions'!$A$2:$A$401,A4)</f>
         <v/>
       </c>
-      <c r="T4" s="32" t="n"/>
+      <c r="T4" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2, Runner strength ×1</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="21">
       <c r="A5" s="30" t="inlineStr">
@@ -2583,7 +2605,11 @@
         <f>COUNTIF('Run sessions'!$A$2:$A$401,A5)</f>
         <v/>
       </c>
-      <c r="T5" s="32" t="n"/>
+      <c r="T5" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2, Runner strength ×1</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="21">
       <c r="A6" s="30" t="inlineStr">
@@ -2657,7 +2683,11 @@
         <f>COUNTIF('Run sessions'!$A$2:$A$401,A6)</f>
         <v/>
       </c>
-      <c r="T6" s="32" t="n"/>
+      <c r="T6" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2, Runner strength ×1</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="21">
       <c r="A7" s="30" t="inlineStr">
@@ -2959,6 +2989,7 @@
       </c>
       <c r="T10" s="32" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12" ht="15" customHeight="1" s="21">
       <c r="A12" s="34" t="inlineStr">
         <is>
@@ -2973,7 +3004,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="O2:O10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Choose from the list" error="Pick one of the options in the drop-down." promptTitle="Tip" prompt="The split suggested in onboarding (the user can change it)." type="list" errorStyle="stop" operator="between">
-      <formula1>Lists!$E$2:$E$13</formula1>
+      <formula1>Lists!$E$2:$E$15</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="Q2:Q10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Choose from the list" error="Pick one of the options in the drop-down." promptTitle="Tip" prompt="Which runners see this goal in onboarding." type="list" errorStyle="stop" operator="between">
@@ -2981,7 +3012,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="T2:T10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>Lists!$E$2:$E$13</formula1>
+      <formula1>Lists!$E$2:$E$15</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -24592,7 +24623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="20" min="1" max="1"/>
@@ -24980,6 +25011,64 @@
       </c>
       <c r="F13" s="33">
         <f>SUMPRODUCT(('Split days'!$A$2:$A$401=A13)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Runners: one short session of single-leg strength, calves and core to stay strong and injury-resistant.</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F14" s="33">
+        <f>SUMPRODUCT(('Split days'!$A$2:$A$401=A14)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="30" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A, Runner strength B</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>Runners: single-leg strength, hamstrings and calves, plus hip power. Short sessions that fit around running.</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="33">
+        <f>SUMPRODUCT(('Split days'!$A$2:$A$401=A15)/COUNTIFS('Split days'!$A$2:$A$401,'Split days'!$A$2:$A$401&amp;"",'Split days'!$B$2:$B$401,'Split days'!$B$2:$B$401&amp;""))</f>
         <v/>
       </c>
     </row>
@@ -32466,215 +32555,681 @@
       <c r="J226" s="32" t="n"/>
     </row>
     <row r="227" ht="15" customHeight="1" s="21">
-      <c r="A227" s="32" t="n"/>
-      <c r="B227" s="32" t="n"/>
-      <c r="C227" s="32" t="n"/>
-      <c r="D227" s="32" t="n"/>
-      <c r="E227" s="32" t="n"/>
-      <c r="F227" s="32" t="n"/>
-      <c r="G227" s="32" t="n"/>
-      <c r="H227" s="32" t="n"/>
-      <c r="I227" s="32" t="n"/>
-      <c r="J227" s="32" t="n"/>
+      <c r="A227" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B227" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C227" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D227" s="32" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat</t>
+        </is>
+      </c>
+      <c r="E227" s="32" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="F227" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G227" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H227" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="I227" s="32" t="n">
+        <v>120</v>
+      </c>
+      <c r="J227" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Back foot on a bench.</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="15" customHeight="1" s="21">
-      <c r="A228" s="37" t="inlineStr">
-        <is>
-          <t>A first draft of every split to edit. 'Any …' lets the app choose for the user's equipment; named exercises are swapped for the closest option if they can't do them. Blank sets/reps/rest use 'Strength by goal'.</t>
-        </is>
-      </c>
-      <c r="B228" s="32" t="n"/>
-      <c r="C228" s="32" t="n"/>
-      <c r="D228" s="32" t="n"/>
-      <c r="E228" s="32" t="n"/>
-      <c r="F228" s="32" t="n"/>
-      <c r="G228" s="32" t="n"/>
-      <c r="H228" s="32" t="n"/>
-      <c r="I228" s="32" t="n"/>
+      <c r="A228" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B228" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C228" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D228" s="32" t="inlineStr">
+        <is>
+          <t>Romanian Deadlift</t>
+        </is>
+      </c>
+      <c r="E228" s="32" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="F228" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G228" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H228" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="I228" s="32" t="n">
+        <v>120</v>
+      </c>
       <c r="J228" s="32" t="n"/>
     </row>
     <row r="229" ht="15" customHeight="1" s="21">
-      <c r="A229" s="37" t="inlineStr">
-        <is>
-          <t>Leg-heavy days are kept away from hard runs and the long run automatically.</t>
-        </is>
-      </c>
-      <c r="B229" s="32" t="n"/>
-      <c r="C229" s="32" t="n"/>
-      <c r="D229" s="32" t="n"/>
-      <c r="E229" s="32" t="n"/>
-      <c r="F229" s="32" t="n"/>
-      <c r="G229" s="32" t="n"/>
-      <c r="H229" s="32" t="n"/>
-      <c r="I229" s="32" t="n"/>
-      <c r="J229" s="32" t="n"/>
+      <c r="A229" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B229" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C229" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D229" s="32" t="inlineStr">
+        <is>
+          <t>Step-Up</t>
+        </is>
+      </c>
+      <c r="E229" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F229" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G229" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H229" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I229" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="J229" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Drive the knee up.</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="15" customHeight="1" s="21">
-      <c r="A230" s="32" t="n"/>
-      <c r="B230" s="32" t="n"/>
-      <c r="C230" s="32" t="n"/>
-      <c r="D230" s="32" t="n"/>
-      <c r="E230" s="32" t="n"/>
-      <c r="F230" s="32" t="n"/>
-      <c r="G230" s="32" t="n"/>
-      <c r="H230" s="32" t="n"/>
-      <c r="I230" s="32" t="n"/>
-      <c r="J230" s="32" t="n"/>
+      <c r="A230" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B230" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C230" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D230" s="32" t="inlineStr">
+        <is>
+          <t>Single-Leg Calf Raise</t>
+        </is>
+      </c>
+      <c r="E230" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F230" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G230" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="H230" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="I230" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="J230" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Pause at the bottom.</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="15" customHeight="1" s="21">
-      <c r="A231" s="32" t="n"/>
-      <c r="B231" s="32" t="n"/>
-      <c r="C231" s="32" t="n"/>
-      <c r="D231" s="32" t="n"/>
-      <c r="E231" s="32" t="n"/>
-      <c r="F231" s="32" t="n"/>
-      <c r="G231" s="32" t="n"/>
-      <c r="H231" s="32" t="n"/>
-      <c r="I231" s="32" t="n"/>
+      <c r="A231" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B231" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C231" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D231" s="32" t="inlineStr">
+        <is>
+          <t>Any horizontal pull (row)</t>
+        </is>
+      </c>
+      <c r="E231" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F231" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G231" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H231" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="I231" s="32" t="n">
+        <v>60</v>
+      </c>
       <c r="J231" s="32" t="n"/>
     </row>
     <row r="232" ht="15" customHeight="1" s="21">
-      <c r="A232" s="32" t="n"/>
-      <c r="B232" s="32" t="n"/>
-      <c r="C232" s="32" t="n"/>
-      <c r="D232" s="32" t="n"/>
-      <c r="E232" s="32" t="n"/>
-      <c r="F232" s="32" t="n"/>
-      <c r="G232" s="32" t="n"/>
-      <c r="H232" s="32" t="n"/>
-      <c r="I232" s="32" t="n"/>
+      <c r="A232" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×1</t>
+        </is>
+      </c>
+      <c r="B232" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength</t>
+        </is>
+      </c>
+      <c r="C232" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D232" s="32" t="inlineStr">
+        <is>
+          <t>Any anti-rotation core</t>
+        </is>
+      </c>
+      <c r="E232" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F232" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G232" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H232" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I232" s="32" t="n">
+        <v>45</v>
+      </c>
       <c r="J232" s="32" t="n"/>
     </row>
     <row r="233" ht="15" customHeight="1" s="21">
-      <c r="A233" s="32" t="n"/>
-      <c r="B233" s="32" t="n"/>
-      <c r="C233" s="32" t="n"/>
-      <c r="D233" s="32" t="n"/>
-      <c r="E233" s="32" t="n"/>
-      <c r="F233" s="32" t="n"/>
-      <c r="G233" s="32" t="n"/>
-      <c r="H233" s="32" t="n"/>
-      <c r="I233" s="32" t="n"/>
+      <c r="A233" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B233" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A</t>
+        </is>
+      </c>
+      <c r="C233" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D233" s="32" t="inlineStr">
+        <is>
+          <t>Any squat</t>
+        </is>
+      </c>
+      <c r="E233" s="32" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="F233" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G233" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="H233" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="I233" s="32" t="n">
+        <v>150</v>
+      </c>
       <c r="J233" s="32" t="n"/>
     </row>
     <row r="234" ht="15" customHeight="1" s="21">
-      <c r="A234" s="32" t="n"/>
-      <c r="B234" s="32" t="n"/>
-      <c r="C234" s="32" t="n"/>
-      <c r="D234" s="32" t="n"/>
-      <c r="E234" s="32" t="n"/>
-      <c r="F234" s="32" t="n"/>
-      <c r="G234" s="32" t="n"/>
-      <c r="H234" s="32" t="n"/>
-      <c r="I234" s="32" t="n"/>
-      <c r="J234" s="32" t="n"/>
+      <c r="A234" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B234" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A</t>
+        </is>
+      </c>
+      <c r="C234" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D234" s="32" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat</t>
+        </is>
+      </c>
+      <c r="E234" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F234" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G234" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="H234" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="I234" s="32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J234" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Back foot on a bench.</t>
+        </is>
+      </c>
     </row>
     <row r="235" ht="15" customHeight="1" s="21">
-      <c r="A235" s="32" t="n"/>
-      <c r="B235" s="32" t="n"/>
-      <c r="C235" s="32" t="n"/>
-      <c r="D235" s="32" t="n"/>
-      <c r="E235" s="32" t="n"/>
-      <c r="F235" s="32" t="n"/>
-      <c r="G235" s="32" t="n"/>
-      <c r="H235" s="32" t="n"/>
-      <c r="I235" s="32" t="n"/>
-      <c r="J235" s="32" t="n"/>
+      <c r="A235" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B235" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A</t>
+        </is>
+      </c>
+      <c r="C235" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D235" s="32" t="inlineStr">
+        <is>
+          <t>Nordic Hamstring Curl</t>
+        </is>
+      </c>
+      <c r="E235" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F235" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G235" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H235" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="I235" s="32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J235" s="32" t="inlineStr">
+        <is>
+          <t>Lower as slowly as you can.</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="15" customHeight="1" s="21">
-      <c r="A236" s="32" t="n"/>
-      <c r="B236" s="32" t="n"/>
-      <c r="C236" s="32" t="n"/>
-      <c r="D236" s="32" t="n"/>
-      <c r="E236" s="32" t="n"/>
-      <c r="F236" s="32" t="n"/>
-      <c r="G236" s="32" t="n"/>
-      <c r="H236" s="32" t="n"/>
-      <c r="I236" s="32" t="n"/>
-      <c r="J236" s="32" t="n"/>
+      <c r="A236" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B236" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A</t>
+        </is>
+      </c>
+      <c r="C236" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D236" s="32" t="inlineStr">
+        <is>
+          <t>Single-Leg Calf Raise</t>
+        </is>
+      </c>
+      <c r="E236" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F236" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G236" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="H236" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="I236" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="J236" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Pause at the bottom.</t>
+        </is>
+      </c>
     </row>
     <row r="237" ht="15" customHeight="1" s="21">
-      <c r="A237" s="32" t="n"/>
-      <c r="B237" s="32" t="n"/>
-      <c r="C237" s="32" t="n"/>
-      <c r="D237" s="32" t="n"/>
-      <c r="E237" s="32" t="n"/>
-      <c r="F237" s="32" t="n"/>
-      <c r="G237" s="32" t="n"/>
-      <c r="H237" s="32" t="n"/>
-      <c r="I237" s="32" t="n"/>
+      <c r="A237" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B237" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength A</t>
+        </is>
+      </c>
+      <c r="C237" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D237" s="32" t="inlineStr">
+        <is>
+          <t>Any anti-rotation core</t>
+        </is>
+      </c>
+      <c r="E237" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F237" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G237" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H237" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I237" s="32" t="n">
+        <v>45</v>
+      </c>
       <c r="J237" s="32" t="n"/>
     </row>
     <row r="238" ht="15" customHeight="1" s="21">
-      <c r="A238" s="32" t="n"/>
-      <c r="B238" s="32" t="n"/>
-      <c r="C238" s="32" t="n"/>
-      <c r="D238" s="32" t="n"/>
-      <c r="E238" s="32" t="n"/>
-      <c r="F238" s="32" t="n"/>
-      <c r="G238" s="32" t="n"/>
-      <c r="H238" s="32" t="n"/>
-      <c r="I238" s="32" t="n"/>
+      <c r="A238" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B238" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C238" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D238" s="32" t="inlineStr">
+        <is>
+          <t>Any hinge (deadlift)</t>
+        </is>
+      </c>
+      <c r="E238" s="32" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="F238" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G238" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="H238" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="I238" s="32" t="n">
+        <v>150</v>
+      </c>
       <c r="J238" s="32" t="n"/>
     </row>
     <row r="239" ht="15" customHeight="1" s="21">
-      <c r="A239" s="32" t="n"/>
-      <c r="B239" s="32" t="n"/>
-      <c r="C239" s="32" t="n"/>
-      <c r="D239" s="32" t="n"/>
-      <c r="E239" s="32" t="n"/>
-      <c r="F239" s="32" t="n"/>
-      <c r="G239" s="32" t="n"/>
-      <c r="H239" s="32" t="n"/>
-      <c r="I239" s="32" t="n"/>
-      <c r="J239" s="32" t="n"/>
+      <c r="A239" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B239" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C239" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D239" s="32" t="inlineStr">
+        <is>
+          <t>Step-Up</t>
+        </is>
+      </c>
+      <c r="E239" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F239" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G239" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H239" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I239" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="J239" s="32" t="inlineStr">
+        <is>
+          <t>Each leg. Drive the knee up.</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="15" customHeight="1" s="21">
-      <c r="A240" s="32" t="n"/>
-      <c r="B240" s="32" t="n"/>
-      <c r="C240" s="32" t="n"/>
-      <c r="D240" s="32" t="n"/>
-      <c r="E240" s="32" t="n"/>
-      <c r="F240" s="32" t="n"/>
-      <c r="G240" s="32" t="n"/>
-      <c r="H240" s="32" t="n"/>
-      <c r="I240" s="32" t="n"/>
+      <c r="A240" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B240" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C240" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D240" s="32" t="inlineStr">
+        <is>
+          <t>Barbell Hip Thrust</t>
+        </is>
+      </c>
+      <c r="E240" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F240" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G240" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H240" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I240" s="32" t="n">
+        <v>90</v>
+      </c>
       <c r="J240" s="32" t="n"/>
     </row>
     <row r="241" ht="15" customHeight="1" s="21">
-      <c r="A241" s="32" t="n"/>
-      <c r="B241" s="32" t="n"/>
-      <c r="C241" s="32" t="n"/>
-      <c r="D241" s="32" t="n"/>
-      <c r="E241" s="32" t="n"/>
-      <c r="F241" s="32" t="n"/>
-      <c r="G241" s="32" t="n"/>
-      <c r="H241" s="32" t="n"/>
-      <c r="I241" s="32" t="n"/>
-      <c r="J241" s="32" t="n"/>
+      <c r="A241" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B241" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C241" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="D241" s="32" t="inlineStr">
+        <is>
+          <t>Kettlebell Swing</t>
+        </is>
+      </c>
+      <c r="E241" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F241" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="G241" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H241" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="I241" s="32" t="n">
+        <v>60</v>
+      </c>
+      <c r="J241" s="32" t="inlineStr">
+        <is>
+          <t>Snap the hips: power for running.</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="15" customHeight="1" s="21">
-      <c r="A242" s="32" t="n"/>
-      <c r="B242" s="32" t="n"/>
-      <c r="C242" s="32" t="n"/>
-      <c r="D242" s="32" t="n"/>
-      <c r="E242" s="32" t="n"/>
-      <c r="F242" s="32" t="n"/>
-      <c r="G242" s="32" t="n"/>
-      <c r="H242" s="32" t="n"/>
-      <c r="I242" s="32" t="n"/>
+      <c r="A242" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B242" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C242" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="D242" s="32" t="inlineStr">
+        <is>
+          <t>Any horizontal pull (row)</t>
+        </is>
+      </c>
+      <c r="E242" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F242" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G242" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="H242" s="32" t="n">
+        <v>12</v>
+      </c>
+      <c r="I242" s="32" t="n">
+        <v>60</v>
+      </c>
       <c r="J242" s="32" t="n"/>
     </row>
     <row r="243" ht="15" customHeight="1" s="21">
-      <c r="A243" s="32" t="n"/>
-      <c r="B243" s="32" t="n"/>
-      <c r="C243" s="32" t="n"/>
-      <c r="D243" s="32" t="n"/>
-      <c r="E243" s="32" t="n"/>
-      <c r="F243" s="32" t="n"/>
-      <c r="G243" s="32" t="n"/>
-      <c r="H243" s="32" t="n"/>
-      <c r="I243" s="32" t="n"/>
+      <c r="A243" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength ×2</t>
+        </is>
+      </c>
+      <c r="B243" s="32" t="inlineStr">
+        <is>
+          <t>Runner strength B</t>
+        </is>
+      </c>
+      <c r="C243" s="32" t="n">
+        <v>6</v>
+      </c>
+      <c r="D243" s="32" t="inlineStr">
+        <is>
+          <t>Any core</t>
+        </is>
+      </c>
+      <c r="E243" s="32" t="inlineStr">
+        <is>
+          <t>Accessory</t>
+        </is>
+      </c>
+      <c r="F243" s="32" t="n">
+        <v>2</v>
+      </c>
+      <c r="G243" s="32" t="n">
+        <v>8</v>
+      </c>
+      <c r="H243" s="32" t="n">
+        <v>10</v>
+      </c>
+      <c r="I243" s="32" t="n">
+        <v>45</v>
+      </c>
       <c r="J243" s="32" t="n"/>
     </row>
     <row r="244" ht="15" customHeight="1" s="21">
@@ -32690,7 +33245,11 @@
       <c r="J244" s="32" t="n"/>
     </row>
     <row r="245" ht="15" customHeight="1" s="21">
-      <c r="A245" s="32" t="n"/>
+      <c r="A245" s="37" t="inlineStr">
+        <is>
+          <t>A first draft of every split to edit. 'Any …' lets the app choose for the user's equipment; named exercises are swapped for the closest option if they can't do them. Blank sets/reps/rest use 'Strength by goal'.</t>
+        </is>
+      </c>
       <c r="B245" s="32" t="n"/>
       <c r="C245" s="32" t="n"/>
       <c r="D245" s="32" t="n"/>
@@ -32702,7 +33261,11 @@
       <c r="J245" s="32" t="n"/>
     </row>
     <row r="246" ht="15" customHeight="1" s="21">
-      <c r="A246" s="32" t="n"/>
+      <c r="A246" s="37" t="inlineStr">
+        <is>
+          <t>Leg-heavy days are kept away from hard runs and the long run automatically.</t>
+        </is>
+      </c>
       <c r="B246" s="32" t="n"/>
       <c r="C246" s="32" t="n"/>
       <c r="D246" s="32" t="n"/>
@@ -34888,7 +35451,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="A2:A401" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Choose from the list" error="Pick one of the options in the drop-down." type="list" errorStyle="stop" operator="between">
-      <formula1>Lists!$E$2:$E$13</formula1>
+      <formula1>Lists!$E$2:$E$15</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D401" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Choose from the list" error="Pick one of the options in the drop-down." promptTitle="Tip" prompt="Pick 'Any …' to let the app choose for the user's equipment, or a named exercise." type="list" errorStyle="stop" operator="between">

</xml_diff>